<commit_message>
Force calcMode=auto inside the file (defeats app-level Manual calc that froze his typing at MONTH(TODAY())=September) + live mode indicator under the boxes
</commit_message>
<xml_diff>
--- a/uploads/inbox/SPV_ROSTER_SMART.xlsx
+++ b/uploads/inbox/SPV_ROSTER_SMART.xlsx
@@ -11,7 +11,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'ROSTER'!$A$1:$AI$88</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" calcOnSave="1"/>
 </workbook>
 </file>
 
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="mmmm\ yyyy"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -193,6 +193,12 @@
       <b val="1"/>
       <color rgb="FF713F12"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00196B24"/>
+      <sz val="8.5"/>
     </font>
   </fonts>
   <fills count="29">
@@ -764,7 +770,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="152">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1183,6 +1189,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="28" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1854,13 +1863,11 @@
           <t>MONTHLY</t>
         </is>
       </c>
-      <c r="AL1" s="106" t="n"/>
       <c r="AN1" s="107" t="inlineStr">
         <is>
           <t>CUSTOM PERIOD</t>
         </is>
       </c>
-      <c r="AO1" s="108" t="n"/>
       <c r="BA1">
         <f>IF(ISNUMBER($BA$5),"P","M")</f>
         <v/>
@@ -2264,6 +2271,10 @@
       <c r="AG5" s="6" t="n"/>
       <c r="AH5" s="26" t="n"/>
       <c r="AI5" s="23" t="n"/>
+      <c r="AK5" s="152">
+        <f>IF($BA$1="P","● PERIOD MODE ACTIVE","● MONTH MODE")</f>
+        <v/>
+      </c>
       <c r="BA5">
         <f>IF(ISNUMBER($AO$2),$AO$2,IFERROR(DATEVALUE(TRIM($AO$2&amp;"")),""))</f>
         <v/>
@@ -6695,7 +6706,7 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="45">
+  <mergeCells count="46">
     <mergeCell ref="X88:AA88"/>
     <mergeCell ref="E2:AC2"/>
     <mergeCell ref="C1:C2"/>
@@ -6716,6 +6727,7 @@
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="M83:S83"/>
     <mergeCell ref="X86:AA86"/>
+    <mergeCell ref="AK5:AO5"/>
     <mergeCell ref="R88:U88"/>
     <mergeCell ref="E64:H64"/>
     <mergeCell ref="R87:U87"/>

</xml_diff>

<commit_message>
Period input = numeric D/M/Y triplet + DAYS (locale-proof, no date parsing at all) + live mode indicator with computed period preview
</commit_message>
<xml_diff>
--- a/uploads/inbox/SPV_ROSTER_SMART.xlsx
+++ b/uploads/inbox/SPV_ROSTER_SMART.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="mmmm\ yyyy"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="32">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -200,6 +200,18 @@
       <color rgb="00196B24"/>
       <sz val="8.5"/>
     </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="7"/>
+    </font>
   </fonts>
   <fills count="29">
     <fill>
@@ -353,7 +365,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="35">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -766,11 +778,12 @@
         <color rgb="007F8C8D"/>
       </bottom>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="153">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1192,6 +1205,25 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1798,8 +1830,11 @@
     <col width="7" customWidth="1" min="37" max="37"/>
     <col width="7.5" customWidth="1" min="38" max="38"/>
     <col width="3.5" customWidth="1" min="39" max="39"/>
-    <col width="6.5" customWidth="1" min="40" max="40"/>
-    <col width="10" customWidth="1" min="41" max="41"/>
+    <col width="6" customWidth="1" min="40" max="40"/>
+    <col width="4.5" customWidth="1" min="41" max="41"/>
+    <col width="4.5" customWidth="1" min="42" max="42"/>
+    <col width="6.5" customWidth="1" min="43" max="43"/>
+    <col width="2" customWidth="1" min="44" max="44"/>
     <col hidden="1" width="13" customWidth="1" min="53" max="53"/>
   </cols>
   <sheetData>
@@ -1858,16 +1893,23 @@
           <t>CC: 264</t>
         </is>
       </c>
-      <c r="AK1" s="105" t="inlineStr">
+      <c r="AK1" s="153" t="inlineStr">
         <is>
           <t>MONTHLY</t>
         </is>
       </c>
-      <c r="AN1" s="107" t="inlineStr">
-        <is>
-          <t>CUSTOM PERIOD</t>
-        </is>
-      </c>
+      <c r="AL1" s="106" t="n"/>
+      <c r="AM1" s="154" t="n"/>
+      <c r="AN1" s="155" t="inlineStr">
+        <is>
+          <t>CUSTOM PERIOD  (numbers only)</t>
+        </is>
+      </c>
+      <c r="AO1" s="108" t="n"/>
+      <c r="AP1" s="108" t="n"/>
+      <c r="AQ1" s="108" t="n"/>
+      <c r="AR1" s="108" t="n"/>
+      <c r="AS1" s="154" t="n"/>
       <c r="BA1">
         <f>IF(ISNUMBER($BA$5),"P","M")</f>
         <v/>
@@ -1922,7 +1964,7 @@
           <t>JUL</t>
         </is>
       </c>
-      <c r="AM2" s="115" t="inlineStr">
+      <c r="AM2" s="156" t="inlineStr">
         <is>
           <t>OR</t>
         </is>
@@ -1932,7 +1974,11 @@
           <t>START</t>
         </is>
       </c>
-      <c r="AO2" s="116" t="n"/>
+      <c r="AO2" s="114" t="n"/>
+      <c r="AP2" s="114" t="n"/>
+      <c r="AQ2" s="114" t="n"/>
+      <c r="AR2" s="154" t="n"/>
+      <c r="AS2" s="154" t="n"/>
       <c r="BA2">
         <f>IFERROR(IF(ISNUMBER($AL$2),$AL$2,MATCH(LEFT(UPPER(TRIM($AL$2)),3),{"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC"},0)),MONTH(TODAY()))</f>
         <v/>
@@ -2082,6 +2128,10 @@
         </is>
       </c>
       <c r="AO3" s="114" t="n"/>
+      <c r="AP3" s="154" t="n"/>
+      <c r="AQ3" s="154" t="n"/>
+      <c r="AR3" s="154" t="n"/>
+      <c r="AS3" s="154" t="n"/>
       <c r="BA3">
         <f>IF($BA$1="P",$BA$5,DATE(IF(ISNUMBER($AL$3),$AL$3,YEAR(TODAY())),$BA$2,1))</f>
         <v/>
@@ -2213,11 +2263,27 @@
         <f>IF(31&lt;=$BA$4,IF($BA$1="P",DAY($BA$3+30),31),"")</f>
         <v/>
       </c>
-      <c r="AK4" s="118" t="inlineStr">
-        <is>
-          <t>fill START date to switch to period</t>
-        </is>
-      </c>
+      <c r="AK4" s="157" t="n"/>
+      <c r="AL4" s="154" t="n"/>
+      <c r="AM4" s="154" t="n"/>
+      <c r="AN4" s="154" t="n"/>
+      <c r="AO4" s="158" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="AP4" s="158" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="AQ4" s="158" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="AR4" s="154" t="n"/>
+      <c r="AS4" s="154" t="n"/>
       <c r="BA4">
         <f>IF($BA$1="P",MIN(31,IF(ISNUMBER($AO$3),$AO$3,30)),DAY(EOMONTH($BA$3,0)))</f>
         <v/>
@@ -2271,12 +2337,13 @@
       <c r="AG5" s="6" t="n"/>
       <c r="AH5" s="26" t="n"/>
       <c r="AI5" s="23" t="n"/>
-      <c r="AK5" s="152">
-        <f>IF($BA$1="P","● PERIOD MODE ACTIVE","● MONTH MODE")</f>
-        <v/>
-      </c>
+      <c r="AK5" s="159">
+        <f>IF($BA$1="P","● PERIOD MODE ACTIVE — "&amp;TEXT($BA$3,"dd/mm")&amp;" +"&amp;$BA$4&amp;"d","● MONTH MODE")</f>
+        <v/>
+      </c>
+      <c r="AS5" s="154" t="n"/>
       <c r="BA5">
-        <f>IF(ISNUMBER($AO$2),$AO$2,IFERROR(DATEVALUE(TRIM($AO$2&amp;"")),""))</f>
+        <f>IF(AND(ISNUMBER($AO$2),ISNUMBER($AP$2),ISNUMBER($AQ$2)),IFERROR(DATE(IF($AQ$2&lt;100,2000+$AQ$2,$AQ$2),$AP$2,$AO$2),""),"")</f>
         <v/>
       </c>
     </row>
@@ -6706,14 +6773,13 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="46">
+  <mergeCells count="45">
     <mergeCell ref="X88:AA88"/>
     <mergeCell ref="E2:AC2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="AD87:AG87"/>
     <mergeCell ref="A74:C78"/>
     <mergeCell ref="W82:AC82"/>
-    <mergeCell ref="AK4:AO4"/>
     <mergeCell ref="E80:J80"/>
     <mergeCell ref="F83:J83"/>
     <mergeCell ref="F88:I88"/>
@@ -6721,13 +6787,13 @@
     <mergeCell ref="A46:D47"/>
     <mergeCell ref="AD1:AI2"/>
     <mergeCell ref="A3:D4"/>
-    <mergeCell ref="AN1:AO1"/>
     <mergeCell ref="F87:I87"/>
     <mergeCell ref="E62:H62"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="M83:S83"/>
     <mergeCell ref="X86:AA86"/>
-    <mergeCell ref="AK5:AO5"/>
+    <mergeCell ref="AN1:AR1"/>
+    <mergeCell ref="AK5:AR5"/>
     <mergeCell ref="R88:U88"/>
     <mergeCell ref="E64:H64"/>
     <mergeCell ref="R87:U87"/>

</xml_diff>

<commit_message>
Omnivorous START parser: single field accepts 3/3/2027, 3-3-2027, 03.03.2027, Arabic-Indic digits, 2-digit years - normalization chain in hidden cells; proofs rendered for dash+Arabic inputs
</commit_message>
<xml_diff>
--- a/uploads/inbox/SPV_ROSTER_SMART.xlsx
+++ b/uploads/inbox/SPV_ROSTER_SMART.xlsx
@@ -365,7 +365,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="36">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -779,11 +779,15 @@
       </bottom>
     </border>
     <border/>
+    <border>
+      <right/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1224,6 +1228,22 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="14" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1831,8 +1851,8 @@
     <col width="7.5" customWidth="1" min="38" max="38"/>
     <col width="3.5" customWidth="1" min="39" max="39"/>
     <col width="6" customWidth="1" min="40" max="40"/>
-    <col width="4.5" customWidth="1" min="41" max="41"/>
-    <col width="4.5" customWidth="1" min="42" max="42"/>
+    <col width="7" customWidth="1" min="41" max="41"/>
+    <col width="7" customWidth="1" min="42" max="42"/>
     <col width="6.5" customWidth="1" min="43" max="43"/>
     <col width="2" customWidth="1" min="44" max="44"/>
     <col hidden="1" width="13" customWidth="1" min="53" max="53"/>
@@ -1893,22 +1913,21 @@
           <t>CC: 264</t>
         </is>
       </c>
-      <c r="AK1" s="153" t="inlineStr">
+      <c r="AK1" s="160" t="inlineStr">
         <is>
           <t>MONTHLY</t>
         </is>
       </c>
-      <c r="AL1" s="106" t="n"/>
       <c r="AM1" s="154" t="n"/>
-      <c r="AN1" s="155" t="inlineStr">
-        <is>
-          <t>CUSTOM PERIOD  (numbers only)</t>
+      <c r="AN1" s="161" t="inlineStr">
+        <is>
+          <t>CUSTOM PERIOD</t>
         </is>
       </c>
       <c r="AO1" s="108" t="n"/>
       <c r="AP1" s="108" t="n"/>
-      <c r="AQ1" s="108" t="n"/>
-      <c r="AR1" s="108" t="n"/>
+      <c r="AQ1" s="154" t="n"/>
+      <c r="AR1" s="154" t="n"/>
       <c r="AS1" s="154" t="n"/>
       <c r="BA1">
         <f>IF(ISNUMBER($BA$5),"P","M")</f>
@@ -1974,9 +1993,9 @@
           <t>START</t>
         </is>
       </c>
-      <c r="AO2" s="114" t="n"/>
-      <c r="AP2" s="114" t="n"/>
-      <c r="AQ2" s="114" t="n"/>
+      <c r="AO2" s="162" t="n"/>
+      <c r="AP2" s="163" t="n"/>
+      <c r="AQ2" s="164" t="n"/>
       <c r="AR2" s="154" t="n"/>
       <c r="AS2" s="154" t="n"/>
       <c r="BA2">
@@ -2127,8 +2146,8 @@
           <t>DAYS</t>
         </is>
       </c>
-      <c r="AO3" s="114" t="n"/>
-      <c r="AP3" s="154" t="n"/>
+      <c r="AO3" s="162" t="n"/>
+      <c r="AP3" s="163" t="n"/>
       <c r="AQ3" s="154" t="n"/>
       <c r="AR3" s="154" t="n"/>
       <c r="AS3" s="154" t="n"/>
@@ -2267,25 +2286,13 @@
       <c r="AL4" s="154" t="n"/>
       <c r="AM4" s="154" t="n"/>
       <c r="AN4" s="154" t="n"/>
-      <c r="AO4" s="158" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="AP4" s="158" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="AQ4" s="158" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="AO4" s="158" t="n"/>
+      <c r="AP4" s="158" t="n"/>
+      <c r="AQ4" s="158" t="n"/>
       <c r="AR4" s="154" t="n"/>
       <c r="AS4" s="154" t="n"/>
       <c r="BA4">
-        <f>IF($BA$1="P",MIN(31,IF(ISNUMBER($AO$3),$AO$3,30)),DAY(EOMONTH($BA$3,0)))</f>
+        <f>IF($BA$1="P",MIN(31,IFERROR(VALUE($BA$12),IF(ISNUMBER($AO$3),$AO$3,30))),DAY(EOMONTH($BA$3,0)))</f>
         <v/>
       </c>
     </row>
@@ -2337,13 +2344,13 @@
       <c r="AG5" s="6" t="n"/>
       <c r="AH5" s="26" t="n"/>
       <c r="AI5" s="23" t="n"/>
-      <c r="AK5" s="159">
-        <f>IF($BA$1="P","● PERIOD MODE ACTIVE — "&amp;TEXT($BA$3,"dd/mm")&amp;" +"&amp;$BA$4&amp;"d","● MONTH MODE")</f>
+      <c r="AK5" s="165">
+        <f>IF($BA$1="P","● PERIOD MODE — "&amp;TEXT($BA$3,"dd/mm/yyyy")&amp;" +"&amp;$BA$4&amp;"d","● MONTH MODE")</f>
         <v/>
       </c>
       <c r="AS5" s="154" t="n"/>
       <c r="BA5">
-        <f>IF(AND(ISNUMBER($AO$2),ISNUMBER($AP$2),ISNUMBER($AQ$2)),IFERROR(DATE(IF($AQ$2&lt;100,2000+$AQ$2,$AQ$2),$AP$2,$AO$2),""),"")</f>
+        <f>IF(ISNUMBER($AO$2),$AO$2,IFERROR(DATE(IF($BA$11&lt;100,2000+$BA$11,$BA$11),$BA$10,$BA$9),""))</f>
         <v/>
       </c>
     </row>
@@ -2395,6 +2402,10 @@
       <c r="AG6" s="6" t="n"/>
       <c r="AH6" s="26" t="n"/>
       <c r="AI6" s="23" t="n"/>
+      <c r="BA6">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(TRIM($AO$2&amp;""),"٠","0"),"١","1"),"٢","2"),"٣","3"),"٤","4"),"٥","5"),"٦","6"),"٧","7"),"٨","8"),"٩","9"),"-","/"),".","/"),"\\","/")," ","")</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="16.2" customHeight="1" thickBot="1">
       <c r="A7" s="5" t="n">
@@ -2444,6 +2455,10 @@
       <c r="AG7" s="6" t="n"/>
       <c r="AH7" s="26" t="n"/>
       <c r="AI7" s="23" t="n"/>
+      <c r="BA7">
+        <f>IFERROR(FIND("/",$BA$6),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="16.2" customHeight="1" thickBot="1">
       <c r="A8" s="5" t="n">
@@ -2493,6 +2508,10 @@
       <c r="AG8" s="6" t="n"/>
       <c r="AH8" s="26" t="n"/>
       <c r="AI8" s="23" t="n"/>
+      <c r="BA8">
+        <f>IFERROR(FIND("/",$BA$6,$BA$7+1),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="16.2" customHeight="1" thickBot="1">
       <c r="A9" s="5" t="n">
@@ -2542,6 +2561,10 @@
       <c r="AG9" s="6" t="n"/>
       <c r="AH9" s="26" t="n"/>
       <c r="AI9" s="23" t="n"/>
+      <c r="BA9">
+        <f>IFERROR(VALUE(LEFT($BA$6,$BA$7-1)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="16.2" customHeight="1" thickBot="1">
       <c r="A10" s="10" t="n">
@@ -2591,6 +2614,10 @@
       <c r="AG10" s="6" t="n"/>
       <c r="AH10" s="26" t="n"/>
       <c r="AI10" s="23" t="n"/>
+      <c r="BA10">
+        <f>IFERROR(VALUE(MID($BA$6,$BA$7+1,$BA$8-$BA$7-1)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="11" ht="16.2" customHeight="1" thickBot="1">
       <c r="A11" s="10" t="n">
@@ -2640,6 +2667,10 @@
       <c r="AG11" s="6" t="n"/>
       <c r="AH11" s="26" t="n"/>
       <c r="AI11" s="23" t="n"/>
+      <c r="BA11">
+        <f>IFERROR(VALUE(MID($BA$6,$BA$8+1,9)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="16.2" customHeight="1" thickBot="1">
       <c r="A12" s="10" t="n">
@@ -2689,6 +2720,10 @@
       <c r="AG12" s="6" t="n"/>
       <c r="AH12" s="26" t="n"/>
       <c r="AI12" s="23" t="n"/>
+      <c r="BA12">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(TRIM($AO$3&amp;""),"٠","0"),"١","1"),"٢","2"),"٣","3"),"٤","4"),"٥","5"),"٦","6"),"٧","7"),"٨","8"),"٩","9"),"-","/"),".","/"),"\\","/")," ","")</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="16.2" customHeight="1" thickBot="1">
       <c r="A13" s="10" t="n">
@@ -6773,8 +6808,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="45">
+  <mergeCells count="47">
     <mergeCell ref="X88:AA88"/>
+    <mergeCell ref="AN1:AP1"/>
+    <mergeCell ref="AO2:AP2"/>
     <mergeCell ref="E2:AC2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="AD87:AG87"/>
@@ -6783,6 +6820,7 @@
     <mergeCell ref="E80:J80"/>
     <mergeCell ref="F83:J83"/>
     <mergeCell ref="F88:I88"/>
+    <mergeCell ref="AO3:AP3"/>
     <mergeCell ref="L86:O86"/>
     <mergeCell ref="A46:D47"/>
     <mergeCell ref="AD1:AI2"/>
@@ -6792,7 +6830,6 @@
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="M83:S83"/>
     <mergeCell ref="X86:AA86"/>
-    <mergeCell ref="AN1:AR1"/>
     <mergeCell ref="AK5:AR5"/>
     <mergeCell ref="R88:U88"/>
     <mergeCell ref="E64:H64"/>

</xml_diff>

<commit_message>
Uniform TNR-12-bold base font across entire code grid + workbook default font set to TNR (kills the Aptos Narrow flicker on typing)
</commit_message>
<xml_diff>
--- a/uploads/inbox/SPV_ROSTER_SMART.xlsx
+++ b/uploads/inbox/SPV_ROSTER_SMART.xlsx
@@ -21,9 +21,9 @@
     <numFmt numFmtId="164" formatCode="mmmm\ yyyy"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="33">
     <font>
-      <name val="Aptos Narrow"/>
+      <name val="Times New Roman"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
@@ -212,6 +212,11 @@
       <color rgb="006B7280"/>
       <sz val="7"/>
     </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="29">
     <fill>
@@ -365,7 +370,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="37">
+  <borders count="40">
     <border>
       <left/>
       <right/>
@@ -783,11 +788,44 @@
       <right/>
       <bottom/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="007F8C8D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="007F8C8D"/>
+      </right>
+      <top style="thin">
+        <color rgb="007F8C8D"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="007F8C8D"/>
+      </right>
+      <top style="thin">
+        <color rgb="007F8C8D"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="007F8C8D"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="166">
+  <cellXfs count="182">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1244,6 +1282,52 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1919,13 +2003,11 @@
         </is>
       </c>
       <c r="AM1" s="154" t="n"/>
-      <c r="AN1" s="161" t="inlineStr">
+      <c r="AN1" s="166" t="inlineStr">
         <is>
           <t>CUSTOM PERIOD</t>
         </is>
       </c>
-      <c r="AO1" s="108" t="n"/>
-      <c r="AP1" s="108" t="n"/>
       <c r="AQ1" s="154" t="n"/>
       <c r="AR1" s="154" t="n"/>
       <c r="AS1" s="154" t="n"/>
@@ -1994,7 +2076,7 @@
         </is>
       </c>
       <c r="AO2" s="162" t="n"/>
-      <c r="AP2" s="163" t="n"/>
+      <c r="AP2" s="167" t="n"/>
       <c r="AQ2" s="164" t="n"/>
       <c r="AR2" s="154" t="n"/>
       <c r="AS2" s="154" t="n"/>
@@ -2147,7 +2229,7 @@
         </is>
       </c>
       <c r="AO3" s="162" t="n"/>
-      <c r="AP3" s="163" t="n"/>
+      <c r="AP3" s="167" t="n"/>
       <c r="AQ3" s="154" t="n"/>
       <c r="AR3" s="154" t="n"/>
       <c r="AS3" s="154" t="n"/>
@@ -2313,37 +2395,37 @@
           <t>ACT/SUPV</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
-      <c r="J5" s="6" t="n"/>
-      <c r="K5" s="6" t="n"/>
-      <c r="L5" s="6" t="n"/>
-      <c r="M5" s="6" t="n"/>
-      <c r="N5" s="6" t="n"/>
-      <c r="O5" s="6" t="n"/>
-      <c r="P5" s="6" t="n"/>
-      <c r="Q5" s="6" t="n"/>
-      <c r="R5" s="6" t="n"/>
-      <c r="S5" s="6" t="n"/>
-      <c r="T5" s="6" t="n"/>
-      <c r="U5" s="6" t="n"/>
-      <c r="V5" s="6" t="n"/>
-      <c r="W5" s="6" t="n"/>
-      <c r="X5" s="6" t="n"/>
-      <c r="Y5" s="6" t="n"/>
-      <c r="Z5" s="6" t="n"/>
-      <c r="AA5" s="6" t="n"/>
-      <c r="AB5" s="6" t="n"/>
-      <c r="AC5" s="6" t="n"/>
-      <c r="AD5" s="6" t="n"/>
-      <c r="AE5" s="6" t="n"/>
-      <c r="AF5" s="6" t="n"/>
-      <c r="AG5" s="6" t="n"/>
-      <c r="AH5" s="26" t="n"/>
-      <c r="AI5" s="23" t="n"/>
+      <c r="E5" s="168" t="n"/>
+      <c r="F5" s="168" t="n"/>
+      <c r="G5" s="169" t="n"/>
+      <c r="H5" s="168" t="n"/>
+      <c r="I5" s="168" t="n"/>
+      <c r="J5" s="168" t="n"/>
+      <c r="K5" s="168" t="n"/>
+      <c r="L5" s="168" t="n"/>
+      <c r="M5" s="168" t="n"/>
+      <c r="N5" s="168" t="n"/>
+      <c r="O5" s="168" t="n"/>
+      <c r="P5" s="168" t="n"/>
+      <c r="Q5" s="168" t="n"/>
+      <c r="R5" s="168" t="n"/>
+      <c r="S5" s="168" t="n"/>
+      <c r="T5" s="168" t="n"/>
+      <c r="U5" s="168" t="n"/>
+      <c r="V5" s="168" t="n"/>
+      <c r="W5" s="168" t="n"/>
+      <c r="X5" s="168" t="n"/>
+      <c r="Y5" s="168" t="n"/>
+      <c r="Z5" s="168" t="n"/>
+      <c r="AA5" s="168" t="n"/>
+      <c r="AB5" s="168" t="n"/>
+      <c r="AC5" s="168" t="n"/>
+      <c r="AD5" s="168" t="n"/>
+      <c r="AE5" s="168" t="n"/>
+      <c r="AF5" s="168" t="n"/>
+      <c r="AG5" s="168" t="n"/>
+      <c r="AH5" s="170" t="n"/>
+      <c r="AI5" s="171" t="n"/>
       <c r="AK5" s="165">
         <f>IF($BA$1="P","● PERIOD MODE — "&amp;TEXT($BA$3,"dd/mm/yyyy")&amp;" +"&amp;$BA$4&amp;"d","● MONTH MODE")</f>
         <v/>
@@ -2371,37 +2453,37 @@
           <t>ACT/SUPV</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="7" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
-      <c r="J6" s="6" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="6" t="n"/>
-      <c r="M6" s="6" t="n"/>
-      <c r="N6" s="6" t="n"/>
-      <c r="O6" s="6" t="n"/>
-      <c r="P6" s="6" t="n"/>
-      <c r="Q6" s="6" t="n"/>
-      <c r="R6" s="6" t="n"/>
-      <c r="S6" s="6" t="n"/>
-      <c r="T6" s="6" t="n"/>
-      <c r="U6" s="6" t="n"/>
-      <c r="V6" s="6" t="n"/>
-      <c r="W6" s="6" t="n"/>
-      <c r="X6" s="6" t="n"/>
-      <c r="Y6" s="6" t="n"/>
-      <c r="Z6" s="6" t="n"/>
-      <c r="AA6" s="6" t="n"/>
-      <c r="AB6" s="6" t="n"/>
-      <c r="AC6" s="6" t="n"/>
-      <c r="AD6" s="6" t="n"/>
-      <c r="AE6" s="6" t="n"/>
-      <c r="AF6" s="6" t="n"/>
-      <c r="AG6" s="6" t="n"/>
-      <c r="AH6" s="26" t="n"/>
-      <c r="AI6" s="23" t="n"/>
+      <c r="E6" s="168" t="n"/>
+      <c r="F6" s="168" t="n"/>
+      <c r="G6" s="169" t="n"/>
+      <c r="H6" s="168" t="n"/>
+      <c r="I6" s="168" t="n"/>
+      <c r="J6" s="168" t="n"/>
+      <c r="K6" s="168" t="n"/>
+      <c r="L6" s="168" t="n"/>
+      <c r="M6" s="168" t="n"/>
+      <c r="N6" s="168" t="n"/>
+      <c r="O6" s="168" t="n"/>
+      <c r="P6" s="168" t="n"/>
+      <c r="Q6" s="168" t="n"/>
+      <c r="R6" s="168" t="n"/>
+      <c r="S6" s="168" t="n"/>
+      <c r="T6" s="168" t="n"/>
+      <c r="U6" s="168" t="n"/>
+      <c r="V6" s="168" t="n"/>
+      <c r="W6" s="168" t="n"/>
+      <c r="X6" s="168" t="n"/>
+      <c r="Y6" s="168" t="n"/>
+      <c r="Z6" s="168" t="n"/>
+      <c r="AA6" s="168" t="n"/>
+      <c r="AB6" s="168" t="n"/>
+      <c r="AC6" s="168" t="n"/>
+      <c r="AD6" s="168" t="n"/>
+      <c r="AE6" s="168" t="n"/>
+      <c r="AF6" s="168" t="n"/>
+      <c r="AG6" s="168" t="n"/>
+      <c r="AH6" s="170" t="n"/>
+      <c r="AI6" s="171" t="n"/>
       <c r="BA6">
         <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(TRIM($AO$2&amp;""),"٠","0"),"١","1"),"٢","2"),"٣","3"),"٤","4"),"٥","5"),"٦","6"),"٧","7"),"٨","8"),"٩","9"),"-","/"),".","/"),"\\","/")," ","")</f>
         <v/>
@@ -2424,37 +2506,37 @@
           <t>ACT/SUPV</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="n"/>
-      <c r="K7" s="6" t="n"/>
-      <c r="L7" s="6" t="n"/>
-      <c r="M7" s="6" t="n"/>
-      <c r="N7" s="6" t="n"/>
-      <c r="O7" s="6" t="n"/>
-      <c r="P7" s="6" t="n"/>
-      <c r="Q7" s="6" t="n"/>
-      <c r="R7" s="6" t="n"/>
-      <c r="S7" s="6" t="n"/>
-      <c r="T7" s="6" t="n"/>
-      <c r="U7" s="6" t="n"/>
-      <c r="V7" s="6" t="n"/>
-      <c r="W7" s="6" t="n"/>
-      <c r="X7" s="6" t="n"/>
-      <c r="Y7" s="6" t="n"/>
-      <c r="Z7" s="6" t="n"/>
-      <c r="AA7" s="6" t="n"/>
-      <c r="AB7" s="6" t="n"/>
-      <c r="AC7" s="6" t="n"/>
-      <c r="AD7" s="6" t="n"/>
-      <c r="AE7" s="6" t="n"/>
-      <c r="AF7" s="6" t="n"/>
-      <c r="AG7" s="6" t="n"/>
-      <c r="AH7" s="26" t="n"/>
-      <c r="AI7" s="23" t="n"/>
+      <c r="E7" s="168" t="n"/>
+      <c r="F7" s="168" t="n"/>
+      <c r="G7" s="169" t="n"/>
+      <c r="H7" s="168" t="n"/>
+      <c r="I7" s="168" t="n"/>
+      <c r="J7" s="168" t="n"/>
+      <c r="K7" s="168" t="n"/>
+      <c r="L7" s="168" t="n"/>
+      <c r="M7" s="168" t="n"/>
+      <c r="N7" s="168" t="n"/>
+      <c r="O7" s="168" t="n"/>
+      <c r="P7" s="168" t="n"/>
+      <c r="Q7" s="168" t="n"/>
+      <c r="R7" s="168" t="n"/>
+      <c r="S7" s="168" t="n"/>
+      <c r="T7" s="168" t="n"/>
+      <c r="U7" s="168" t="n"/>
+      <c r="V7" s="168" t="n"/>
+      <c r="W7" s="168" t="n"/>
+      <c r="X7" s="168" t="n"/>
+      <c r="Y7" s="168" t="n"/>
+      <c r="Z7" s="168" t="n"/>
+      <c r="AA7" s="168" t="n"/>
+      <c r="AB7" s="168" t="n"/>
+      <c r="AC7" s="168" t="n"/>
+      <c r="AD7" s="168" t="n"/>
+      <c r="AE7" s="168" t="n"/>
+      <c r="AF7" s="168" t="n"/>
+      <c r="AG7" s="168" t="n"/>
+      <c r="AH7" s="170" t="n"/>
+      <c r="AI7" s="171" t="n"/>
       <c r="BA7">
         <f>IFERROR(FIND("/",$BA$6),0)</f>
         <v/>
@@ -2477,37 +2559,37 @@
           <t>ACT/SUPV</t>
         </is>
       </c>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="n"/>
-      <c r="K8" s="6" t="n"/>
-      <c r="L8" s="6" t="n"/>
-      <c r="M8" s="6" t="n"/>
-      <c r="N8" s="6" t="n"/>
-      <c r="O8" s="6" t="n"/>
-      <c r="P8" s="6" t="n"/>
-      <c r="Q8" s="6" t="n"/>
-      <c r="R8" s="6" t="n"/>
-      <c r="S8" s="6" t="n"/>
-      <c r="T8" s="6" t="n"/>
-      <c r="U8" s="6" t="n"/>
-      <c r="V8" s="6" t="n"/>
-      <c r="W8" s="6" t="n"/>
-      <c r="X8" s="6" t="n"/>
-      <c r="Y8" s="6" t="n"/>
-      <c r="Z8" s="6" t="n"/>
-      <c r="AA8" s="6" t="n"/>
-      <c r="AB8" s="6" t="n"/>
-      <c r="AC8" s="6" t="n"/>
-      <c r="AD8" s="6" t="n"/>
-      <c r="AE8" s="6" t="n"/>
-      <c r="AF8" s="6" t="n"/>
-      <c r="AG8" s="6" t="n"/>
-      <c r="AH8" s="26" t="n"/>
-      <c r="AI8" s="23" t="n"/>
+      <c r="E8" s="168" t="n"/>
+      <c r="F8" s="168" t="n"/>
+      <c r="G8" s="169" t="n"/>
+      <c r="H8" s="168" t="n"/>
+      <c r="I8" s="168" t="n"/>
+      <c r="J8" s="168" t="n"/>
+      <c r="K8" s="168" t="n"/>
+      <c r="L8" s="168" t="n"/>
+      <c r="M8" s="168" t="n"/>
+      <c r="N8" s="168" t="n"/>
+      <c r="O8" s="168" t="n"/>
+      <c r="P8" s="168" t="n"/>
+      <c r="Q8" s="168" t="n"/>
+      <c r="R8" s="168" t="n"/>
+      <c r="S8" s="168" t="n"/>
+      <c r="T8" s="168" t="n"/>
+      <c r="U8" s="168" t="n"/>
+      <c r="V8" s="168" t="n"/>
+      <c r="W8" s="168" t="n"/>
+      <c r="X8" s="168" t="n"/>
+      <c r="Y8" s="168" t="n"/>
+      <c r="Z8" s="168" t="n"/>
+      <c r="AA8" s="168" t="n"/>
+      <c r="AB8" s="168" t="n"/>
+      <c r="AC8" s="168" t="n"/>
+      <c r="AD8" s="168" t="n"/>
+      <c r="AE8" s="168" t="n"/>
+      <c r="AF8" s="168" t="n"/>
+      <c r="AG8" s="168" t="n"/>
+      <c r="AH8" s="170" t="n"/>
+      <c r="AI8" s="171" t="n"/>
       <c r="BA8">
         <f>IFERROR(FIND("/",$BA$6,$BA$7+1),0)</f>
         <v/>
@@ -2530,37 +2612,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
-      <c r="J9" s="6" t="n"/>
-      <c r="K9" s="6" t="n"/>
-      <c r="L9" s="6" t="n"/>
-      <c r="M9" s="6" t="n"/>
-      <c r="N9" s="6" t="n"/>
-      <c r="O9" s="6" t="n"/>
-      <c r="P9" s="6" t="n"/>
-      <c r="Q9" s="6" t="n"/>
-      <c r="R9" s="6" t="n"/>
-      <c r="S9" s="6" t="n"/>
-      <c r="T9" s="6" t="n"/>
-      <c r="U9" s="6" t="n"/>
-      <c r="V9" s="6" t="n"/>
-      <c r="W9" s="6" t="n"/>
-      <c r="X9" s="6" t="n"/>
-      <c r="Y9" s="6" t="n"/>
-      <c r="Z9" s="6" t="n"/>
-      <c r="AA9" s="6" t="n"/>
-      <c r="AB9" s="6" t="n"/>
-      <c r="AC9" s="6" t="n"/>
-      <c r="AD9" s="6" t="n"/>
-      <c r="AE9" s="6" t="n"/>
-      <c r="AF9" s="6" t="n"/>
-      <c r="AG9" s="6" t="n"/>
-      <c r="AH9" s="26" t="n"/>
-      <c r="AI9" s="23" t="n"/>
+      <c r="E9" s="168" t="n"/>
+      <c r="F9" s="168" t="n"/>
+      <c r="G9" s="169" t="n"/>
+      <c r="H9" s="168" t="n"/>
+      <c r="I9" s="168" t="n"/>
+      <c r="J9" s="168" t="n"/>
+      <c r="K9" s="168" t="n"/>
+      <c r="L9" s="168" t="n"/>
+      <c r="M9" s="168" t="n"/>
+      <c r="N9" s="168" t="n"/>
+      <c r="O9" s="168" t="n"/>
+      <c r="P9" s="168" t="n"/>
+      <c r="Q9" s="168" t="n"/>
+      <c r="R9" s="168" t="n"/>
+      <c r="S9" s="168" t="n"/>
+      <c r="T9" s="168" t="n"/>
+      <c r="U9" s="168" t="n"/>
+      <c r="V9" s="168" t="n"/>
+      <c r="W9" s="168" t="n"/>
+      <c r="X9" s="168" t="n"/>
+      <c r="Y9" s="168" t="n"/>
+      <c r="Z9" s="168" t="n"/>
+      <c r="AA9" s="168" t="n"/>
+      <c r="AB9" s="168" t="n"/>
+      <c r="AC9" s="168" t="n"/>
+      <c r="AD9" s="168" t="n"/>
+      <c r="AE9" s="168" t="n"/>
+      <c r="AF9" s="168" t="n"/>
+      <c r="AG9" s="168" t="n"/>
+      <c r="AH9" s="170" t="n"/>
+      <c r="AI9" s="171" t="n"/>
       <c r="BA9">
         <f>IFERROR(VALUE(LEFT($BA$6,$BA$7-1)),"")</f>
         <v/>
@@ -2583,37 +2665,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
-      <c r="J10" s="6" t="n"/>
-      <c r="K10" s="6" t="n"/>
-      <c r="L10" s="6" t="n"/>
-      <c r="M10" s="6" t="n"/>
-      <c r="N10" s="6" t="n"/>
-      <c r="O10" s="6" t="n"/>
-      <c r="P10" s="6" t="n"/>
-      <c r="Q10" s="6" t="n"/>
-      <c r="R10" s="6" t="n"/>
-      <c r="S10" s="6" t="n"/>
-      <c r="T10" s="6" t="n"/>
-      <c r="U10" s="6" t="n"/>
-      <c r="V10" s="6" t="n"/>
-      <c r="W10" s="6" t="n"/>
-      <c r="X10" s="6" t="n"/>
-      <c r="Y10" s="6" t="n"/>
-      <c r="Z10" s="6" t="n"/>
-      <c r="AA10" s="6" t="n"/>
-      <c r="AB10" s="6" t="n"/>
-      <c r="AC10" s="6" t="n"/>
-      <c r="AD10" s="6" t="n"/>
-      <c r="AE10" s="6" t="n"/>
-      <c r="AF10" s="6" t="n"/>
-      <c r="AG10" s="6" t="n"/>
-      <c r="AH10" s="26" t="n"/>
-      <c r="AI10" s="23" t="n"/>
+      <c r="E10" s="168" t="n"/>
+      <c r="F10" s="168" t="n"/>
+      <c r="G10" s="169" t="n"/>
+      <c r="H10" s="168" t="n"/>
+      <c r="I10" s="168" t="n"/>
+      <c r="J10" s="168" t="n"/>
+      <c r="K10" s="168" t="n"/>
+      <c r="L10" s="168" t="n"/>
+      <c r="M10" s="168" t="n"/>
+      <c r="N10" s="168" t="n"/>
+      <c r="O10" s="168" t="n"/>
+      <c r="P10" s="168" t="n"/>
+      <c r="Q10" s="168" t="n"/>
+      <c r="R10" s="168" t="n"/>
+      <c r="S10" s="168" t="n"/>
+      <c r="T10" s="168" t="n"/>
+      <c r="U10" s="168" t="n"/>
+      <c r="V10" s="168" t="n"/>
+      <c r="W10" s="168" t="n"/>
+      <c r="X10" s="168" t="n"/>
+      <c r="Y10" s="168" t="n"/>
+      <c r="Z10" s="168" t="n"/>
+      <c r="AA10" s="168" t="n"/>
+      <c r="AB10" s="168" t="n"/>
+      <c r="AC10" s="168" t="n"/>
+      <c r="AD10" s="168" t="n"/>
+      <c r="AE10" s="168" t="n"/>
+      <c r="AF10" s="168" t="n"/>
+      <c r="AG10" s="168" t="n"/>
+      <c r="AH10" s="170" t="n"/>
+      <c r="AI10" s="171" t="n"/>
       <c r="BA10">
         <f>IFERROR(VALUE(MID($BA$6,$BA$7+1,$BA$8-$BA$7-1)),"")</f>
         <v/>
@@ -2636,37 +2718,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="6" t="n"/>
-      <c r="I11" s="6" t="n"/>
-      <c r="J11" s="6" t="n"/>
-      <c r="K11" s="6" t="n"/>
-      <c r="L11" s="6" t="n"/>
-      <c r="M11" s="6" t="n"/>
-      <c r="N11" s="6" t="n"/>
-      <c r="O11" s="6" t="n"/>
-      <c r="P11" s="6" t="n"/>
-      <c r="Q11" s="6" t="n"/>
-      <c r="R11" s="6" t="n"/>
-      <c r="S11" s="6" t="n"/>
-      <c r="T11" s="6" t="n"/>
-      <c r="U11" s="6" t="n"/>
-      <c r="V11" s="6" t="n"/>
-      <c r="W11" s="6" t="n"/>
-      <c r="X11" s="6" t="n"/>
-      <c r="Y11" s="6" t="n"/>
-      <c r="Z11" s="6" t="n"/>
-      <c r="AA11" s="6" t="n"/>
-      <c r="AB11" s="6" t="n"/>
-      <c r="AC11" s="6" t="n"/>
-      <c r="AD11" s="6" t="n"/>
-      <c r="AE11" s="6" t="n"/>
-      <c r="AF11" s="6" t="n"/>
-      <c r="AG11" s="6" t="n"/>
-      <c r="AH11" s="26" t="n"/>
-      <c r="AI11" s="23" t="n"/>
+      <c r="E11" s="168" t="n"/>
+      <c r="F11" s="168" t="n"/>
+      <c r="G11" s="169" t="n"/>
+      <c r="H11" s="168" t="n"/>
+      <c r="I11" s="168" t="n"/>
+      <c r="J11" s="168" t="n"/>
+      <c r="K11" s="168" t="n"/>
+      <c r="L11" s="168" t="n"/>
+      <c r="M11" s="168" t="n"/>
+      <c r="N11" s="168" t="n"/>
+      <c r="O11" s="168" t="n"/>
+      <c r="P11" s="168" t="n"/>
+      <c r="Q11" s="168" t="n"/>
+      <c r="R11" s="168" t="n"/>
+      <c r="S11" s="168" t="n"/>
+      <c r="T11" s="168" t="n"/>
+      <c r="U11" s="168" t="n"/>
+      <c r="V11" s="168" t="n"/>
+      <c r="W11" s="168" t="n"/>
+      <c r="X11" s="168" t="n"/>
+      <c r="Y11" s="168" t="n"/>
+      <c r="Z11" s="168" t="n"/>
+      <c r="AA11" s="168" t="n"/>
+      <c r="AB11" s="168" t="n"/>
+      <c r="AC11" s="168" t="n"/>
+      <c r="AD11" s="168" t="n"/>
+      <c r="AE11" s="168" t="n"/>
+      <c r="AF11" s="168" t="n"/>
+      <c r="AG11" s="168" t="n"/>
+      <c r="AH11" s="170" t="n"/>
+      <c r="AI11" s="171" t="n"/>
       <c r="BA11">
         <f>IFERROR(VALUE(MID($BA$6,$BA$8+1,9)),"")</f>
         <v/>
@@ -2689,37 +2771,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="7" t="n"/>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="6" t="n"/>
-      <c r="J12" s="6" t="n"/>
-      <c r="K12" s="6" t="n"/>
-      <c r="L12" s="6" t="n"/>
-      <c r="M12" s="6" t="n"/>
-      <c r="N12" s="6" t="n"/>
-      <c r="O12" s="6" t="n"/>
-      <c r="P12" s="6" t="n"/>
-      <c r="Q12" s="6" t="n"/>
-      <c r="R12" s="6" t="n"/>
-      <c r="S12" s="6" t="n"/>
-      <c r="T12" s="6" t="n"/>
-      <c r="U12" s="6" t="n"/>
-      <c r="V12" s="6" t="n"/>
-      <c r="W12" s="6" t="n"/>
-      <c r="X12" s="6" t="n"/>
-      <c r="Y12" s="6" t="n"/>
-      <c r="Z12" s="6" t="n"/>
-      <c r="AA12" s="6" t="n"/>
-      <c r="AB12" s="6" t="n"/>
-      <c r="AC12" s="6" t="n"/>
-      <c r="AD12" s="6" t="n"/>
-      <c r="AE12" s="6" t="n"/>
-      <c r="AF12" s="6" t="n"/>
-      <c r="AG12" s="6" t="n"/>
-      <c r="AH12" s="26" t="n"/>
-      <c r="AI12" s="23" t="n"/>
+      <c r="E12" s="168" t="n"/>
+      <c r="F12" s="168" t="n"/>
+      <c r="G12" s="169" t="n"/>
+      <c r="H12" s="168" t="n"/>
+      <c r="I12" s="168" t="n"/>
+      <c r="J12" s="168" t="n"/>
+      <c r="K12" s="168" t="n"/>
+      <c r="L12" s="168" t="n"/>
+      <c r="M12" s="168" t="n"/>
+      <c r="N12" s="168" t="n"/>
+      <c r="O12" s="168" t="n"/>
+      <c r="P12" s="168" t="n"/>
+      <c r="Q12" s="168" t="n"/>
+      <c r="R12" s="168" t="n"/>
+      <c r="S12" s="168" t="n"/>
+      <c r="T12" s="168" t="n"/>
+      <c r="U12" s="168" t="n"/>
+      <c r="V12" s="168" t="n"/>
+      <c r="W12" s="168" t="n"/>
+      <c r="X12" s="168" t="n"/>
+      <c r="Y12" s="168" t="n"/>
+      <c r="Z12" s="168" t="n"/>
+      <c r="AA12" s="168" t="n"/>
+      <c r="AB12" s="168" t="n"/>
+      <c r="AC12" s="168" t="n"/>
+      <c r="AD12" s="168" t="n"/>
+      <c r="AE12" s="168" t="n"/>
+      <c r="AF12" s="168" t="n"/>
+      <c r="AG12" s="168" t="n"/>
+      <c r="AH12" s="170" t="n"/>
+      <c r="AI12" s="171" t="n"/>
       <c r="BA12">
         <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(TRIM($AO$3&amp;""),"٠","0"),"١","1"),"٢","2"),"٣","3"),"٤","4"),"٥","5"),"٦","6"),"٧","7"),"٨","8"),"٩","9"),"-","/"),".","/"),"\\","/")," ","")</f>
         <v/>
@@ -2742,37 +2824,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="6" t="n"/>
-      <c r="J13" s="6" t="n"/>
-      <c r="K13" s="6" t="n"/>
-      <c r="L13" s="6" t="n"/>
-      <c r="M13" s="6" t="n"/>
-      <c r="N13" s="6" t="n"/>
-      <c r="O13" s="6" t="n"/>
-      <c r="P13" s="6" t="n"/>
-      <c r="Q13" s="6" t="n"/>
-      <c r="R13" s="6" t="n"/>
-      <c r="S13" s="6" t="n"/>
-      <c r="T13" s="6" t="n"/>
-      <c r="U13" s="6" t="n"/>
-      <c r="V13" s="6" t="n"/>
-      <c r="W13" s="6" t="n"/>
-      <c r="X13" s="6" t="n"/>
-      <c r="Y13" s="6" t="n"/>
-      <c r="Z13" s="6" t="n"/>
-      <c r="AA13" s="6" t="n"/>
-      <c r="AB13" s="6" t="n"/>
-      <c r="AC13" s="6" t="n"/>
-      <c r="AD13" s="6" t="n"/>
-      <c r="AE13" s="6" t="n"/>
-      <c r="AF13" s="6" t="n"/>
-      <c r="AG13" s="6" t="n"/>
-      <c r="AH13" s="26" t="n"/>
-      <c r="AI13" s="23" t="n"/>
+      <c r="E13" s="168" t="n"/>
+      <c r="F13" s="168" t="n"/>
+      <c r="G13" s="169" t="n"/>
+      <c r="H13" s="168" t="n"/>
+      <c r="I13" s="168" t="n"/>
+      <c r="J13" s="168" t="n"/>
+      <c r="K13" s="168" t="n"/>
+      <c r="L13" s="168" t="n"/>
+      <c r="M13" s="168" t="n"/>
+      <c r="N13" s="168" t="n"/>
+      <c r="O13" s="168" t="n"/>
+      <c r="P13" s="168" t="n"/>
+      <c r="Q13" s="168" t="n"/>
+      <c r="R13" s="168" t="n"/>
+      <c r="S13" s="168" t="n"/>
+      <c r="T13" s="168" t="n"/>
+      <c r="U13" s="168" t="n"/>
+      <c r="V13" s="168" t="n"/>
+      <c r="W13" s="168" t="n"/>
+      <c r="X13" s="168" t="n"/>
+      <c r="Y13" s="168" t="n"/>
+      <c r="Z13" s="168" t="n"/>
+      <c r="AA13" s="168" t="n"/>
+      <c r="AB13" s="168" t="n"/>
+      <c r="AC13" s="168" t="n"/>
+      <c r="AD13" s="168" t="n"/>
+      <c r="AE13" s="168" t="n"/>
+      <c r="AF13" s="168" t="n"/>
+      <c r="AG13" s="168" t="n"/>
+      <c r="AH13" s="170" t="n"/>
+      <c r="AI13" s="171" t="n"/>
     </row>
     <row r="14" ht="16.2" customHeight="1" thickBot="1">
       <c r="A14" s="10" t="n">
@@ -2791,37 +2873,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
-      <c r="H14" s="11" t="n"/>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="11" t="n"/>
-      <c r="K14" s="11" t="n"/>
-      <c r="L14" s="11" t="n"/>
-      <c r="M14" s="11" t="n"/>
-      <c r="N14" s="11" t="n"/>
-      <c r="O14" s="11" t="n"/>
-      <c r="P14" s="11" t="n"/>
-      <c r="Q14" s="11" t="n"/>
-      <c r="R14" s="11" t="n"/>
-      <c r="S14" s="11" t="n"/>
-      <c r="T14" s="11" t="n"/>
-      <c r="U14" s="11" t="n"/>
-      <c r="V14" s="11" t="n"/>
-      <c r="W14" s="11" t="n"/>
-      <c r="X14" s="11" t="n"/>
-      <c r="Y14" s="11" t="n"/>
-      <c r="Z14" s="11" t="n"/>
-      <c r="AA14" s="11" t="n"/>
-      <c r="AB14" s="11" t="n"/>
-      <c r="AC14" s="11" t="n"/>
-      <c r="AD14" s="11" t="n"/>
-      <c r="AE14" s="11" t="n"/>
-      <c r="AF14" s="11" t="n"/>
-      <c r="AG14" s="11" t="n"/>
-      <c r="AH14" s="11" t="n"/>
-      <c r="AI14" s="23" t="n"/>
+      <c r="E14" s="172" t="n"/>
+      <c r="F14" s="172" t="n"/>
+      <c r="G14" s="172" t="n"/>
+      <c r="H14" s="172" t="n"/>
+      <c r="I14" s="172" t="n"/>
+      <c r="J14" s="172" t="n"/>
+      <c r="K14" s="172" t="n"/>
+      <c r="L14" s="172" t="n"/>
+      <c r="M14" s="172" t="n"/>
+      <c r="N14" s="172" t="n"/>
+      <c r="O14" s="172" t="n"/>
+      <c r="P14" s="172" t="n"/>
+      <c r="Q14" s="172" t="n"/>
+      <c r="R14" s="172" t="n"/>
+      <c r="S14" s="172" t="n"/>
+      <c r="T14" s="172" t="n"/>
+      <c r="U14" s="172" t="n"/>
+      <c r="V14" s="172" t="n"/>
+      <c r="W14" s="172" t="n"/>
+      <c r="X14" s="172" t="n"/>
+      <c r="Y14" s="172" t="n"/>
+      <c r="Z14" s="172" t="n"/>
+      <c r="AA14" s="172" t="n"/>
+      <c r="AB14" s="172" t="n"/>
+      <c r="AC14" s="172" t="n"/>
+      <c r="AD14" s="172" t="n"/>
+      <c r="AE14" s="172" t="n"/>
+      <c r="AF14" s="172" t="n"/>
+      <c r="AG14" s="172" t="n"/>
+      <c r="AH14" s="172" t="n"/>
+      <c r="AI14" s="171" t="n"/>
     </row>
     <row r="15" ht="16.2" customHeight="1" thickBot="1">
       <c r="A15" s="10" t="n">
@@ -2840,37 +2922,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="7" t="n"/>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="6" t="n"/>
-      <c r="J15" s="6" t="n"/>
-      <c r="K15" s="6" t="n"/>
-      <c r="L15" s="6" t="n"/>
-      <c r="M15" s="6" t="n"/>
-      <c r="N15" s="6" t="n"/>
-      <c r="O15" s="6" t="n"/>
-      <c r="P15" s="6" t="n"/>
-      <c r="Q15" s="6" t="n"/>
-      <c r="R15" s="6" t="n"/>
-      <c r="S15" s="6" t="n"/>
-      <c r="T15" s="6" t="n"/>
-      <c r="U15" s="6" t="n"/>
-      <c r="V15" s="6" t="n"/>
-      <c r="W15" s="6" t="n"/>
-      <c r="X15" s="6" t="n"/>
-      <c r="Y15" s="6" t="n"/>
-      <c r="Z15" s="6" t="n"/>
-      <c r="AA15" s="6" t="n"/>
-      <c r="AB15" s="6" t="n"/>
-      <c r="AC15" s="6" t="n"/>
-      <c r="AD15" s="6" t="n"/>
-      <c r="AE15" s="6" t="n"/>
-      <c r="AF15" s="6" t="n"/>
-      <c r="AG15" s="6" t="n"/>
-      <c r="AH15" s="26" t="n"/>
-      <c r="AI15" s="23" t="n"/>
+      <c r="E15" s="168" t="n"/>
+      <c r="F15" s="168" t="n"/>
+      <c r="G15" s="169" t="n"/>
+      <c r="H15" s="168" t="n"/>
+      <c r="I15" s="168" t="n"/>
+      <c r="J15" s="168" t="n"/>
+      <c r="K15" s="168" t="n"/>
+      <c r="L15" s="168" t="n"/>
+      <c r="M15" s="168" t="n"/>
+      <c r="N15" s="168" t="n"/>
+      <c r="O15" s="168" t="n"/>
+      <c r="P15" s="168" t="n"/>
+      <c r="Q15" s="168" t="n"/>
+      <c r="R15" s="168" t="n"/>
+      <c r="S15" s="168" t="n"/>
+      <c r="T15" s="168" t="n"/>
+      <c r="U15" s="168" t="n"/>
+      <c r="V15" s="168" t="n"/>
+      <c r="W15" s="168" t="n"/>
+      <c r="X15" s="168" t="n"/>
+      <c r="Y15" s="168" t="n"/>
+      <c r="Z15" s="168" t="n"/>
+      <c r="AA15" s="168" t="n"/>
+      <c r="AB15" s="168" t="n"/>
+      <c r="AC15" s="168" t="n"/>
+      <c r="AD15" s="168" t="n"/>
+      <c r="AE15" s="168" t="n"/>
+      <c r="AF15" s="168" t="n"/>
+      <c r="AG15" s="168" t="n"/>
+      <c r="AH15" s="170" t="n"/>
+      <c r="AI15" s="171" t="n"/>
     </row>
     <row r="16" ht="16.2" customHeight="1" thickBot="1">
       <c r="A16" s="8" t="n">
@@ -2889,37 +2971,37 @@
           <t>FITTER</t>
         </is>
       </c>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="7" t="n"/>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="6" t="n"/>
-      <c r="J16" s="6" t="n"/>
-      <c r="K16" s="6" t="n"/>
-      <c r="L16" s="6" t="n"/>
-      <c r="M16" s="6" t="n"/>
-      <c r="N16" s="6" t="n"/>
-      <c r="O16" s="6" t="n"/>
-      <c r="P16" s="6" t="n"/>
-      <c r="Q16" s="6" t="n"/>
-      <c r="R16" s="6" t="n"/>
-      <c r="S16" s="6" t="n"/>
-      <c r="T16" s="6" t="n"/>
-      <c r="U16" s="6" t="n"/>
-      <c r="V16" s="6" t="n"/>
-      <c r="W16" s="6" t="n"/>
-      <c r="X16" s="6" t="n"/>
-      <c r="Y16" s="6" t="n"/>
-      <c r="Z16" s="6" t="n"/>
-      <c r="AA16" s="6" t="n"/>
-      <c r="AB16" s="6" t="n"/>
-      <c r="AC16" s="6" t="n"/>
-      <c r="AD16" s="6" t="n"/>
-      <c r="AE16" s="6" t="n"/>
-      <c r="AF16" s="6" t="n"/>
-      <c r="AG16" s="6" t="n"/>
-      <c r="AH16" s="26" t="n"/>
-      <c r="AI16" s="23" t="n"/>
+      <c r="E16" s="168" t="n"/>
+      <c r="F16" s="168" t="n"/>
+      <c r="G16" s="169" t="n"/>
+      <c r="H16" s="168" t="n"/>
+      <c r="I16" s="168" t="n"/>
+      <c r="J16" s="168" t="n"/>
+      <c r="K16" s="168" t="n"/>
+      <c r="L16" s="168" t="n"/>
+      <c r="M16" s="168" t="n"/>
+      <c r="N16" s="168" t="n"/>
+      <c r="O16" s="168" t="n"/>
+      <c r="P16" s="168" t="n"/>
+      <c r="Q16" s="168" t="n"/>
+      <c r="R16" s="168" t="n"/>
+      <c r="S16" s="168" t="n"/>
+      <c r="T16" s="168" t="n"/>
+      <c r="U16" s="168" t="n"/>
+      <c r="V16" s="168" t="n"/>
+      <c r="W16" s="168" t="n"/>
+      <c r="X16" s="168" t="n"/>
+      <c r="Y16" s="168" t="n"/>
+      <c r="Z16" s="168" t="n"/>
+      <c r="AA16" s="168" t="n"/>
+      <c r="AB16" s="168" t="n"/>
+      <c r="AC16" s="168" t="n"/>
+      <c r="AD16" s="168" t="n"/>
+      <c r="AE16" s="168" t="n"/>
+      <c r="AF16" s="168" t="n"/>
+      <c r="AG16" s="168" t="n"/>
+      <c r="AH16" s="170" t="n"/>
+      <c r="AI16" s="171" t="n"/>
     </row>
     <row r="17" ht="16.2" customHeight="1" thickBot="1">
       <c r="A17" s="8" t="n">
@@ -2938,37 +3020,37 @@
           <t>FITTER</t>
         </is>
       </c>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="6" t="n"/>
-      <c r="J17" s="6" t="n"/>
-      <c r="K17" s="6" t="n"/>
-      <c r="L17" s="6" t="n"/>
-      <c r="M17" s="6" t="n"/>
-      <c r="N17" s="6" t="n"/>
-      <c r="O17" s="6" t="n"/>
-      <c r="P17" s="6" t="n"/>
-      <c r="Q17" s="6" t="n"/>
-      <c r="R17" s="6" t="n"/>
-      <c r="S17" s="6" t="n"/>
-      <c r="T17" s="6" t="n"/>
-      <c r="U17" s="6" t="n"/>
-      <c r="V17" s="6" t="n"/>
-      <c r="W17" s="6" t="n"/>
-      <c r="X17" s="6" t="n"/>
-      <c r="Y17" s="6" t="n"/>
-      <c r="Z17" s="6" t="n"/>
-      <c r="AA17" s="6" t="n"/>
-      <c r="AB17" s="6" t="n"/>
-      <c r="AC17" s="6" t="n"/>
-      <c r="AD17" s="6" t="n"/>
-      <c r="AE17" s="6" t="n"/>
-      <c r="AF17" s="6" t="n"/>
-      <c r="AG17" s="6" t="n"/>
-      <c r="AH17" s="26" t="n"/>
-      <c r="AI17" s="23" t="n"/>
+      <c r="E17" s="168" t="n"/>
+      <c r="F17" s="168" t="n"/>
+      <c r="G17" s="169" t="n"/>
+      <c r="H17" s="168" t="n"/>
+      <c r="I17" s="168" t="n"/>
+      <c r="J17" s="168" t="n"/>
+      <c r="K17" s="168" t="n"/>
+      <c r="L17" s="168" t="n"/>
+      <c r="M17" s="168" t="n"/>
+      <c r="N17" s="168" t="n"/>
+      <c r="O17" s="168" t="n"/>
+      <c r="P17" s="168" t="n"/>
+      <c r="Q17" s="168" t="n"/>
+      <c r="R17" s="168" t="n"/>
+      <c r="S17" s="168" t="n"/>
+      <c r="T17" s="168" t="n"/>
+      <c r="U17" s="168" t="n"/>
+      <c r="V17" s="168" t="n"/>
+      <c r="W17" s="168" t="n"/>
+      <c r="X17" s="168" t="n"/>
+      <c r="Y17" s="168" t="n"/>
+      <c r="Z17" s="168" t="n"/>
+      <c r="AA17" s="168" t="n"/>
+      <c r="AB17" s="168" t="n"/>
+      <c r="AC17" s="168" t="n"/>
+      <c r="AD17" s="168" t="n"/>
+      <c r="AE17" s="168" t="n"/>
+      <c r="AF17" s="168" t="n"/>
+      <c r="AG17" s="168" t="n"/>
+      <c r="AH17" s="170" t="n"/>
+      <c r="AI17" s="171" t="n"/>
     </row>
     <row r="18" ht="16.2" customHeight="1" thickBot="1">
       <c r="A18" s="8" t="n">
@@ -2987,37 +3069,37 @@
           <t>FITTER</t>
         </is>
       </c>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="6" t="n"/>
-      <c r="I18" s="6" t="n"/>
-      <c r="J18" s="6" t="n"/>
-      <c r="K18" s="6" t="n"/>
-      <c r="L18" s="6" t="n"/>
-      <c r="M18" s="6" t="n"/>
-      <c r="N18" s="6" t="n"/>
-      <c r="O18" s="6" t="n"/>
-      <c r="P18" s="6" t="n"/>
-      <c r="Q18" s="6" t="n"/>
-      <c r="R18" s="6" t="n"/>
-      <c r="S18" s="6" t="n"/>
-      <c r="T18" s="6" t="n"/>
-      <c r="U18" s="6" t="n"/>
-      <c r="V18" s="6" t="n"/>
-      <c r="W18" s="6" t="n"/>
-      <c r="X18" s="6" t="n"/>
-      <c r="Y18" s="6" t="n"/>
-      <c r="Z18" s="6" t="n"/>
-      <c r="AA18" s="6" t="n"/>
-      <c r="AB18" s="6" t="n"/>
-      <c r="AC18" s="6" t="n"/>
-      <c r="AD18" s="6" t="n"/>
-      <c r="AE18" s="6" t="n"/>
-      <c r="AF18" s="6" t="n"/>
-      <c r="AG18" s="6" t="n"/>
-      <c r="AH18" s="26" t="n"/>
-      <c r="AI18" s="23" t="n"/>
+      <c r="E18" s="168" t="n"/>
+      <c r="F18" s="168" t="n"/>
+      <c r="G18" s="169" t="n"/>
+      <c r="H18" s="168" t="n"/>
+      <c r="I18" s="168" t="n"/>
+      <c r="J18" s="168" t="n"/>
+      <c r="K18" s="168" t="n"/>
+      <c r="L18" s="168" t="n"/>
+      <c r="M18" s="168" t="n"/>
+      <c r="N18" s="168" t="n"/>
+      <c r="O18" s="168" t="n"/>
+      <c r="P18" s="168" t="n"/>
+      <c r="Q18" s="168" t="n"/>
+      <c r="R18" s="168" t="n"/>
+      <c r="S18" s="168" t="n"/>
+      <c r="T18" s="168" t="n"/>
+      <c r="U18" s="168" t="n"/>
+      <c r="V18" s="168" t="n"/>
+      <c r="W18" s="168" t="n"/>
+      <c r="X18" s="168" t="n"/>
+      <c r="Y18" s="168" t="n"/>
+      <c r="Z18" s="168" t="n"/>
+      <c r="AA18" s="168" t="n"/>
+      <c r="AB18" s="168" t="n"/>
+      <c r="AC18" s="168" t="n"/>
+      <c r="AD18" s="168" t="n"/>
+      <c r="AE18" s="168" t="n"/>
+      <c r="AF18" s="168" t="n"/>
+      <c r="AG18" s="168" t="n"/>
+      <c r="AH18" s="170" t="n"/>
+      <c r="AI18" s="171" t="n"/>
     </row>
     <row r="19" ht="16.2" customHeight="1" thickBot="1">
       <c r="A19" s="8" t="n">
@@ -3036,37 +3118,37 @@
           <t>FITTER</t>
         </is>
       </c>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="6" t="n"/>
-      <c r="I19" s="6" t="n"/>
-      <c r="J19" s="6" t="n"/>
-      <c r="K19" s="6" t="n"/>
-      <c r="L19" s="6" t="n"/>
-      <c r="M19" s="6" t="n"/>
-      <c r="N19" s="6" t="n"/>
-      <c r="O19" s="6" t="n"/>
-      <c r="P19" s="6" t="n"/>
-      <c r="Q19" s="6" t="n"/>
-      <c r="R19" s="6" t="n"/>
-      <c r="S19" s="6" t="n"/>
-      <c r="T19" s="6" t="n"/>
-      <c r="U19" s="6" t="n"/>
-      <c r="V19" s="6" t="n"/>
-      <c r="W19" s="6" t="n"/>
-      <c r="X19" s="6" t="n"/>
-      <c r="Y19" s="6" t="n"/>
-      <c r="Z19" s="6" t="n"/>
-      <c r="AA19" s="6" t="n"/>
-      <c r="AB19" s="6" t="n"/>
-      <c r="AC19" s="6" t="n"/>
-      <c r="AD19" s="6" t="n"/>
-      <c r="AE19" s="6" t="n"/>
-      <c r="AF19" s="6" t="n"/>
-      <c r="AG19" s="6" t="n"/>
-      <c r="AH19" s="26" t="n"/>
-      <c r="AI19" s="23" t="n"/>
+      <c r="E19" s="168" t="n"/>
+      <c r="F19" s="168" t="n"/>
+      <c r="G19" s="169" t="n"/>
+      <c r="H19" s="168" t="n"/>
+      <c r="I19" s="168" t="n"/>
+      <c r="J19" s="168" t="n"/>
+      <c r="K19" s="168" t="n"/>
+      <c r="L19" s="168" t="n"/>
+      <c r="M19" s="168" t="n"/>
+      <c r="N19" s="168" t="n"/>
+      <c r="O19" s="168" t="n"/>
+      <c r="P19" s="168" t="n"/>
+      <c r="Q19" s="168" t="n"/>
+      <c r="R19" s="168" t="n"/>
+      <c r="S19" s="168" t="n"/>
+      <c r="T19" s="168" t="n"/>
+      <c r="U19" s="168" t="n"/>
+      <c r="V19" s="168" t="n"/>
+      <c r="W19" s="168" t="n"/>
+      <c r="X19" s="168" t="n"/>
+      <c r="Y19" s="168" t="n"/>
+      <c r="Z19" s="168" t="n"/>
+      <c r="AA19" s="168" t="n"/>
+      <c r="AB19" s="168" t="n"/>
+      <c r="AC19" s="168" t="n"/>
+      <c r="AD19" s="168" t="n"/>
+      <c r="AE19" s="168" t="n"/>
+      <c r="AF19" s="168" t="n"/>
+      <c r="AG19" s="168" t="n"/>
+      <c r="AH19" s="170" t="n"/>
+      <c r="AI19" s="171" t="n"/>
     </row>
     <row r="20" ht="16.2" customHeight="1" thickBot="1">
       <c r="A20" s="8" t="n">
@@ -3085,53 +3167,73 @@
           <t>FITTER</t>
         </is>
       </c>
-      <c r="E20" s="27" t="n"/>
-      <c r="F20" s="27" t="n"/>
-      <c r="G20" s="28" t="n"/>
-      <c r="H20" s="27" t="n"/>
-      <c r="I20" s="27" t="n"/>
-      <c r="J20" s="27" t="n"/>
-      <c r="K20" s="27" t="n"/>
-      <c r="L20" s="27" t="n"/>
-      <c r="M20" s="27" t="n"/>
-      <c r="N20" s="27" t="n"/>
-      <c r="O20" s="27" t="n"/>
-      <c r="P20" s="27" t="n"/>
-      <c r="Q20" s="27" t="n"/>
-      <c r="R20" s="27" t="n"/>
-      <c r="S20" s="27" t="n"/>
-      <c r="T20" s="27" t="n"/>
-      <c r="U20" s="27" t="n"/>
-      <c r="V20" s="27" t="n"/>
-      <c r="W20" s="27" t="n"/>
-      <c r="X20" s="27" t="n"/>
-      <c r="Y20" s="27" t="n"/>
-      <c r="Z20" s="27" t="n"/>
-      <c r="AA20" s="27" t="n"/>
-      <c r="AB20" s="27" t="n"/>
-      <c r="AC20" s="27" t="n"/>
-      <c r="AD20" s="27" t="n"/>
-      <c r="AE20" s="27" t="n"/>
-      <c r="AF20" s="27" t="n"/>
-      <c r="AG20" s="27" t="n"/>
-      <c r="AH20" s="29" t="n"/>
-      <c r="AI20" s="23" t="n"/>
+      <c r="E20" s="173" t="n"/>
+      <c r="F20" s="173" t="n"/>
+      <c r="G20" s="174" t="n"/>
+      <c r="H20" s="173" t="n"/>
+      <c r="I20" s="173" t="n"/>
+      <c r="J20" s="173" t="n"/>
+      <c r="K20" s="173" t="n"/>
+      <c r="L20" s="173" t="n"/>
+      <c r="M20" s="173" t="n"/>
+      <c r="N20" s="173" t="n"/>
+      <c r="O20" s="173" t="n"/>
+      <c r="P20" s="173" t="n"/>
+      <c r="Q20" s="173" t="n"/>
+      <c r="R20" s="173" t="n"/>
+      <c r="S20" s="173" t="n"/>
+      <c r="T20" s="173" t="n"/>
+      <c r="U20" s="173" t="n"/>
+      <c r="V20" s="173" t="n"/>
+      <c r="W20" s="173" t="n"/>
+      <c r="X20" s="173" t="n"/>
+      <c r="Y20" s="173" t="n"/>
+      <c r="Z20" s="173" t="n"/>
+      <c r="AA20" s="173" t="n"/>
+      <c r="AB20" s="173" t="n"/>
+      <c r="AC20" s="173" t="n"/>
+      <c r="AD20" s="173" t="n"/>
+      <c r="AE20" s="173" t="n"/>
+      <c r="AF20" s="173" t="n"/>
+      <c r="AG20" s="173" t="n"/>
+      <c r="AH20" s="175" t="n"/>
+      <c r="AI20" s="171" t="n"/>
     </row>
     <row r="21" ht="16.2" customHeight="1" thickBot="1">
       <c r="A21" s="12" t="n"/>
       <c r="C21" s="13" t="n"/>
       <c r="D21" s="13" t="n"/>
-      <c r="E21" s="14" t="n"/>
-      <c r="F21" s="14" t="n"/>
-      <c r="G21" s="14" t="n"/>
-      <c r="H21" s="14" t="n"/>
-      <c r="I21" s="14" t="n"/>
-      <c r="J21" s="14" t="n"/>
-      <c r="K21" s="14" t="n"/>
-      <c r="L21" s="14" t="n"/>
-      <c r="M21" s="14" t="n"/>
-      <c r="N21" s="14" t="n"/>
-      <c r="O21" s="14" t="n"/>
+      <c r="E21" s="176" t="n"/>
+      <c r="F21" s="176" t="n"/>
+      <c r="G21" s="176" t="n"/>
+      <c r="H21" s="176" t="n"/>
+      <c r="I21" s="176" t="n"/>
+      <c r="J21" s="176" t="n"/>
+      <c r="K21" s="176" t="n"/>
+      <c r="L21" s="176" t="n"/>
+      <c r="M21" s="176" t="n"/>
+      <c r="N21" s="176" t="n"/>
+      <c r="O21" s="176" t="n"/>
+      <c r="P21" s="176" t="n"/>
+      <c r="Q21" s="176" t="n"/>
+      <c r="R21" s="176" t="n"/>
+      <c r="S21" s="176" t="n"/>
+      <c r="T21" s="176" t="n"/>
+      <c r="U21" s="176" t="n"/>
+      <c r="V21" s="176" t="n"/>
+      <c r="W21" s="176" t="n"/>
+      <c r="X21" s="176" t="n"/>
+      <c r="Y21" s="176" t="n"/>
+      <c r="Z21" s="176" t="n"/>
+      <c r="AA21" s="176" t="n"/>
+      <c r="AB21" s="176" t="n"/>
+      <c r="AC21" s="176" t="n"/>
+      <c r="AD21" s="176" t="n"/>
+      <c r="AE21" s="176" t="n"/>
+      <c r="AF21" s="176" t="n"/>
+      <c r="AG21" s="176" t="n"/>
+      <c r="AH21" s="176" t="n"/>
+      <c r="AI21" s="176" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" thickBot="1">
       <c r="A22" s="74" t="inlineStr">
@@ -3142,127 +3244,127 @@
       <c r="B22" s="123" t="n"/>
       <c r="C22" s="123" t="n"/>
       <c r="D22" s="123" t="n"/>
-      <c r="E22" s="30">
+      <c r="E22" s="177">
         <f>IF(1&lt;=$BA$4,TEXT($BA$3+0,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="F22" s="30">
+      <c r="F22" s="177">
         <f>IF(2&lt;=$BA$4,TEXT($BA$3+1,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="G22" s="30">
+      <c r="G22" s="177">
         <f>IF(3&lt;=$BA$4,TEXT($BA$3+2,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="H22" s="30">
+      <c r="H22" s="177">
         <f>IF(4&lt;=$BA$4,TEXT($BA$3+3,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="I22" s="30">
+      <c r="I22" s="177">
         <f>IF(5&lt;=$BA$4,TEXT($BA$3+4,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="J22" s="30">
+      <c r="J22" s="177">
         <f>IF(6&lt;=$BA$4,TEXT($BA$3+5,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="K22" s="30">
+      <c r="K22" s="177">
         <f>IF(7&lt;=$BA$4,TEXT($BA$3+6,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="L22" s="30">
+      <c r="L22" s="177">
         <f>IF(8&lt;=$BA$4,TEXT($BA$3+7,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="M22" s="30">
+      <c r="M22" s="177">
         <f>IF(9&lt;=$BA$4,TEXT($BA$3+8,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="N22" s="30">
+      <c r="N22" s="177">
         <f>IF(10&lt;=$BA$4,TEXT($BA$3+9,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="O22" s="30">
+      <c r="O22" s="177">
         <f>IF(11&lt;=$BA$4,TEXT($BA$3+10,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="P22" s="30">
+      <c r="P22" s="177">
         <f>IF(12&lt;=$BA$4,TEXT($BA$3+11,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Q22" s="30">
+      <c r="Q22" s="177">
         <f>IF(13&lt;=$BA$4,TEXT($BA$3+12,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="R22" s="30">
+      <c r="R22" s="177">
         <f>IF(14&lt;=$BA$4,TEXT($BA$3+13,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="S22" s="30">
+      <c r="S22" s="177">
         <f>IF(15&lt;=$BA$4,TEXT($BA$3+14,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="T22" s="30">
+      <c r="T22" s="177">
         <f>IF(16&lt;=$BA$4,TEXT($BA$3+15,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="U22" s="30">
+      <c r="U22" s="177">
         <f>IF(17&lt;=$BA$4,TEXT($BA$3+16,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="V22" s="30">
+      <c r="V22" s="177">
         <f>IF(18&lt;=$BA$4,TEXT($BA$3+17,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="W22" s="30">
+      <c r="W22" s="177">
         <f>IF(19&lt;=$BA$4,TEXT($BA$3+18,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="X22" s="30">
+      <c r="X22" s="177">
         <f>IF(20&lt;=$BA$4,TEXT($BA$3+19,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Y22" s="30">
+      <c r="Y22" s="177">
         <f>IF(21&lt;=$BA$4,TEXT($BA$3+20,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Z22" s="30">
+      <c r="Z22" s="177">
         <f>IF(22&lt;=$BA$4,TEXT($BA$3+21,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AA22" s="30">
+      <c r="AA22" s="177">
         <f>IF(23&lt;=$BA$4,TEXT($BA$3+22,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AB22" s="30">
+      <c r="AB22" s="177">
         <f>IF(24&lt;=$BA$4,TEXT($BA$3+23,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AC22" s="30">
+      <c r="AC22" s="177">
         <f>IF(25&lt;=$BA$4,TEXT($BA$3+24,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AD22" s="30">
+      <c r="AD22" s="177">
         <f>IF(26&lt;=$BA$4,TEXT($BA$3+25,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AE22" s="30">
+      <c r="AE22" s="177">
         <f>IF(27&lt;=$BA$4,TEXT($BA$3+26,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AF22" s="30">
+      <c r="AF22" s="177">
         <f>IF(28&lt;=$BA$4,TEXT($BA$3+27,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AG22" s="30">
+      <c r="AG22" s="177">
         <f>IF(29&lt;=$BA$4,TEXT($BA$3+28,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AH22" s="30">
+      <c r="AH22" s="177">
         <f>IF(30&lt;=$BA$4,TEXT($BA$3+29,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AI22" s="31">
+      <c r="AI22" s="178">
         <f>IF(31&lt;=$BA$4,TEXT($BA$3+30,"ddd"),"")</f>
         <v/>
       </c>
@@ -3414,37 +3516,37 @@
           <t>ACT/SUPV</t>
         </is>
       </c>
-      <c r="E24" s="6" t="n"/>
-      <c r="F24" s="6" t="n"/>
-      <c r="G24" s="6" t="n"/>
-      <c r="H24" s="6" t="n"/>
-      <c r="I24" s="6" t="n"/>
-      <c r="J24" s="6" t="n"/>
-      <c r="K24" s="6" t="n"/>
-      <c r="L24" s="6" t="n"/>
-      <c r="M24" s="6" t="n"/>
-      <c r="N24" s="6" t="n"/>
-      <c r="O24" s="6" t="n"/>
-      <c r="P24" s="6" t="n"/>
-      <c r="Q24" s="6" t="n"/>
-      <c r="R24" s="6" t="n"/>
-      <c r="S24" s="6" t="n"/>
-      <c r="T24" s="6" t="n"/>
-      <c r="U24" s="6" t="n"/>
-      <c r="V24" s="6" t="n"/>
-      <c r="W24" s="6" t="n"/>
-      <c r="X24" s="6" t="n"/>
-      <c r="Y24" s="6" t="n"/>
-      <c r="Z24" s="6" t="n"/>
-      <c r="AA24" s="6" t="n"/>
-      <c r="AB24" s="6" t="n"/>
-      <c r="AC24" s="6" t="n"/>
-      <c r="AD24" s="6" t="n"/>
-      <c r="AE24" s="6" t="n"/>
-      <c r="AF24" s="6" t="n"/>
-      <c r="AG24" s="6" t="n"/>
-      <c r="AH24" s="6" t="n"/>
-      <c r="AI24" s="26" t="n"/>
+      <c r="E24" s="168" t="n"/>
+      <c r="F24" s="168" t="n"/>
+      <c r="G24" s="168" t="n"/>
+      <c r="H24" s="168" t="n"/>
+      <c r="I24" s="168" t="n"/>
+      <c r="J24" s="168" t="n"/>
+      <c r="K24" s="168" t="n"/>
+      <c r="L24" s="168" t="n"/>
+      <c r="M24" s="168" t="n"/>
+      <c r="N24" s="168" t="n"/>
+      <c r="O24" s="168" t="n"/>
+      <c r="P24" s="168" t="n"/>
+      <c r="Q24" s="168" t="n"/>
+      <c r="R24" s="168" t="n"/>
+      <c r="S24" s="168" t="n"/>
+      <c r="T24" s="168" t="n"/>
+      <c r="U24" s="168" t="n"/>
+      <c r="V24" s="168" t="n"/>
+      <c r="W24" s="168" t="n"/>
+      <c r="X24" s="168" t="n"/>
+      <c r="Y24" s="168" t="n"/>
+      <c r="Z24" s="168" t="n"/>
+      <c r="AA24" s="168" t="n"/>
+      <c r="AB24" s="168" t="n"/>
+      <c r="AC24" s="168" t="n"/>
+      <c r="AD24" s="168" t="n"/>
+      <c r="AE24" s="168" t="n"/>
+      <c r="AF24" s="168" t="n"/>
+      <c r="AG24" s="168" t="n"/>
+      <c r="AH24" s="168" t="n"/>
+      <c r="AI24" s="170" t="n"/>
     </row>
     <row r="25" ht="16.2" customHeight="1" thickBot="1">
       <c r="A25" s="5" t="n">
@@ -3463,37 +3565,37 @@
           <t>ACT/SUPV</t>
         </is>
       </c>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n"/>
-      <c r="I25" s="6" t="n"/>
-      <c r="J25" s="6" t="n"/>
-      <c r="K25" s="6" t="n"/>
-      <c r="L25" s="6" t="n"/>
-      <c r="M25" s="6" t="n"/>
-      <c r="N25" s="6" t="n"/>
-      <c r="O25" s="6" t="n"/>
-      <c r="P25" s="6" t="n"/>
-      <c r="Q25" s="6" t="n"/>
-      <c r="R25" s="6" t="n"/>
-      <c r="S25" s="6" t="n"/>
-      <c r="T25" s="6" t="n"/>
-      <c r="U25" s="6" t="n"/>
-      <c r="V25" s="6" t="n"/>
-      <c r="W25" s="6" t="n"/>
-      <c r="X25" s="6" t="n"/>
-      <c r="Y25" s="6" t="n"/>
-      <c r="Z25" s="6" t="n"/>
-      <c r="AA25" s="6" t="n"/>
-      <c r="AB25" s="6" t="n"/>
-      <c r="AC25" s="6" t="n"/>
-      <c r="AD25" s="6" t="n"/>
-      <c r="AE25" s="6" t="n"/>
-      <c r="AF25" s="6" t="n"/>
-      <c r="AG25" s="6" t="n"/>
-      <c r="AH25" s="6" t="n"/>
-      <c r="AI25" s="26" t="n"/>
+      <c r="E25" s="168" t="n"/>
+      <c r="F25" s="168" t="n"/>
+      <c r="G25" s="168" t="n"/>
+      <c r="H25" s="168" t="n"/>
+      <c r="I25" s="168" t="n"/>
+      <c r="J25" s="168" t="n"/>
+      <c r="K25" s="168" t="n"/>
+      <c r="L25" s="168" t="n"/>
+      <c r="M25" s="168" t="n"/>
+      <c r="N25" s="168" t="n"/>
+      <c r="O25" s="168" t="n"/>
+      <c r="P25" s="168" t="n"/>
+      <c r="Q25" s="168" t="n"/>
+      <c r="R25" s="168" t="n"/>
+      <c r="S25" s="168" t="n"/>
+      <c r="T25" s="168" t="n"/>
+      <c r="U25" s="168" t="n"/>
+      <c r="V25" s="168" t="n"/>
+      <c r="W25" s="168" t="n"/>
+      <c r="X25" s="168" t="n"/>
+      <c r="Y25" s="168" t="n"/>
+      <c r="Z25" s="168" t="n"/>
+      <c r="AA25" s="168" t="n"/>
+      <c r="AB25" s="168" t="n"/>
+      <c r="AC25" s="168" t="n"/>
+      <c r="AD25" s="168" t="n"/>
+      <c r="AE25" s="168" t="n"/>
+      <c r="AF25" s="168" t="n"/>
+      <c r="AG25" s="168" t="n"/>
+      <c r="AH25" s="168" t="n"/>
+      <c r="AI25" s="170" t="n"/>
     </row>
     <row r="26" ht="16.2" customHeight="1" thickBot="1">
       <c r="A26" s="5" t="n">
@@ -3512,37 +3614,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
-      <c r="I26" s="6" t="n"/>
-      <c r="J26" s="6" t="n"/>
-      <c r="K26" s="6" t="n"/>
-      <c r="L26" s="6" t="n"/>
-      <c r="M26" s="6" t="n"/>
-      <c r="N26" s="6" t="n"/>
-      <c r="O26" s="6" t="n"/>
-      <c r="P26" s="6" t="n"/>
-      <c r="Q26" s="6" t="n"/>
-      <c r="R26" s="6" t="n"/>
-      <c r="S26" s="6" t="n"/>
-      <c r="T26" s="6" t="n"/>
-      <c r="U26" s="6" t="n"/>
-      <c r="V26" s="6" t="n"/>
-      <c r="W26" s="6" t="n"/>
-      <c r="X26" s="6" t="n"/>
-      <c r="Y26" s="6" t="n"/>
-      <c r="Z26" s="6" t="n"/>
-      <c r="AA26" s="6" t="n"/>
-      <c r="AB26" s="6" t="n"/>
-      <c r="AC26" s="6" t="n"/>
-      <c r="AD26" s="6" t="n"/>
-      <c r="AE26" s="6" t="n"/>
-      <c r="AF26" s="6" t="n"/>
-      <c r="AG26" s="6" t="n"/>
-      <c r="AH26" s="6" t="n"/>
-      <c r="AI26" s="26" t="n"/>
+      <c r="E26" s="168" t="n"/>
+      <c r="F26" s="168" t="n"/>
+      <c r="G26" s="168" t="n"/>
+      <c r="H26" s="168" t="n"/>
+      <c r="I26" s="168" t="n"/>
+      <c r="J26" s="168" t="n"/>
+      <c r="K26" s="168" t="n"/>
+      <c r="L26" s="168" t="n"/>
+      <c r="M26" s="168" t="n"/>
+      <c r="N26" s="168" t="n"/>
+      <c r="O26" s="168" t="n"/>
+      <c r="P26" s="168" t="n"/>
+      <c r="Q26" s="168" t="n"/>
+      <c r="R26" s="168" t="n"/>
+      <c r="S26" s="168" t="n"/>
+      <c r="T26" s="168" t="n"/>
+      <c r="U26" s="168" t="n"/>
+      <c r="V26" s="168" t="n"/>
+      <c r="W26" s="168" t="n"/>
+      <c r="X26" s="168" t="n"/>
+      <c r="Y26" s="168" t="n"/>
+      <c r="Z26" s="168" t="n"/>
+      <c r="AA26" s="168" t="n"/>
+      <c r="AB26" s="168" t="n"/>
+      <c r="AC26" s="168" t="n"/>
+      <c r="AD26" s="168" t="n"/>
+      <c r="AE26" s="168" t="n"/>
+      <c r="AF26" s="168" t="n"/>
+      <c r="AG26" s="168" t="n"/>
+      <c r="AH26" s="168" t="n"/>
+      <c r="AI26" s="170" t="n"/>
     </row>
     <row r="27" ht="16.2" customHeight="1" thickBot="1">
       <c r="A27" s="5" t="n">
@@ -3561,37 +3663,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="6" t="n"/>
-      <c r="G27" s="6" t="n"/>
-      <c r="H27" s="6" t="n"/>
-      <c r="I27" s="6" t="n"/>
-      <c r="J27" s="6" t="n"/>
-      <c r="K27" s="6" t="n"/>
-      <c r="L27" s="6" t="n"/>
-      <c r="M27" s="6" t="n"/>
-      <c r="N27" s="6" t="n"/>
-      <c r="O27" s="6" t="n"/>
-      <c r="P27" s="6" t="n"/>
-      <c r="Q27" s="6" t="n"/>
-      <c r="R27" s="6" t="n"/>
-      <c r="S27" s="6" t="n"/>
-      <c r="T27" s="6" t="n"/>
-      <c r="U27" s="6" t="n"/>
-      <c r="V27" s="6" t="n"/>
-      <c r="W27" s="6" t="n"/>
-      <c r="X27" s="6" t="n"/>
-      <c r="Y27" s="6" t="n"/>
-      <c r="Z27" s="6" t="n"/>
-      <c r="AA27" s="6" t="n"/>
-      <c r="AB27" s="6" t="n"/>
-      <c r="AC27" s="6" t="n"/>
-      <c r="AD27" s="6" t="n"/>
-      <c r="AE27" s="6" t="n"/>
-      <c r="AF27" s="6" t="n"/>
-      <c r="AG27" s="6" t="n"/>
-      <c r="AH27" s="6" t="n"/>
-      <c r="AI27" s="26" t="n"/>
+      <c r="E27" s="168" t="n"/>
+      <c r="F27" s="168" t="n"/>
+      <c r="G27" s="168" t="n"/>
+      <c r="H27" s="168" t="n"/>
+      <c r="I27" s="168" t="n"/>
+      <c r="J27" s="168" t="n"/>
+      <c r="K27" s="168" t="n"/>
+      <c r="L27" s="168" t="n"/>
+      <c r="M27" s="168" t="n"/>
+      <c r="N27" s="168" t="n"/>
+      <c r="O27" s="168" t="n"/>
+      <c r="P27" s="168" t="n"/>
+      <c r="Q27" s="168" t="n"/>
+      <c r="R27" s="168" t="n"/>
+      <c r="S27" s="168" t="n"/>
+      <c r="T27" s="168" t="n"/>
+      <c r="U27" s="168" t="n"/>
+      <c r="V27" s="168" t="n"/>
+      <c r="W27" s="168" t="n"/>
+      <c r="X27" s="168" t="n"/>
+      <c r="Y27" s="168" t="n"/>
+      <c r="Z27" s="168" t="n"/>
+      <c r="AA27" s="168" t="n"/>
+      <c r="AB27" s="168" t="n"/>
+      <c r="AC27" s="168" t="n"/>
+      <c r="AD27" s="168" t="n"/>
+      <c r="AE27" s="168" t="n"/>
+      <c r="AF27" s="168" t="n"/>
+      <c r="AG27" s="168" t="n"/>
+      <c r="AH27" s="168" t="n"/>
+      <c r="AI27" s="170" t="n"/>
     </row>
     <row r="28" ht="16.2" customHeight="1" thickBot="1">
       <c r="A28" s="5" t="n">
@@ -3610,37 +3712,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" s="6" t="n"/>
-      <c r="H28" s="6" t="n"/>
-      <c r="I28" s="6" t="n"/>
-      <c r="J28" s="6" t="n"/>
-      <c r="K28" s="6" t="n"/>
-      <c r="L28" s="6" t="n"/>
-      <c r="M28" s="6" t="n"/>
-      <c r="N28" s="6" t="n"/>
-      <c r="O28" s="6" t="n"/>
-      <c r="P28" s="6" t="n"/>
-      <c r="Q28" s="6" t="n"/>
-      <c r="R28" s="6" t="n"/>
-      <c r="S28" s="6" t="n"/>
-      <c r="T28" s="6" t="n"/>
-      <c r="U28" s="6" t="n"/>
-      <c r="V28" s="6" t="n"/>
-      <c r="W28" s="6" t="n"/>
-      <c r="X28" s="6" t="n"/>
-      <c r="Y28" s="6" t="n"/>
-      <c r="Z28" s="6" t="n"/>
-      <c r="AA28" s="6" t="n"/>
-      <c r="AB28" s="6" t="n"/>
-      <c r="AC28" s="6" t="n"/>
-      <c r="AD28" s="6" t="n"/>
-      <c r="AE28" s="6" t="n"/>
-      <c r="AF28" s="6" t="n"/>
-      <c r="AG28" s="6" t="n"/>
-      <c r="AH28" s="6" t="n"/>
-      <c r="AI28" s="26" t="n"/>
+      <c r="E28" s="168" t="n"/>
+      <c r="F28" s="168" t="n"/>
+      <c r="G28" s="168" t="n"/>
+      <c r="H28" s="168" t="n"/>
+      <c r="I28" s="168" t="n"/>
+      <c r="J28" s="168" t="n"/>
+      <c r="K28" s="168" t="n"/>
+      <c r="L28" s="168" t="n"/>
+      <c r="M28" s="168" t="n"/>
+      <c r="N28" s="168" t="n"/>
+      <c r="O28" s="168" t="n"/>
+      <c r="P28" s="168" t="n"/>
+      <c r="Q28" s="168" t="n"/>
+      <c r="R28" s="168" t="n"/>
+      <c r="S28" s="168" t="n"/>
+      <c r="T28" s="168" t="n"/>
+      <c r="U28" s="168" t="n"/>
+      <c r="V28" s="168" t="n"/>
+      <c r="W28" s="168" t="n"/>
+      <c r="X28" s="168" t="n"/>
+      <c r="Y28" s="168" t="n"/>
+      <c r="Z28" s="168" t="n"/>
+      <c r="AA28" s="168" t="n"/>
+      <c r="AB28" s="168" t="n"/>
+      <c r="AC28" s="168" t="n"/>
+      <c r="AD28" s="168" t="n"/>
+      <c r="AE28" s="168" t="n"/>
+      <c r="AF28" s="168" t="n"/>
+      <c r="AG28" s="168" t="n"/>
+      <c r="AH28" s="168" t="n"/>
+      <c r="AI28" s="170" t="n"/>
     </row>
     <row r="29" ht="16.2" customHeight="1" thickBot="1">
       <c r="A29" s="10" t="n">
@@ -3659,37 +3761,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="6" t="n"/>
-      <c r="I29" s="6" t="n"/>
-      <c r="J29" s="6" t="n"/>
-      <c r="K29" s="6" t="n"/>
-      <c r="L29" s="6" t="n"/>
-      <c r="M29" s="6" t="n"/>
-      <c r="N29" s="6" t="n"/>
-      <c r="O29" s="6" t="n"/>
-      <c r="P29" s="6" t="n"/>
-      <c r="Q29" s="6" t="n"/>
-      <c r="R29" s="6" t="n"/>
-      <c r="S29" s="6" t="n"/>
-      <c r="T29" s="6" t="n"/>
-      <c r="U29" s="6" t="n"/>
-      <c r="V29" s="6" t="n"/>
-      <c r="W29" s="6" t="n"/>
-      <c r="X29" s="6" t="n"/>
-      <c r="Y29" s="6" t="n"/>
-      <c r="Z29" s="6" t="n"/>
-      <c r="AA29" s="6" t="n"/>
-      <c r="AB29" s="6" t="n"/>
-      <c r="AC29" s="6" t="n"/>
-      <c r="AD29" s="6" t="n"/>
-      <c r="AE29" s="6" t="n"/>
-      <c r="AF29" s="6" t="n"/>
-      <c r="AG29" s="6" t="n"/>
-      <c r="AH29" s="6" t="n"/>
-      <c r="AI29" s="26" t="n"/>
+      <c r="E29" s="168" t="n"/>
+      <c r="F29" s="168" t="n"/>
+      <c r="G29" s="168" t="n"/>
+      <c r="H29" s="168" t="n"/>
+      <c r="I29" s="168" t="n"/>
+      <c r="J29" s="168" t="n"/>
+      <c r="K29" s="168" t="n"/>
+      <c r="L29" s="168" t="n"/>
+      <c r="M29" s="168" t="n"/>
+      <c r="N29" s="168" t="n"/>
+      <c r="O29" s="168" t="n"/>
+      <c r="P29" s="168" t="n"/>
+      <c r="Q29" s="168" t="n"/>
+      <c r="R29" s="168" t="n"/>
+      <c r="S29" s="168" t="n"/>
+      <c r="T29" s="168" t="n"/>
+      <c r="U29" s="168" t="n"/>
+      <c r="V29" s="168" t="n"/>
+      <c r="W29" s="168" t="n"/>
+      <c r="X29" s="168" t="n"/>
+      <c r="Y29" s="168" t="n"/>
+      <c r="Z29" s="168" t="n"/>
+      <c r="AA29" s="168" t="n"/>
+      <c r="AB29" s="168" t="n"/>
+      <c r="AC29" s="168" t="n"/>
+      <c r="AD29" s="168" t="n"/>
+      <c r="AE29" s="168" t="n"/>
+      <c r="AF29" s="168" t="n"/>
+      <c r="AG29" s="168" t="n"/>
+      <c r="AH29" s="168" t="n"/>
+      <c r="AI29" s="170" t="n"/>
     </row>
     <row r="30" ht="16.2" customHeight="1" thickBot="1">
       <c r="A30" s="10" t="n">
@@ -3708,37 +3810,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="n"/>
-      <c r="H30" s="6" t="n"/>
-      <c r="I30" s="6" t="n"/>
-      <c r="J30" s="6" t="n"/>
-      <c r="K30" s="6" t="n"/>
-      <c r="L30" s="6" t="n"/>
-      <c r="M30" s="6" t="n"/>
-      <c r="N30" s="6" t="n"/>
-      <c r="O30" s="6" t="n"/>
-      <c r="P30" s="6" t="n"/>
-      <c r="Q30" s="6" t="n"/>
-      <c r="R30" s="6" t="n"/>
-      <c r="S30" s="6" t="n"/>
-      <c r="T30" s="6" t="n"/>
-      <c r="U30" s="6" t="n"/>
-      <c r="V30" s="6" t="n"/>
-      <c r="W30" s="6" t="n"/>
-      <c r="X30" s="6" t="n"/>
-      <c r="Y30" s="6" t="n"/>
-      <c r="Z30" s="6" t="n"/>
-      <c r="AA30" s="6" t="n"/>
-      <c r="AB30" s="6" t="n"/>
-      <c r="AC30" s="6" t="n"/>
-      <c r="AD30" s="6" t="n"/>
-      <c r="AE30" s="6" t="n"/>
-      <c r="AF30" s="6" t="n"/>
-      <c r="AG30" s="6" t="n"/>
-      <c r="AH30" s="6" t="n"/>
-      <c r="AI30" s="26" t="n"/>
+      <c r="E30" s="168" t="n"/>
+      <c r="F30" s="168" t="n"/>
+      <c r="G30" s="168" t="n"/>
+      <c r="H30" s="168" t="n"/>
+      <c r="I30" s="168" t="n"/>
+      <c r="J30" s="168" t="n"/>
+      <c r="K30" s="168" t="n"/>
+      <c r="L30" s="168" t="n"/>
+      <c r="M30" s="168" t="n"/>
+      <c r="N30" s="168" t="n"/>
+      <c r="O30" s="168" t="n"/>
+      <c r="P30" s="168" t="n"/>
+      <c r="Q30" s="168" t="n"/>
+      <c r="R30" s="168" t="n"/>
+      <c r="S30" s="168" t="n"/>
+      <c r="T30" s="168" t="n"/>
+      <c r="U30" s="168" t="n"/>
+      <c r="V30" s="168" t="n"/>
+      <c r="W30" s="168" t="n"/>
+      <c r="X30" s="168" t="n"/>
+      <c r="Y30" s="168" t="n"/>
+      <c r="Z30" s="168" t="n"/>
+      <c r="AA30" s="168" t="n"/>
+      <c r="AB30" s="168" t="n"/>
+      <c r="AC30" s="168" t="n"/>
+      <c r="AD30" s="168" t="n"/>
+      <c r="AE30" s="168" t="n"/>
+      <c r="AF30" s="168" t="n"/>
+      <c r="AG30" s="168" t="n"/>
+      <c r="AH30" s="168" t="n"/>
+      <c r="AI30" s="170" t="n"/>
     </row>
     <row r="31" ht="16.2" customHeight="1" thickBot="1">
       <c r="A31" s="10" t="n">
@@ -3757,37 +3859,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="6" t="n"/>
-      <c r="H31" s="6" t="n"/>
-      <c r="I31" s="6" t="n"/>
-      <c r="J31" s="6" t="n"/>
-      <c r="K31" s="6" t="n"/>
-      <c r="L31" s="6" t="n"/>
-      <c r="M31" s="6" t="n"/>
-      <c r="N31" s="6" t="n"/>
-      <c r="O31" s="6" t="n"/>
-      <c r="P31" s="6" t="n"/>
-      <c r="Q31" s="6" t="n"/>
-      <c r="R31" s="6" t="n"/>
-      <c r="S31" s="6" t="n"/>
-      <c r="T31" s="6" t="n"/>
-      <c r="U31" s="6" t="n"/>
-      <c r="V31" s="6" t="n"/>
-      <c r="W31" s="6" t="n"/>
-      <c r="X31" s="6" t="n"/>
-      <c r="Y31" s="6" t="n"/>
-      <c r="Z31" s="6" t="n"/>
-      <c r="AA31" s="6" t="n"/>
-      <c r="AB31" s="6" t="n"/>
-      <c r="AC31" s="6" t="n"/>
-      <c r="AD31" s="6" t="n"/>
-      <c r="AE31" s="6" t="n"/>
-      <c r="AF31" s="6" t="n"/>
-      <c r="AG31" s="6" t="n"/>
-      <c r="AH31" s="6" t="n"/>
-      <c r="AI31" s="26" t="n"/>
+      <c r="E31" s="168" t="n"/>
+      <c r="F31" s="168" t="n"/>
+      <c r="G31" s="168" t="n"/>
+      <c r="H31" s="168" t="n"/>
+      <c r="I31" s="168" t="n"/>
+      <c r="J31" s="168" t="n"/>
+      <c r="K31" s="168" t="n"/>
+      <c r="L31" s="168" t="n"/>
+      <c r="M31" s="168" t="n"/>
+      <c r="N31" s="168" t="n"/>
+      <c r="O31" s="168" t="n"/>
+      <c r="P31" s="168" t="n"/>
+      <c r="Q31" s="168" t="n"/>
+      <c r="R31" s="168" t="n"/>
+      <c r="S31" s="168" t="n"/>
+      <c r="T31" s="168" t="n"/>
+      <c r="U31" s="168" t="n"/>
+      <c r="V31" s="168" t="n"/>
+      <c r="W31" s="168" t="n"/>
+      <c r="X31" s="168" t="n"/>
+      <c r="Y31" s="168" t="n"/>
+      <c r="Z31" s="168" t="n"/>
+      <c r="AA31" s="168" t="n"/>
+      <c r="AB31" s="168" t="n"/>
+      <c r="AC31" s="168" t="n"/>
+      <c r="AD31" s="168" t="n"/>
+      <c r="AE31" s="168" t="n"/>
+      <c r="AF31" s="168" t="n"/>
+      <c r="AG31" s="168" t="n"/>
+      <c r="AH31" s="168" t="n"/>
+      <c r="AI31" s="170" t="n"/>
     </row>
     <row r="32" ht="16.2" customHeight="1" thickBot="1">
       <c r="A32" s="10" t="n">
@@ -3806,37 +3908,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="n"/>
-      <c r="H32" s="6" t="n"/>
-      <c r="I32" s="6" t="n"/>
-      <c r="J32" s="6" t="n"/>
-      <c r="K32" s="6" t="n"/>
-      <c r="L32" s="6" t="n"/>
-      <c r="M32" s="6" t="n"/>
-      <c r="N32" s="6" t="n"/>
-      <c r="O32" s="6" t="n"/>
-      <c r="P32" s="6" t="n"/>
-      <c r="Q32" s="6" t="n"/>
-      <c r="R32" s="6" t="n"/>
-      <c r="S32" s="6" t="n"/>
-      <c r="T32" s="6" t="n"/>
-      <c r="U32" s="6" t="n"/>
-      <c r="V32" s="6" t="n"/>
-      <c r="W32" s="6" t="n"/>
-      <c r="X32" s="6" t="n"/>
-      <c r="Y32" s="6" t="n"/>
-      <c r="Z32" s="6" t="n"/>
-      <c r="AA32" s="6" t="n"/>
-      <c r="AB32" s="6" t="n"/>
-      <c r="AC32" s="6" t="n"/>
-      <c r="AD32" s="6" t="n"/>
-      <c r="AE32" s="6" t="n"/>
-      <c r="AF32" s="6" t="n"/>
-      <c r="AG32" s="6" t="n"/>
-      <c r="AH32" s="6" t="n"/>
-      <c r="AI32" s="26" t="n"/>
+      <c r="E32" s="168" t="n"/>
+      <c r="F32" s="168" t="n"/>
+      <c r="G32" s="168" t="n"/>
+      <c r="H32" s="168" t="n"/>
+      <c r="I32" s="168" t="n"/>
+      <c r="J32" s="168" t="n"/>
+      <c r="K32" s="168" t="n"/>
+      <c r="L32" s="168" t="n"/>
+      <c r="M32" s="168" t="n"/>
+      <c r="N32" s="168" t="n"/>
+      <c r="O32" s="168" t="n"/>
+      <c r="P32" s="168" t="n"/>
+      <c r="Q32" s="168" t="n"/>
+      <c r="R32" s="168" t="n"/>
+      <c r="S32" s="168" t="n"/>
+      <c r="T32" s="168" t="n"/>
+      <c r="U32" s="168" t="n"/>
+      <c r="V32" s="168" t="n"/>
+      <c r="W32" s="168" t="n"/>
+      <c r="X32" s="168" t="n"/>
+      <c r="Y32" s="168" t="n"/>
+      <c r="Z32" s="168" t="n"/>
+      <c r="AA32" s="168" t="n"/>
+      <c r="AB32" s="168" t="n"/>
+      <c r="AC32" s="168" t="n"/>
+      <c r="AD32" s="168" t="n"/>
+      <c r="AE32" s="168" t="n"/>
+      <c r="AF32" s="168" t="n"/>
+      <c r="AG32" s="168" t="n"/>
+      <c r="AH32" s="168" t="n"/>
+      <c r="AI32" s="170" t="n"/>
     </row>
     <row r="33" ht="16.2" customHeight="1" thickBot="1">
       <c r="A33" s="10" t="n">
@@ -3855,37 +3957,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="6" t="n"/>
-      <c r="G33" s="6" t="n"/>
-      <c r="H33" s="6" t="n"/>
-      <c r="I33" s="6" t="n"/>
-      <c r="J33" s="6" t="n"/>
-      <c r="K33" s="6" t="n"/>
-      <c r="L33" s="6" t="n"/>
-      <c r="M33" s="6" t="n"/>
-      <c r="N33" s="6" t="n"/>
-      <c r="O33" s="6" t="n"/>
-      <c r="P33" s="6" t="n"/>
-      <c r="Q33" s="6" t="n"/>
-      <c r="R33" s="6" t="n"/>
-      <c r="S33" s="6" t="n"/>
-      <c r="T33" s="6" t="n"/>
-      <c r="U33" s="6" t="n"/>
-      <c r="V33" s="6" t="n"/>
-      <c r="W33" s="6" t="n"/>
-      <c r="X33" s="6" t="n"/>
-      <c r="Y33" s="6" t="n"/>
-      <c r="Z33" s="6" t="n"/>
-      <c r="AA33" s="6" t="n"/>
-      <c r="AB33" s="6" t="n"/>
-      <c r="AC33" s="6" t="n"/>
-      <c r="AD33" s="6" t="n"/>
-      <c r="AE33" s="6" t="n"/>
-      <c r="AF33" s="6" t="n"/>
-      <c r="AG33" s="6" t="n"/>
-      <c r="AH33" s="6" t="n"/>
-      <c r="AI33" s="26" t="n"/>
+      <c r="E33" s="168" t="n"/>
+      <c r="F33" s="168" t="n"/>
+      <c r="G33" s="168" t="n"/>
+      <c r="H33" s="168" t="n"/>
+      <c r="I33" s="168" t="n"/>
+      <c r="J33" s="168" t="n"/>
+      <c r="K33" s="168" t="n"/>
+      <c r="L33" s="168" t="n"/>
+      <c r="M33" s="168" t="n"/>
+      <c r="N33" s="168" t="n"/>
+      <c r="O33" s="168" t="n"/>
+      <c r="P33" s="168" t="n"/>
+      <c r="Q33" s="168" t="n"/>
+      <c r="R33" s="168" t="n"/>
+      <c r="S33" s="168" t="n"/>
+      <c r="T33" s="168" t="n"/>
+      <c r="U33" s="168" t="n"/>
+      <c r="V33" s="168" t="n"/>
+      <c r="W33" s="168" t="n"/>
+      <c r="X33" s="168" t="n"/>
+      <c r="Y33" s="168" t="n"/>
+      <c r="Z33" s="168" t="n"/>
+      <c r="AA33" s="168" t="n"/>
+      <c r="AB33" s="168" t="n"/>
+      <c r="AC33" s="168" t="n"/>
+      <c r="AD33" s="168" t="n"/>
+      <c r="AE33" s="168" t="n"/>
+      <c r="AF33" s="168" t="n"/>
+      <c r="AG33" s="168" t="n"/>
+      <c r="AH33" s="168" t="n"/>
+      <c r="AI33" s="170" t="n"/>
     </row>
     <row r="34" ht="16.2" customHeight="1" thickBot="1">
       <c r="A34" s="10" t="n">
@@ -3904,37 +4006,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E34" s="6" t="n"/>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="6" t="n"/>
-      <c r="H34" s="6" t="n"/>
-      <c r="I34" s="6" t="n"/>
-      <c r="J34" s="6" t="n"/>
-      <c r="K34" s="6" t="n"/>
-      <c r="L34" s="6" t="n"/>
-      <c r="M34" s="6" t="n"/>
-      <c r="N34" s="6" t="n"/>
-      <c r="O34" s="6" t="n"/>
-      <c r="P34" s="6" t="n"/>
-      <c r="Q34" s="6" t="n"/>
-      <c r="R34" s="6" t="n"/>
-      <c r="S34" s="6" t="n"/>
-      <c r="T34" s="6" t="n"/>
-      <c r="U34" s="6" t="n"/>
-      <c r="V34" s="6" t="n"/>
-      <c r="W34" s="6" t="n"/>
-      <c r="X34" s="6" t="n"/>
-      <c r="Y34" s="6" t="n"/>
-      <c r="Z34" s="6" t="n"/>
-      <c r="AA34" s="6" t="n"/>
-      <c r="AB34" s="6" t="n"/>
-      <c r="AC34" s="6" t="n"/>
-      <c r="AD34" s="6" t="n"/>
-      <c r="AE34" s="6" t="n"/>
-      <c r="AF34" s="6" t="n"/>
-      <c r="AG34" s="6" t="n"/>
-      <c r="AH34" s="6" t="n"/>
-      <c r="AI34" s="26" t="n"/>
+      <c r="E34" s="168" t="n"/>
+      <c r="F34" s="168" t="n"/>
+      <c r="G34" s="168" t="n"/>
+      <c r="H34" s="168" t="n"/>
+      <c r="I34" s="168" t="n"/>
+      <c r="J34" s="168" t="n"/>
+      <c r="K34" s="168" t="n"/>
+      <c r="L34" s="168" t="n"/>
+      <c r="M34" s="168" t="n"/>
+      <c r="N34" s="168" t="n"/>
+      <c r="O34" s="168" t="n"/>
+      <c r="P34" s="168" t="n"/>
+      <c r="Q34" s="168" t="n"/>
+      <c r="R34" s="168" t="n"/>
+      <c r="S34" s="168" t="n"/>
+      <c r="T34" s="168" t="n"/>
+      <c r="U34" s="168" t="n"/>
+      <c r="V34" s="168" t="n"/>
+      <c r="W34" s="168" t="n"/>
+      <c r="X34" s="168" t="n"/>
+      <c r="Y34" s="168" t="n"/>
+      <c r="Z34" s="168" t="n"/>
+      <c r="AA34" s="168" t="n"/>
+      <c r="AB34" s="168" t="n"/>
+      <c r="AC34" s="168" t="n"/>
+      <c r="AD34" s="168" t="n"/>
+      <c r="AE34" s="168" t="n"/>
+      <c r="AF34" s="168" t="n"/>
+      <c r="AG34" s="168" t="n"/>
+      <c r="AH34" s="168" t="n"/>
+      <c r="AI34" s="170" t="n"/>
     </row>
     <row r="35" ht="16.2" customHeight="1" thickBot="1">
       <c r="A35" s="10" t="n">
@@ -3953,37 +4055,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="6" t="n"/>
-      <c r="G35" s="6" t="n"/>
-      <c r="H35" s="6" t="n"/>
-      <c r="I35" s="6" t="n"/>
-      <c r="J35" s="6" t="n"/>
-      <c r="K35" s="6" t="n"/>
-      <c r="L35" s="6" t="n"/>
-      <c r="M35" s="6" t="n"/>
-      <c r="N35" s="6" t="n"/>
-      <c r="O35" s="6" t="n"/>
-      <c r="P35" s="6" t="n"/>
-      <c r="Q35" s="6" t="n"/>
-      <c r="R35" s="6" t="n"/>
-      <c r="S35" s="6" t="n"/>
-      <c r="T35" s="6" t="n"/>
-      <c r="U35" s="6" t="n"/>
-      <c r="V35" s="6" t="n"/>
-      <c r="W35" s="6" t="n"/>
-      <c r="X35" s="6" t="n"/>
-      <c r="Y35" s="6" t="n"/>
-      <c r="Z35" s="6" t="n"/>
-      <c r="AA35" s="6" t="n"/>
-      <c r="AB35" s="6" t="n"/>
-      <c r="AC35" s="6" t="n"/>
-      <c r="AD35" s="6" t="n"/>
-      <c r="AE35" s="6" t="n"/>
-      <c r="AF35" s="6" t="n"/>
-      <c r="AG35" s="6" t="n"/>
-      <c r="AH35" s="6" t="n"/>
-      <c r="AI35" s="26" t="n"/>
+      <c r="E35" s="168" t="n"/>
+      <c r="F35" s="168" t="n"/>
+      <c r="G35" s="168" t="n"/>
+      <c r="H35" s="168" t="n"/>
+      <c r="I35" s="168" t="n"/>
+      <c r="J35" s="168" t="n"/>
+      <c r="K35" s="168" t="n"/>
+      <c r="L35" s="168" t="n"/>
+      <c r="M35" s="168" t="n"/>
+      <c r="N35" s="168" t="n"/>
+      <c r="O35" s="168" t="n"/>
+      <c r="P35" s="168" t="n"/>
+      <c r="Q35" s="168" t="n"/>
+      <c r="R35" s="168" t="n"/>
+      <c r="S35" s="168" t="n"/>
+      <c r="T35" s="168" t="n"/>
+      <c r="U35" s="168" t="n"/>
+      <c r="V35" s="168" t="n"/>
+      <c r="W35" s="168" t="n"/>
+      <c r="X35" s="168" t="n"/>
+      <c r="Y35" s="168" t="n"/>
+      <c r="Z35" s="168" t="n"/>
+      <c r="AA35" s="168" t="n"/>
+      <c r="AB35" s="168" t="n"/>
+      <c r="AC35" s="168" t="n"/>
+      <c r="AD35" s="168" t="n"/>
+      <c r="AE35" s="168" t="n"/>
+      <c r="AF35" s="168" t="n"/>
+      <c r="AG35" s="168" t="n"/>
+      <c r="AH35" s="168" t="n"/>
+      <c r="AI35" s="170" t="n"/>
     </row>
     <row r="36" ht="16.2" customHeight="1" thickBot="1">
       <c r="A36" s="10" t="n">
@@ -4002,37 +4104,37 @@
           <t>OJT</t>
         </is>
       </c>
-      <c r="E36" s="6" t="n"/>
-      <c r="F36" s="6" t="n"/>
-      <c r="G36" s="6" t="n"/>
-      <c r="H36" s="6" t="n"/>
-      <c r="I36" s="6" t="n"/>
-      <c r="J36" s="6" t="n"/>
-      <c r="K36" s="6" t="n"/>
-      <c r="L36" s="6" t="n"/>
-      <c r="M36" s="6" t="n"/>
-      <c r="N36" s="6" t="n"/>
-      <c r="O36" s="6" t="n"/>
-      <c r="P36" s="6" t="n"/>
-      <c r="Q36" s="6" t="n"/>
-      <c r="R36" s="6" t="n"/>
-      <c r="S36" s="6" t="n"/>
-      <c r="T36" s="6" t="n"/>
-      <c r="U36" s="6" t="n"/>
-      <c r="V36" s="6" t="n"/>
-      <c r="W36" s="6" t="n"/>
-      <c r="X36" s="6" t="n"/>
-      <c r="Y36" s="6" t="n"/>
-      <c r="Z36" s="6" t="n"/>
-      <c r="AA36" s="6" t="n"/>
-      <c r="AB36" s="6" t="n"/>
-      <c r="AC36" s="6" t="n"/>
-      <c r="AD36" s="6" t="n"/>
-      <c r="AE36" s="6" t="n"/>
-      <c r="AF36" s="6" t="n"/>
-      <c r="AG36" s="6" t="n"/>
-      <c r="AH36" s="6" t="n"/>
-      <c r="AI36" s="26" t="n"/>
+      <c r="E36" s="168" t="n"/>
+      <c r="F36" s="168" t="n"/>
+      <c r="G36" s="168" t="n"/>
+      <c r="H36" s="168" t="n"/>
+      <c r="I36" s="168" t="n"/>
+      <c r="J36" s="168" t="n"/>
+      <c r="K36" s="168" t="n"/>
+      <c r="L36" s="168" t="n"/>
+      <c r="M36" s="168" t="n"/>
+      <c r="N36" s="168" t="n"/>
+      <c r="O36" s="168" t="n"/>
+      <c r="P36" s="168" t="n"/>
+      <c r="Q36" s="168" t="n"/>
+      <c r="R36" s="168" t="n"/>
+      <c r="S36" s="168" t="n"/>
+      <c r="T36" s="168" t="n"/>
+      <c r="U36" s="168" t="n"/>
+      <c r="V36" s="168" t="n"/>
+      <c r="W36" s="168" t="n"/>
+      <c r="X36" s="168" t="n"/>
+      <c r="Y36" s="168" t="n"/>
+      <c r="Z36" s="168" t="n"/>
+      <c r="AA36" s="168" t="n"/>
+      <c r="AB36" s="168" t="n"/>
+      <c r="AC36" s="168" t="n"/>
+      <c r="AD36" s="168" t="n"/>
+      <c r="AE36" s="168" t="n"/>
+      <c r="AF36" s="168" t="n"/>
+      <c r="AG36" s="168" t="n"/>
+      <c r="AH36" s="168" t="n"/>
+      <c r="AI36" s="170" t="n"/>
     </row>
     <row r="37" ht="16.2" customHeight="1" thickBot="1">
       <c r="A37" s="8" t="n">
@@ -4051,37 +4153,37 @@
           <t>FITTER</t>
         </is>
       </c>
-      <c r="E37" s="6" t="n"/>
-      <c r="F37" s="6" t="n"/>
-      <c r="G37" s="6" t="n"/>
-      <c r="H37" s="6" t="n"/>
-      <c r="I37" s="6" t="n"/>
-      <c r="J37" s="6" t="n"/>
-      <c r="K37" s="6" t="n"/>
-      <c r="L37" s="6" t="n"/>
-      <c r="M37" s="6" t="n"/>
-      <c r="N37" s="6" t="n"/>
-      <c r="O37" s="6" t="n"/>
-      <c r="P37" s="6" t="n"/>
-      <c r="Q37" s="6" t="n"/>
-      <c r="R37" s="6" t="n"/>
-      <c r="S37" s="6" t="n"/>
-      <c r="T37" s="6" t="n"/>
-      <c r="U37" s="6" t="n"/>
-      <c r="V37" s="6" t="n"/>
-      <c r="W37" s="6" t="n"/>
-      <c r="X37" s="6" t="n"/>
-      <c r="Y37" s="6" t="n"/>
-      <c r="Z37" s="6" t="n"/>
-      <c r="AA37" s="6" t="n"/>
-      <c r="AB37" s="6" t="n"/>
-      <c r="AC37" s="6" t="n"/>
-      <c r="AD37" s="6" t="n"/>
-      <c r="AE37" s="6" t="n"/>
-      <c r="AF37" s="6" t="n"/>
-      <c r="AG37" s="6" t="n"/>
-      <c r="AH37" s="6" t="n"/>
-      <c r="AI37" s="26" t="n"/>
+      <c r="E37" s="168" t="n"/>
+      <c r="F37" s="168" t="n"/>
+      <c r="G37" s="168" t="n"/>
+      <c r="H37" s="168" t="n"/>
+      <c r="I37" s="168" t="n"/>
+      <c r="J37" s="168" t="n"/>
+      <c r="K37" s="168" t="n"/>
+      <c r="L37" s="168" t="n"/>
+      <c r="M37" s="168" t="n"/>
+      <c r="N37" s="168" t="n"/>
+      <c r="O37" s="168" t="n"/>
+      <c r="P37" s="168" t="n"/>
+      <c r="Q37" s="168" t="n"/>
+      <c r="R37" s="168" t="n"/>
+      <c r="S37" s="168" t="n"/>
+      <c r="T37" s="168" t="n"/>
+      <c r="U37" s="168" t="n"/>
+      <c r="V37" s="168" t="n"/>
+      <c r="W37" s="168" t="n"/>
+      <c r="X37" s="168" t="n"/>
+      <c r="Y37" s="168" t="n"/>
+      <c r="Z37" s="168" t="n"/>
+      <c r="AA37" s="168" t="n"/>
+      <c r="AB37" s="168" t="n"/>
+      <c r="AC37" s="168" t="n"/>
+      <c r="AD37" s="168" t="n"/>
+      <c r="AE37" s="168" t="n"/>
+      <c r="AF37" s="168" t="n"/>
+      <c r="AG37" s="168" t="n"/>
+      <c r="AH37" s="168" t="n"/>
+      <c r="AI37" s="170" t="n"/>
     </row>
     <row r="38" ht="16.2" customHeight="1" thickBot="1">
       <c r="A38" s="8" t="n">
@@ -4100,37 +4202,37 @@
           <t>FITTER</t>
         </is>
       </c>
-      <c r="E38" s="6" t="n"/>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" s="6" t="n"/>
-      <c r="H38" s="6" t="n"/>
-      <c r="I38" s="6" t="n"/>
-      <c r="J38" s="6" t="n"/>
-      <c r="K38" s="6" t="n"/>
-      <c r="L38" s="6" t="n"/>
-      <c r="M38" s="6" t="n"/>
-      <c r="N38" s="6" t="n"/>
-      <c r="O38" s="6" t="n"/>
-      <c r="P38" s="6" t="n"/>
-      <c r="Q38" s="6" t="n"/>
-      <c r="R38" s="6" t="n"/>
-      <c r="S38" s="6" t="n"/>
-      <c r="T38" s="6" t="n"/>
-      <c r="U38" s="6" t="n"/>
-      <c r="V38" s="6" t="n"/>
-      <c r="W38" s="6" t="n"/>
-      <c r="X38" s="6" t="n"/>
-      <c r="Y38" s="6" t="n"/>
-      <c r="Z38" s="6" t="n"/>
-      <c r="AA38" s="6" t="n"/>
-      <c r="AB38" s="6" t="n"/>
-      <c r="AC38" s="6" t="n"/>
-      <c r="AD38" s="6" t="n"/>
-      <c r="AE38" s="6" t="n"/>
-      <c r="AF38" s="6" t="n"/>
-      <c r="AG38" s="6" t="n"/>
-      <c r="AH38" s="6" t="n"/>
-      <c r="AI38" s="26" t="n"/>
+      <c r="E38" s="168" t="n"/>
+      <c r="F38" s="168" t="n"/>
+      <c r="G38" s="168" t="n"/>
+      <c r="H38" s="168" t="n"/>
+      <c r="I38" s="168" t="n"/>
+      <c r="J38" s="168" t="n"/>
+      <c r="K38" s="168" t="n"/>
+      <c r="L38" s="168" t="n"/>
+      <c r="M38" s="168" t="n"/>
+      <c r="N38" s="168" t="n"/>
+      <c r="O38" s="168" t="n"/>
+      <c r="P38" s="168" t="n"/>
+      <c r="Q38" s="168" t="n"/>
+      <c r="R38" s="168" t="n"/>
+      <c r="S38" s="168" t="n"/>
+      <c r="T38" s="168" t="n"/>
+      <c r="U38" s="168" t="n"/>
+      <c r="V38" s="168" t="n"/>
+      <c r="W38" s="168" t="n"/>
+      <c r="X38" s="168" t="n"/>
+      <c r="Y38" s="168" t="n"/>
+      <c r="Z38" s="168" t="n"/>
+      <c r="AA38" s="168" t="n"/>
+      <c r="AB38" s="168" t="n"/>
+      <c r="AC38" s="168" t="n"/>
+      <c r="AD38" s="168" t="n"/>
+      <c r="AE38" s="168" t="n"/>
+      <c r="AF38" s="168" t="n"/>
+      <c r="AG38" s="168" t="n"/>
+      <c r="AH38" s="168" t="n"/>
+      <c r="AI38" s="170" t="n"/>
     </row>
     <row r="39" ht="16.2" customHeight="1" thickBot="1">
       <c r="A39" s="8" t="n">
@@ -4149,37 +4251,37 @@
           <t>FITTER</t>
         </is>
       </c>
-      <c r="E39" s="6" t="n"/>
-      <c r="F39" s="6" t="n"/>
-      <c r="G39" s="6" t="n"/>
-      <c r="H39" s="6" t="n"/>
-      <c r="I39" s="6" t="n"/>
-      <c r="J39" s="6" t="n"/>
-      <c r="K39" s="6" t="n"/>
-      <c r="L39" s="6" t="n"/>
-      <c r="M39" s="6" t="n"/>
-      <c r="N39" s="6" t="n"/>
-      <c r="O39" s="6" t="n"/>
-      <c r="P39" s="6" t="n"/>
-      <c r="Q39" s="6" t="n"/>
-      <c r="R39" s="6" t="n"/>
-      <c r="S39" s="6" t="n"/>
-      <c r="T39" s="6" t="n"/>
-      <c r="U39" s="6" t="n"/>
-      <c r="V39" s="6" t="n"/>
-      <c r="W39" s="6" t="n"/>
-      <c r="X39" s="6" t="n"/>
-      <c r="Y39" s="6" t="n"/>
-      <c r="Z39" s="6" t="n"/>
-      <c r="AA39" s="6" t="n"/>
-      <c r="AB39" s="6" t="n"/>
-      <c r="AC39" s="6" t="n"/>
-      <c r="AD39" s="6" t="n"/>
-      <c r="AE39" s="6" t="n"/>
-      <c r="AF39" s="6" t="n"/>
-      <c r="AG39" s="6" t="n"/>
-      <c r="AH39" s="6" t="n"/>
-      <c r="AI39" s="26" t="n"/>
+      <c r="E39" s="168" t="n"/>
+      <c r="F39" s="168" t="n"/>
+      <c r="G39" s="168" t="n"/>
+      <c r="H39" s="168" t="n"/>
+      <c r="I39" s="168" t="n"/>
+      <c r="J39" s="168" t="n"/>
+      <c r="K39" s="168" t="n"/>
+      <c r="L39" s="168" t="n"/>
+      <c r="M39" s="168" t="n"/>
+      <c r="N39" s="168" t="n"/>
+      <c r="O39" s="168" t="n"/>
+      <c r="P39" s="168" t="n"/>
+      <c r="Q39" s="168" t="n"/>
+      <c r="R39" s="168" t="n"/>
+      <c r="S39" s="168" t="n"/>
+      <c r="T39" s="168" t="n"/>
+      <c r="U39" s="168" t="n"/>
+      <c r="V39" s="168" t="n"/>
+      <c r="W39" s="168" t="n"/>
+      <c r="X39" s="168" t="n"/>
+      <c r="Y39" s="168" t="n"/>
+      <c r="Z39" s="168" t="n"/>
+      <c r="AA39" s="168" t="n"/>
+      <c r="AB39" s="168" t="n"/>
+      <c r="AC39" s="168" t="n"/>
+      <c r="AD39" s="168" t="n"/>
+      <c r="AE39" s="168" t="n"/>
+      <c r="AF39" s="168" t="n"/>
+      <c r="AG39" s="168" t="n"/>
+      <c r="AH39" s="168" t="n"/>
+      <c r="AI39" s="170" t="n"/>
     </row>
     <row r="40" ht="16.2" customHeight="1" thickBot="1">
       <c r="A40" s="8" t="n">
@@ -4198,39 +4300,71 @@
           <t>FITTER</t>
         </is>
       </c>
-      <c r="E40" s="27" t="n"/>
-      <c r="F40" s="27" t="n"/>
-      <c r="G40" s="27" t="n"/>
-      <c r="H40" s="27" t="n"/>
-      <c r="I40" s="27" t="n"/>
-      <c r="J40" s="27" t="n"/>
-      <c r="K40" s="27" t="n"/>
-      <c r="L40" s="27" t="n"/>
-      <c r="M40" s="27" t="n"/>
-      <c r="N40" s="27" t="n"/>
-      <c r="O40" s="27" t="n"/>
-      <c r="P40" s="27" t="n"/>
-      <c r="Q40" s="27" t="n"/>
-      <c r="R40" s="27" t="n"/>
-      <c r="S40" s="27" t="n"/>
-      <c r="T40" s="27" t="n"/>
-      <c r="U40" s="27" t="n"/>
-      <c r="V40" s="27" t="n"/>
-      <c r="W40" s="27" t="n"/>
-      <c r="X40" s="27" t="n"/>
-      <c r="Y40" s="27" t="n"/>
-      <c r="Z40" s="27" t="n"/>
-      <c r="AA40" s="27" t="n"/>
-      <c r="AB40" s="27" t="n"/>
-      <c r="AC40" s="27" t="n"/>
-      <c r="AD40" s="27" t="n"/>
-      <c r="AE40" s="27" t="n"/>
-      <c r="AF40" s="27" t="n"/>
-      <c r="AG40" s="27" t="n"/>
-      <c r="AH40" s="27" t="n"/>
-      <c r="AI40" s="29" t="n"/>
-    </row>
-    <row r="41" ht="15" customHeight="1" thickBot="1"/>
+      <c r="E40" s="173" t="n"/>
+      <c r="F40" s="173" t="n"/>
+      <c r="G40" s="173" t="n"/>
+      <c r="H40" s="173" t="n"/>
+      <c r="I40" s="173" t="n"/>
+      <c r="J40" s="173" t="n"/>
+      <c r="K40" s="173" t="n"/>
+      <c r="L40" s="173" t="n"/>
+      <c r="M40" s="173" t="n"/>
+      <c r="N40" s="173" t="n"/>
+      <c r="O40" s="173" t="n"/>
+      <c r="P40" s="173" t="n"/>
+      <c r="Q40" s="173" t="n"/>
+      <c r="R40" s="173" t="n"/>
+      <c r="S40" s="173" t="n"/>
+      <c r="T40" s="173" t="n"/>
+      <c r="U40" s="173" t="n"/>
+      <c r="V40" s="173" t="n"/>
+      <c r="W40" s="173" t="n"/>
+      <c r="X40" s="173" t="n"/>
+      <c r="Y40" s="173" t="n"/>
+      <c r="Z40" s="173" t="n"/>
+      <c r="AA40" s="173" t="n"/>
+      <c r="AB40" s="173" t="n"/>
+      <c r="AC40" s="173" t="n"/>
+      <c r="AD40" s="173" t="n"/>
+      <c r="AE40" s="173" t="n"/>
+      <c r="AF40" s="173" t="n"/>
+      <c r="AG40" s="173" t="n"/>
+      <c r="AH40" s="173" t="n"/>
+      <c r="AI40" s="175" t="n"/>
+    </row>
+    <row r="41" ht="15" customHeight="1" thickBot="1">
+      <c r="E41" s="176" t="n"/>
+      <c r="F41" s="176" t="n"/>
+      <c r="G41" s="176" t="n"/>
+      <c r="H41" s="176" t="n"/>
+      <c r="I41" s="176" t="n"/>
+      <c r="J41" s="176" t="n"/>
+      <c r="K41" s="176" t="n"/>
+      <c r="L41" s="176" t="n"/>
+      <c r="M41" s="176" t="n"/>
+      <c r="N41" s="176" t="n"/>
+      <c r="O41" s="176" t="n"/>
+      <c r="P41" s="176" t="n"/>
+      <c r="Q41" s="176" t="n"/>
+      <c r="R41" s="176" t="n"/>
+      <c r="S41" s="176" t="n"/>
+      <c r="T41" s="176" t="n"/>
+      <c r="U41" s="176" t="n"/>
+      <c r="V41" s="176" t="n"/>
+      <c r="W41" s="176" t="n"/>
+      <c r="X41" s="176" t="n"/>
+      <c r="Y41" s="176" t="n"/>
+      <c r="Z41" s="176" t="n"/>
+      <c r="AA41" s="176" t="n"/>
+      <c r="AB41" s="176" t="n"/>
+      <c r="AC41" s="176" t="n"/>
+      <c r="AD41" s="176" t="n"/>
+      <c r="AE41" s="176" t="n"/>
+      <c r="AF41" s="176" t="n"/>
+      <c r="AG41" s="176" t="n"/>
+      <c r="AH41" s="176" t="n"/>
+      <c r="AI41" s="176" t="n"/>
+    </row>
     <row r="42" ht="15" customHeight="1" thickBot="1">
       <c r="A42" s="126" t="inlineStr">
         <is>
@@ -4240,127 +4374,127 @@
       <c r="B42" s="123" t="n"/>
       <c r="C42" s="123" t="n"/>
       <c r="D42" s="127" t="n"/>
-      <c r="E42" s="1">
+      <c r="E42" s="179">
         <f>IF(1&lt;=$BA$4,TEXT($BA$3+0,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="F42" s="1">
+      <c r="F42" s="179">
         <f>IF(2&lt;=$BA$4,TEXT($BA$3+1,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="G42" s="1">
+      <c r="G42" s="179">
         <f>IF(3&lt;=$BA$4,TEXT($BA$3+2,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="H42" s="1">
+      <c r="H42" s="179">
         <f>IF(4&lt;=$BA$4,TEXT($BA$3+3,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="I42" s="1">
+      <c r="I42" s="179">
         <f>IF(5&lt;=$BA$4,TEXT($BA$3+4,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="J42" s="1">
+      <c r="J42" s="179">
         <f>IF(6&lt;=$BA$4,TEXT($BA$3+5,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="179">
         <f>IF(7&lt;=$BA$4,TEXT($BA$3+6,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="L42" s="1">
+      <c r="L42" s="179">
         <f>IF(8&lt;=$BA$4,TEXT($BA$3+7,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="M42" s="1">
+      <c r="M42" s="179">
         <f>IF(9&lt;=$BA$4,TEXT($BA$3+8,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="N42" s="1">
+      <c r="N42" s="179">
         <f>IF(10&lt;=$BA$4,TEXT($BA$3+9,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="O42" s="1">
+      <c r="O42" s="179">
         <f>IF(11&lt;=$BA$4,TEXT($BA$3+10,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="P42" s="1">
+      <c r="P42" s="179">
         <f>IF(12&lt;=$BA$4,TEXT($BA$3+11,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Q42" s="1">
+      <c r="Q42" s="179">
         <f>IF(13&lt;=$BA$4,TEXT($BA$3+12,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="R42" s="1">
+      <c r="R42" s="179">
         <f>IF(14&lt;=$BA$4,TEXT($BA$3+13,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="S42" s="1">
+      <c r="S42" s="179">
         <f>IF(15&lt;=$BA$4,TEXT($BA$3+14,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="179">
         <f>IF(16&lt;=$BA$4,TEXT($BA$3+15,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="U42" s="1">
+      <c r="U42" s="179">
         <f>IF(17&lt;=$BA$4,TEXT($BA$3+16,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="V42" s="1">
+      <c r="V42" s="179">
         <f>IF(18&lt;=$BA$4,TEXT($BA$3+17,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="W42" s="1">
+      <c r="W42" s="179">
         <f>IF(19&lt;=$BA$4,TEXT($BA$3+18,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="X42" s="1">
+      <c r="X42" s="179">
         <f>IF(20&lt;=$BA$4,TEXT($BA$3+19,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Y42" s="1">
+      <c r="Y42" s="179">
         <f>IF(21&lt;=$BA$4,TEXT($BA$3+20,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Z42" s="1">
+      <c r="Z42" s="179">
         <f>IF(22&lt;=$BA$4,TEXT($BA$3+21,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AA42" s="1">
+      <c r="AA42" s="179">
         <f>IF(23&lt;=$BA$4,TEXT($BA$3+22,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AB42" s="1">
+      <c r="AB42" s="179">
         <f>IF(24&lt;=$BA$4,TEXT($BA$3+23,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AC42" s="1">
+      <c r="AC42" s="179">
         <f>IF(25&lt;=$BA$4,TEXT($BA$3+24,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AD42" s="1">
+      <c r="AD42" s="179">
         <f>IF(26&lt;=$BA$4,TEXT($BA$3+25,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AE42" s="1">
+      <c r="AE42" s="179">
         <f>IF(27&lt;=$BA$4,TEXT($BA$3+26,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AF42" s="1">
+      <c r="AF42" s="179">
         <f>IF(28&lt;=$BA$4,TEXT($BA$3+27,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AG42" s="1">
+      <c r="AG42" s="179">
         <f>IF(29&lt;=$BA$4,TEXT($BA$3+28,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AH42" s="1">
+      <c r="AH42" s="179">
         <f>IF(30&lt;=$BA$4,TEXT($BA$3+29,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AI42" s="1">
+      <c r="AI42" s="179">
         <f>IF(31&lt;=$BA$4,TEXT($BA$3+30,"ddd"),"")</f>
         <v/>
       </c>
@@ -4512,54 +4646,74 @@
           <t>SUPV</t>
         </is>
       </c>
-      <c r="E44" s="6" t="n"/>
-      <c r="F44" s="6" t="n"/>
-      <c r="G44" s="6" t="n"/>
-      <c r="H44" s="6" t="n"/>
-      <c r="I44" s="6" t="n"/>
-      <c r="J44" s="6" t="n"/>
-      <c r="K44" s="6" t="n"/>
-      <c r="L44" s="6" t="n"/>
-      <c r="M44" s="6" t="n"/>
-      <c r="N44" s="6" t="n"/>
-      <c r="O44" s="6" t="n"/>
-      <c r="P44" s="6" t="n"/>
-      <c r="Q44" s="6" t="n"/>
-      <c r="R44" s="6" t="n"/>
-      <c r="S44" s="6" t="n"/>
-      <c r="T44" s="6" t="n"/>
-      <c r="U44" s="6" t="n"/>
-      <c r="V44" s="6" t="n"/>
-      <c r="W44" s="6" t="n"/>
-      <c r="X44" s="6" t="n"/>
-      <c r="Y44" s="6" t="n"/>
-      <c r="Z44" s="6" t="n"/>
-      <c r="AA44" s="6" t="n"/>
-      <c r="AB44" s="6" t="n"/>
-      <c r="AC44" s="6" t="n"/>
-      <c r="AD44" s="6" t="n"/>
-      <c r="AE44" s="6" t="n"/>
-      <c r="AF44" s="6" t="n"/>
-      <c r="AG44" s="6" t="n"/>
-      <c r="AH44" s="6" t="n"/>
-      <c r="AI44" s="29" t="n"/>
+      <c r="E44" s="168" t="n"/>
+      <c r="F44" s="168" t="n"/>
+      <c r="G44" s="168" t="n"/>
+      <c r="H44" s="168" t="n"/>
+      <c r="I44" s="168" t="n"/>
+      <c r="J44" s="168" t="n"/>
+      <c r="K44" s="168" t="n"/>
+      <c r="L44" s="168" t="n"/>
+      <c r="M44" s="168" t="n"/>
+      <c r="N44" s="168" t="n"/>
+      <c r="O44" s="168" t="n"/>
+      <c r="P44" s="168" t="n"/>
+      <c r="Q44" s="168" t="n"/>
+      <c r="R44" s="168" t="n"/>
+      <c r="S44" s="168" t="n"/>
+      <c r="T44" s="168" t="n"/>
+      <c r="U44" s="168" t="n"/>
+      <c r="V44" s="168" t="n"/>
+      <c r="W44" s="168" t="n"/>
+      <c r="X44" s="168" t="n"/>
+      <c r="Y44" s="168" t="n"/>
+      <c r="Z44" s="168" t="n"/>
+      <c r="AA44" s="168" t="n"/>
+      <c r="AB44" s="168" t="n"/>
+      <c r="AC44" s="168" t="n"/>
+      <c r="AD44" s="168" t="n"/>
+      <c r="AE44" s="168" t="n"/>
+      <c r="AF44" s="168" t="n"/>
+      <c r="AG44" s="168" t="n"/>
+      <c r="AH44" s="168" t="n"/>
+      <c r="AI44" s="175" t="n"/>
     </row>
     <row r="45" ht="16.2" customHeight="1" thickBot="1">
       <c r="A45" s="12" t="n"/>
       <c r="B45" s="129" t="n"/>
       <c r="C45" s="130" t="n"/>
       <c r="D45" s="129" t="n"/>
-      <c r="E45" s="14" t="n"/>
-      <c r="F45" s="14" t="n"/>
-      <c r="G45" s="14" t="n"/>
-      <c r="H45" s="14" t="n"/>
-      <c r="I45" s="14" t="n"/>
-      <c r="J45" s="14" t="n"/>
-      <c r="K45" s="14" t="n"/>
-      <c r="L45" s="14" t="n"/>
-      <c r="M45" s="14" t="n"/>
-      <c r="N45" s="14" t="n"/>
-      <c r="O45" s="14" t="n"/>
+      <c r="E45" s="176" t="n"/>
+      <c r="F45" s="176" t="n"/>
+      <c r="G45" s="176" t="n"/>
+      <c r="H45" s="176" t="n"/>
+      <c r="I45" s="176" t="n"/>
+      <c r="J45" s="176" t="n"/>
+      <c r="K45" s="176" t="n"/>
+      <c r="L45" s="176" t="n"/>
+      <c r="M45" s="176" t="n"/>
+      <c r="N45" s="176" t="n"/>
+      <c r="O45" s="176" t="n"/>
+      <c r="P45" s="176" t="n"/>
+      <c r="Q45" s="176" t="n"/>
+      <c r="R45" s="176" t="n"/>
+      <c r="S45" s="176" t="n"/>
+      <c r="T45" s="176" t="n"/>
+      <c r="U45" s="176" t="n"/>
+      <c r="V45" s="176" t="n"/>
+      <c r="W45" s="176" t="n"/>
+      <c r="X45" s="176" t="n"/>
+      <c r="Y45" s="176" t="n"/>
+      <c r="Z45" s="176" t="n"/>
+      <c r="AA45" s="176" t="n"/>
+      <c r="AB45" s="176" t="n"/>
+      <c r="AC45" s="176" t="n"/>
+      <c r="AD45" s="176" t="n"/>
+      <c r="AE45" s="176" t="n"/>
+      <c r="AF45" s="176" t="n"/>
+      <c r="AG45" s="176" t="n"/>
+      <c r="AH45" s="176" t="n"/>
+      <c r="AI45" s="176" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
       <c r="A46" s="126" t="inlineStr">
@@ -4570,127 +4724,127 @@
       <c r="B46" s="123" t="n"/>
       <c r="C46" s="123" t="n"/>
       <c r="D46" s="127" t="n"/>
-      <c r="E46" s="1">
+      <c r="E46" s="179">
         <f>IF(1&lt;=$BA$4,TEXT($BA$3+0,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="F46" s="1">
+      <c r="F46" s="179">
         <f>IF(2&lt;=$BA$4,TEXT($BA$3+1,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="G46" s="1">
+      <c r="G46" s="179">
         <f>IF(3&lt;=$BA$4,TEXT($BA$3+2,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="H46" s="1">
+      <c r="H46" s="179">
         <f>IF(4&lt;=$BA$4,TEXT($BA$3+3,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="I46" s="1">
+      <c r="I46" s="179">
         <f>IF(5&lt;=$BA$4,TEXT($BA$3+4,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="J46" s="1">
+      <c r="J46" s="179">
         <f>IF(6&lt;=$BA$4,TEXT($BA$3+5,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="179">
         <f>IF(7&lt;=$BA$4,TEXT($BA$3+6,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="L46" s="1">
+      <c r="L46" s="179">
         <f>IF(8&lt;=$BA$4,TEXT($BA$3+7,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="M46" s="1">
+      <c r="M46" s="179">
         <f>IF(9&lt;=$BA$4,TEXT($BA$3+8,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="N46" s="1">
+      <c r="N46" s="179">
         <f>IF(10&lt;=$BA$4,TEXT($BA$3+9,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="O46" s="1">
+      <c r="O46" s="179">
         <f>IF(11&lt;=$BA$4,TEXT($BA$3+10,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="P46" s="1">
+      <c r="P46" s="179">
         <f>IF(12&lt;=$BA$4,TEXT($BA$3+11,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Q46" s="1">
+      <c r="Q46" s="179">
         <f>IF(13&lt;=$BA$4,TEXT($BA$3+12,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="R46" s="1">
+      <c r="R46" s="179">
         <f>IF(14&lt;=$BA$4,TEXT($BA$3+13,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="S46" s="1">
+      <c r="S46" s="179">
         <f>IF(15&lt;=$BA$4,TEXT($BA$3+14,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="T46" s="1">
+      <c r="T46" s="179">
         <f>IF(16&lt;=$BA$4,TEXT($BA$3+15,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="U46" s="1">
+      <c r="U46" s="179">
         <f>IF(17&lt;=$BA$4,TEXT($BA$3+16,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="V46" s="1">
+      <c r="V46" s="179">
         <f>IF(18&lt;=$BA$4,TEXT($BA$3+17,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="W46" s="1">
+      <c r="W46" s="179">
         <f>IF(19&lt;=$BA$4,TEXT($BA$3+18,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="X46" s="1">
+      <c r="X46" s="179">
         <f>IF(20&lt;=$BA$4,TEXT($BA$3+19,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Y46" s="1">
+      <c r="Y46" s="179">
         <f>IF(21&lt;=$BA$4,TEXT($BA$3+20,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="Z46" s="1">
+      <c r="Z46" s="179">
         <f>IF(22&lt;=$BA$4,TEXT($BA$3+21,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AA46" s="1">
+      <c r="AA46" s="179">
         <f>IF(23&lt;=$BA$4,TEXT($BA$3+22,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AB46" s="1">
+      <c r="AB46" s="179">
         <f>IF(24&lt;=$BA$4,TEXT($BA$3+23,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AC46" s="1">
+      <c r="AC46" s="179">
         <f>IF(25&lt;=$BA$4,TEXT($BA$3+24,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AD46" s="1">
+      <c r="AD46" s="179">
         <f>IF(26&lt;=$BA$4,TEXT($BA$3+25,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AE46" s="1">
+      <c r="AE46" s="179">
         <f>IF(27&lt;=$BA$4,TEXT($BA$3+26,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AF46" s="1">
+      <c r="AF46" s="179">
         <f>IF(28&lt;=$BA$4,TEXT($BA$3+27,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AG46" s="1">
+      <c r="AG46" s="179">
         <f>IF(29&lt;=$BA$4,TEXT($BA$3+28,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AH46" s="1">
+      <c r="AH46" s="179">
         <f>IF(30&lt;=$BA$4,TEXT($BA$3+29,"ddd"),"")</f>
         <v/>
       </c>
-      <c r="AI46" s="1">
+      <c r="AI46" s="179">
         <f>IF(31&lt;=$BA$4,TEXT($BA$3+30,"ddd"),"")</f>
         <v/>
       </c>
@@ -4842,37 +4996,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E48" s="6" t="n"/>
-      <c r="F48" s="6" t="n"/>
-      <c r="G48" s="6" t="n"/>
-      <c r="H48" s="6" t="n"/>
-      <c r="I48" s="6" t="n"/>
-      <c r="J48" s="6" t="n"/>
-      <c r="K48" s="6" t="n"/>
-      <c r="L48" s="6" t="n"/>
-      <c r="M48" s="6" t="n"/>
-      <c r="N48" s="6" t="n"/>
-      <c r="O48" s="6" t="n"/>
-      <c r="P48" s="6" t="n"/>
-      <c r="Q48" s="6" t="n"/>
-      <c r="R48" s="6" t="n"/>
-      <c r="S48" s="6" t="n"/>
-      <c r="T48" s="6" t="n"/>
-      <c r="U48" s="6" t="n"/>
-      <c r="V48" s="6" t="n"/>
-      <c r="W48" s="6" t="n"/>
-      <c r="X48" s="6" t="n"/>
-      <c r="Y48" s="6" t="n"/>
-      <c r="Z48" s="6" t="n"/>
-      <c r="AA48" s="6" t="n"/>
-      <c r="AB48" s="6" t="n"/>
-      <c r="AC48" s="6" t="n"/>
-      <c r="AD48" s="6" t="n"/>
-      <c r="AE48" s="6" t="n"/>
-      <c r="AF48" s="6" t="n"/>
-      <c r="AG48" s="6" t="n"/>
-      <c r="AH48" s="6" t="n"/>
-      <c r="AI48" s="6" t="n"/>
+      <c r="E48" s="168" t="n"/>
+      <c r="F48" s="168" t="n"/>
+      <c r="G48" s="168" t="n"/>
+      <c r="H48" s="168" t="n"/>
+      <c r="I48" s="168" t="n"/>
+      <c r="J48" s="168" t="n"/>
+      <c r="K48" s="168" t="n"/>
+      <c r="L48" s="168" t="n"/>
+      <c r="M48" s="168" t="n"/>
+      <c r="N48" s="168" t="n"/>
+      <c r="O48" s="168" t="n"/>
+      <c r="P48" s="168" t="n"/>
+      <c r="Q48" s="168" t="n"/>
+      <c r="R48" s="168" t="n"/>
+      <c r="S48" s="168" t="n"/>
+      <c r="T48" s="168" t="n"/>
+      <c r="U48" s="168" t="n"/>
+      <c r="V48" s="168" t="n"/>
+      <c r="W48" s="168" t="n"/>
+      <c r="X48" s="168" t="n"/>
+      <c r="Y48" s="168" t="n"/>
+      <c r="Z48" s="168" t="n"/>
+      <c r="AA48" s="168" t="n"/>
+      <c r="AB48" s="168" t="n"/>
+      <c r="AC48" s="168" t="n"/>
+      <c r="AD48" s="168" t="n"/>
+      <c r="AE48" s="168" t="n"/>
+      <c r="AF48" s="168" t="n"/>
+      <c r="AG48" s="168" t="n"/>
+      <c r="AH48" s="168" t="n"/>
+      <c r="AI48" s="168" t="n"/>
     </row>
     <row r="49" ht="16.2" customHeight="1" thickBot="1">
       <c r="A49" s="9" t="n">
@@ -4891,37 +5045,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E49" s="6" t="n"/>
-      <c r="F49" s="6" t="n"/>
-      <c r="G49" s="6" t="n"/>
-      <c r="H49" s="6" t="n"/>
-      <c r="I49" s="6" t="n"/>
-      <c r="J49" s="6" t="n"/>
-      <c r="K49" s="6" t="n"/>
-      <c r="L49" s="6" t="n"/>
-      <c r="M49" s="6" t="n"/>
-      <c r="N49" s="6" t="n"/>
-      <c r="O49" s="6" t="n"/>
-      <c r="P49" s="6" t="n"/>
-      <c r="Q49" s="6" t="n"/>
-      <c r="R49" s="6" t="n"/>
-      <c r="S49" s="6" t="n"/>
-      <c r="T49" s="6" t="n"/>
-      <c r="U49" s="6" t="n"/>
-      <c r="V49" s="6" t="n"/>
-      <c r="W49" s="6" t="n"/>
-      <c r="X49" s="6" t="n"/>
-      <c r="Y49" s="6" t="n"/>
-      <c r="Z49" s="6" t="n"/>
-      <c r="AA49" s="6" t="n"/>
-      <c r="AB49" s="6" t="n"/>
-      <c r="AC49" s="6" t="n"/>
-      <c r="AD49" s="6" t="n"/>
-      <c r="AE49" s="6" t="n"/>
-      <c r="AF49" s="6" t="n"/>
-      <c r="AG49" s="6" t="n"/>
-      <c r="AH49" s="6" t="n"/>
-      <c r="AI49" s="6" t="n"/>
+      <c r="E49" s="168" t="n"/>
+      <c r="F49" s="168" t="n"/>
+      <c r="G49" s="168" t="n"/>
+      <c r="H49" s="168" t="n"/>
+      <c r="I49" s="168" t="n"/>
+      <c r="J49" s="168" t="n"/>
+      <c r="K49" s="168" t="n"/>
+      <c r="L49" s="168" t="n"/>
+      <c r="M49" s="168" t="n"/>
+      <c r="N49" s="168" t="n"/>
+      <c r="O49" s="168" t="n"/>
+      <c r="P49" s="168" t="n"/>
+      <c r="Q49" s="168" t="n"/>
+      <c r="R49" s="168" t="n"/>
+      <c r="S49" s="168" t="n"/>
+      <c r="T49" s="168" t="n"/>
+      <c r="U49" s="168" t="n"/>
+      <c r="V49" s="168" t="n"/>
+      <c r="W49" s="168" t="n"/>
+      <c r="X49" s="168" t="n"/>
+      <c r="Y49" s="168" t="n"/>
+      <c r="Z49" s="168" t="n"/>
+      <c r="AA49" s="168" t="n"/>
+      <c r="AB49" s="168" t="n"/>
+      <c r="AC49" s="168" t="n"/>
+      <c r="AD49" s="168" t="n"/>
+      <c r="AE49" s="168" t="n"/>
+      <c r="AF49" s="168" t="n"/>
+      <c r="AG49" s="168" t="n"/>
+      <c r="AH49" s="168" t="n"/>
+      <c r="AI49" s="168" t="n"/>
     </row>
     <row r="50" ht="16.2" customHeight="1" thickBot="1">
       <c r="A50" s="9" t="n">
@@ -4940,37 +5094,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E50" s="6" t="n"/>
-      <c r="F50" s="6" t="n"/>
-      <c r="G50" s="6" t="n"/>
-      <c r="H50" s="6" t="n"/>
-      <c r="I50" s="6" t="n"/>
-      <c r="J50" s="6" t="n"/>
-      <c r="K50" s="6" t="n"/>
-      <c r="L50" s="6" t="n"/>
-      <c r="M50" s="6" t="n"/>
-      <c r="N50" s="6" t="n"/>
-      <c r="O50" s="6" t="n"/>
-      <c r="P50" s="6" t="n"/>
-      <c r="Q50" s="6" t="n"/>
-      <c r="R50" s="6" t="n"/>
-      <c r="S50" s="6" t="n"/>
-      <c r="T50" s="6" t="n"/>
-      <c r="U50" s="6" t="n"/>
-      <c r="V50" s="6" t="n"/>
-      <c r="W50" s="6" t="n"/>
-      <c r="X50" s="6" t="n"/>
-      <c r="Y50" s="6" t="n"/>
-      <c r="Z50" s="6" t="n"/>
-      <c r="AA50" s="6" t="n"/>
-      <c r="AB50" s="6" t="n"/>
-      <c r="AC50" s="6" t="n"/>
-      <c r="AD50" s="6" t="n"/>
-      <c r="AE50" s="6" t="n"/>
-      <c r="AF50" s="6" t="n"/>
-      <c r="AG50" s="6" t="n"/>
-      <c r="AH50" s="6" t="n"/>
-      <c r="AI50" s="6" t="n"/>
+      <c r="E50" s="168" t="n"/>
+      <c r="F50" s="168" t="n"/>
+      <c r="G50" s="168" t="n"/>
+      <c r="H50" s="168" t="n"/>
+      <c r="I50" s="168" t="n"/>
+      <c r="J50" s="168" t="n"/>
+      <c r="K50" s="168" t="n"/>
+      <c r="L50" s="168" t="n"/>
+      <c r="M50" s="168" t="n"/>
+      <c r="N50" s="168" t="n"/>
+      <c r="O50" s="168" t="n"/>
+      <c r="P50" s="168" t="n"/>
+      <c r="Q50" s="168" t="n"/>
+      <c r="R50" s="168" t="n"/>
+      <c r="S50" s="168" t="n"/>
+      <c r="T50" s="168" t="n"/>
+      <c r="U50" s="168" t="n"/>
+      <c r="V50" s="168" t="n"/>
+      <c r="W50" s="168" t="n"/>
+      <c r="X50" s="168" t="n"/>
+      <c r="Y50" s="168" t="n"/>
+      <c r="Z50" s="168" t="n"/>
+      <c r="AA50" s="168" t="n"/>
+      <c r="AB50" s="168" t="n"/>
+      <c r="AC50" s="168" t="n"/>
+      <c r="AD50" s="168" t="n"/>
+      <c r="AE50" s="168" t="n"/>
+      <c r="AF50" s="168" t="n"/>
+      <c r="AG50" s="168" t="n"/>
+      <c r="AH50" s="168" t="n"/>
+      <c r="AI50" s="168" t="n"/>
     </row>
     <row r="51" ht="16.2" customHeight="1" thickBot="1">
       <c r="A51" s="9" t="n">
@@ -4989,37 +5143,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E51" s="6" t="n"/>
-      <c r="F51" s="6" t="n"/>
-      <c r="G51" s="6" t="n"/>
-      <c r="H51" s="6" t="n"/>
-      <c r="I51" s="6" t="n"/>
-      <c r="J51" s="6" t="n"/>
-      <c r="K51" s="6" t="n"/>
-      <c r="L51" s="6" t="n"/>
-      <c r="M51" s="6" t="n"/>
-      <c r="N51" s="6" t="n"/>
-      <c r="O51" s="6" t="n"/>
-      <c r="P51" s="6" t="n"/>
-      <c r="Q51" s="6" t="n"/>
-      <c r="R51" s="6" t="n"/>
-      <c r="S51" s="6" t="n"/>
-      <c r="T51" s="6" t="n"/>
-      <c r="U51" s="6" t="n"/>
-      <c r="V51" s="6" t="n"/>
-      <c r="W51" s="6" t="n"/>
-      <c r="X51" s="6" t="n"/>
-      <c r="Y51" s="6" t="n"/>
-      <c r="Z51" s="6" t="n"/>
-      <c r="AA51" s="6" t="n"/>
-      <c r="AB51" s="6" t="n"/>
-      <c r="AC51" s="6" t="n"/>
-      <c r="AD51" s="6" t="n"/>
-      <c r="AE51" s="6" t="n"/>
-      <c r="AF51" s="6" t="n"/>
-      <c r="AG51" s="6" t="n"/>
-      <c r="AH51" s="6" t="n"/>
-      <c r="AI51" s="6" t="n"/>
+      <c r="E51" s="168" t="n"/>
+      <c r="F51" s="168" t="n"/>
+      <c r="G51" s="168" t="n"/>
+      <c r="H51" s="168" t="n"/>
+      <c r="I51" s="168" t="n"/>
+      <c r="J51" s="168" t="n"/>
+      <c r="K51" s="168" t="n"/>
+      <c r="L51" s="168" t="n"/>
+      <c r="M51" s="168" t="n"/>
+      <c r="N51" s="168" t="n"/>
+      <c r="O51" s="168" t="n"/>
+      <c r="P51" s="168" t="n"/>
+      <c r="Q51" s="168" t="n"/>
+      <c r="R51" s="168" t="n"/>
+      <c r="S51" s="168" t="n"/>
+      <c r="T51" s="168" t="n"/>
+      <c r="U51" s="168" t="n"/>
+      <c r="V51" s="168" t="n"/>
+      <c r="W51" s="168" t="n"/>
+      <c r="X51" s="168" t="n"/>
+      <c r="Y51" s="168" t="n"/>
+      <c r="Z51" s="168" t="n"/>
+      <c r="AA51" s="168" t="n"/>
+      <c r="AB51" s="168" t="n"/>
+      <c r="AC51" s="168" t="n"/>
+      <c r="AD51" s="168" t="n"/>
+      <c r="AE51" s="168" t="n"/>
+      <c r="AF51" s="168" t="n"/>
+      <c r="AG51" s="168" t="n"/>
+      <c r="AH51" s="168" t="n"/>
+      <c r="AI51" s="168" t="n"/>
     </row>
     <row r="52" ht="16.2" customHeight="1" thickBot="1">
       <c r="A52" s="9" t="n">
@@ -5038,37 +5192,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E52" s="6" t="n"/>
-      <c r="F52" s="6" t="n"/>
-      <c r="G52" s="6" t="n"/>
-      <c r="H52" s="6" t="n"/>
-      <c r="I52" s="6" t="n"/>
-      <c r="J52" s="6" t="n"/>
-      <c r="K52" s="6" t="n"/>
-      <c r="L52" s="6" t="n"/>
-      <c r="M52" s="6" t="n"/>
-      <c r="N52" s="6" t="n"/>
-      <c r="O52" s="6" t="n"/>
-      <c r="P52" s="6" t="n"/>
-      <c r="Q52" s="6" t="n"/>
-      <c r="R52" s="6" t="n"/>
-      <c r="S52" s="6" t="n"/>
-      <c r="T52" s="6" t="n"/>
-      <c r="U52" s="6" t="n"/>
-      <c r="V52" s="6" t="n"/>
-      <c r="W52" s="6" t="n"/>
-      <c r="X52" s="6" t="n"/>
-      <c r="Y52" s="6" t="n"/>
-      <c r="Z52" s="6" t="n"/>
-      <c r="AA52" s="6" t="n"/>
-      <c r="AB52" s="6" t="n"/>
-      <c r="AC52" s="6" t="n"/>
-      <c r="AD52" s="6" t="n"/>
-      <c r="AE52" s="6" t="n"/>
-      <c r="AF52" s="6" t="n"/>
-      <c r="AG52" s="6" t="n"/>
-      <c r="AH52" s="6" t="n"/>
-      <c r="AI52" s="6" t="n"/>
+      <c r="E52" s="168" t="n"/>
+      <c r="F52" s="168" t="n"/>
+      <c r="G52" s="168" t="n"/>
+      <c r="H52" s="168" t="n"/>
+      <c r="I52" s="168" t="n"/>
+      <c r="J52" s="168" t="n"/>
+      <c r="K52" s="168" t="n"/>
+      <c r="L52" s="168" t="n"/>
+      <c r="M52" s="168" t="n"/>
+      <c r="N52" s="168" t="n"/>
+      <c r="O52" s="168" t="n"/>
+      <c r="P52" s="168" t="n"/>
+      <c r="Q52" s="168" t="n"/>
+      <c r="R52" s="168" t="n"/>
+      <c r="S52" s="168" t="n"/>
+      <c r="T52" s="168" t="n"/>
+      <c r="U52" s="168" t="n"/>
+      <c r="V52" s="168" t="n"/>
+      <c r="W52" s="168" t="n"/>
+      <c r="X52" s="168" t="n"/>
+      <c r="Y52" s="168" t="n"/>
+      <c r="Z52" s="168" t="n"/>
+      <c r="AA52" s="168" t="n"/>
+      <c r="AB52" s="168" t="n"/>
+      <c r="AC52" s="168" t="n"/>
+      <c r="AD52" s="168" t="n"/>
+      <c r="AE52" s="168" t="n"/>
+      <c r="AF52" s="168" t="n"/>
+      <c r="AG52" s="168" t="n"/>
+      <c r="AH52" s="168" t="n"/>
+      <c r="AI52" s="168" t="n"/>
     </row>
     <row r="53" ht="16.2" customHeight="1" thickBot="1">
       <c r="A53" s="9" t="n">
@@ -5087,37 +5241,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E53" s="6" t="n"/>
-      <c r="F53" s="6" t="n"/>
-      <c r="G53" s="6" t="n"/>
-      <c r="H53" s="6" t="n"/>
-      <c r="I53" s="6" t="n"/>
-      <c r="J53" s="6" t="n"/>
-      <c r="K53" s="6" t="n"/>
-      <c r="L53" s="6" t="n"/>
-      <c r="M53" s="6" t="n"/>
-      <c r="N53" s="6" t="n"/>
-      <c r="O53" s="6" t="n"/>
-      <c r="P53" s="6" t="n"/>
-      <c r="Q53" s="6" t="n"/>
-      <c r="R53" s="6" t="n"/>
-      <c r="S53" s="6" t="n"/>
-      <c r="T53" s="6" t="n"/>
-      <c r="U53" s="6" t="n"/>
-      <c r="V53" s="6" t="n"/>
-      <c r="W53" s="6" t="n"/>
-      <c r="X53" s="6" t="n"/>
-      <c r="Y53" s="6" t="n"/>
-      <c r="Z53" s="6" t="n"/>
-      <c r="AA53" s="6" t="n"/>
-      <c r="AB53" s="6" t="n"/>
-      <c r="AC53" s="6" t="n"/>
-      <c r="AD53" s="6" t="n"/>
-      <c r="AE53" s="6" t="n"/>
-      <c r="AF53" s="6" t="n"/>
-      <c r="AG53" s="6" t="n"/>
-      <c r="AH53" s="6" t="n"/>
-      <c r="AI53" s="6" t="n"/>
+      <c r="E53" s="168" t="n"/>
+      <c r="F53" s="168" t="n"/>
+      <c r="G53" s="168" t="n"/>
+      <c r="H53" s="168" t="n"/>
+      <c r="I53" s="168" t="n"/>
+      <c r="J53" s="168" t="n"/>
+      <c r="K53" s="168" t="n"/>
+      <c r="L53" s="168" t="n"/>
+      <c r="M53" s="168" t="n"/>
+      <c r="N53" s="168" t="n"/>
+      <c r="O53" s="168" t="n"/>
+      <c r="P53" s="168" t="n"/>
+      <c r="Q53" s="168" t="n"/>
+      <c r="R53" s="168" t="n"/>
+      <c r="S53" s="168" t="n"/>
+      <c r="T53" s="168" t="n"/>
+      <c r="U53" s="168" t="n"/>
+      <c r="V53" s="168" t="n"/>
+      <c r="W53" s="168" t="n"/>
+      <c r="X53" s="168" t="n"/>
+      <c r="Y53" s="168" t="n"/>
+      <c r="Z53" s="168" t="n"/>
+      <c r="AA53" s="168" t="n"/>
+      <c r="AB53" s="168" t="n"/>
+      <c r="AC53" s="168" t="n"/>
+      <c r="AD53" s="168" t="n"/>
+      <c r="AE53" s="168" t="n"/>
+      <c r="AF53" s="168" t="n"/>
+      <c r="AG53" s="168" t="n"/>
+      <c r="AH53" s="168" t="n"/>
+      <c r="AI53" s="168" t="n"/>
     </row>
     <row r="54" ht="16.2" customHeight="1" thickBot="1">
       <c r="A54" s="9" t="n">
@@ -5136,37 +5290,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E54" s="6" t="n"/>
-      <c r="F54" s="6" t="n"/>
-      <c r="G54" s="6" t="n"/>
-      <c r="H54" s="6" t="n"/>
-      <c r="I54" s="6" t="n"/>
-      <c r="J54" s="6" t="n"/>
-      <c r="K54" s="6" t="n"/>
-      <c r="L54" s="6" t="n"/>
-      <c r="M54" s="6" t="n"/>
-      <c r="N54" s="6" t="n"/>
-      <c r="O54" s="6" t="n"/>
-      <c r="P54" s="6" t="n"/>
-      <c r="Q54" s="6" t="n"/>
-      <c r="R54" s="6" t="n"/>
-      <c r="S54" s="6" t="n"/>
-      <c r="T54" s="6" t="n"/>
-      <c r="U54" s="6" t="n"/>
-      <c r="V54" s="6" t="n"/>
-      <c r="W54" s="6" t="n"/>
-      <c r="X54" s="6" t="n"/>
-      <c r="Y54" s="6" t="n"/>
-      <c r="Z54" s="6" t="n"/>
-      <c r="AA54" s="6" t="n"/>
-      <c r="AB54" s="6" t="n"/>
-      <c r="AC54" s="6" t="n"/>
-      <c r="AD54" s="6" t="n"/>
-      <c r="AE54" s="6" t="n"/>
-      <c r="AF54" s="6" t="n"/>
-      <c r="AG54" s="6" t="n"/>
-      <c r="AH54" s="6" t="n"/>
-      <c r="AI54" s="6" t="n"/>
+      <c r="E54" s="168" t="n"/>
+      <c r="F54" s="168" t="n"/>
+      <c r="G54" s="168" t="n"/>
+      <c r="H54" s="168" t="n"/>
+      <c r="I54" s="168" t="n"/>
+      <c r="J54" s="168" t="n"/>
+      <c r="K54" s="168" t="n"/>
+      <c r="L54" s="168" t="n"/>
+      <c r="M54" s="168" t="n"/>
+      <c r="N54" s="168" t="n"/>
+      <c r="O54" s="168" t="n"/>
+      <c r="P54" s="168" t="n"/>
+      <c r="Q54" s="168" t="n"/>
+      <c r="R54" s="168" t="n"/>
+      <c r="S54" s="168" t="n"/>
+      <c r="T54" s="168" t="n"/>
+      <c r="U54" s="168" t="n"/>
+      <c r="V54" s="168" t="n"/>
+      <c r="W54" s="168" t="n"/>
+      <c r="X54" s="168" t="n"/>
+      <c r="Y54" s="168" t="n"/>
+      <c r="Z54" s="168" t="n"/>
+      <c r="AA54" s="168" t="n"/>
+      <c r="AB54" s="168" t="n"/>
+      <c r="AC54" s="168" t="n"/>
+      <c r="AD54" s="168" t="n"/>
+      <c r="AE54" s="168" t="n"/>
+      <c r="AF54" s="168" t="n"/>
+      <c r="AG54" s="168" t="n"/>
+      <c r="AH54" s="168" t="n"/>
+      <c r="AI54" s="168" t="n"/>
     </row>
     <row r="55" ht="16.2" customHeight="1" thickBot="1">
       <c r="A55" s="9" t="n">
@@ -5185,37 +5339,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E55" s="6" t="n"/>
-      <c r="F55" s="6" t="n"/>
-      <c r="G55" s="6" t="n"/>
-      <c r="H55" s="6" t="n"/>
-      <c r="I55" s="6" t="n"/>
-      <c r="J55" s="6" t="n"/>
-      <c r="K55" s="6" t="n"/>
-      <c r="L55" s="6" t="n"/>
-      <c r="M55" s="6" t="n"/>
-      <c r="N55" s="6" t="n"/>
-      <c r="O55" s="6" t="n"/>
-      <c r="P55" s="6" t="n"/>
-      <c r="Q55" s="6" t="n"/>
-      <c r="R55" s="6" t="n"/>
-      <c r="S55" s="6" t="n"/>
-      <c r="T55" s="6" t="n"/>
-      <c r="U55" s="6" t="n"/>
-      <c r="V55" s="6" t="n"/>
-      <c r="W55" s="6" t="n"/>
-      <c r="X55" s="6" t="n"/>
-      <c r="Y55" s="6" t="n"/>
-      <c r="Z55" s="6" t="n"/>
-      <c r="AA55" s="6" t="n"/>
-      <c r="AB55" s="6" t="n"/>
-      <c r="AC55" s="6" t="n"/>
-      <c r="AD55" s="6" t="n"/>
-      <c r="AE55" s="6" t="n"/>
-      <c r="AF55" s="6" t="n"/>
-      <c r="AG55" s="6" t="n"/>
-      <c r="AH55" s="6" t="n"/>
-      <c r="AI55" s="6" t="n"/>
+      <c r="E55" s="168" t="n"/>
+      <c r="F55" s="168" t="n"/>
+      <c r="G55" s="168" t="n"/>
+      <c r="H55" s="168" t="n"/>
+      <c r="I55" s="168" t="n"/>
+      <c r="J55" s="168" t="n"/>
+      <c r="K55" s="168" t="n"/>
+      <c r="L55" s="168" t="n"/>
+      <c r="M55" s="168" t="n"/>
+      <c r="N55" s="168" t="n"/>
+      <c r="O55" s="168" t="n"/>
+      <c r="P55" s="168" t="n"/>
+      <c r="Q55" s="168" t="n"/>
+      <c r="R55" s="168" t="n"/>
+      <c r="S55" s="168" t="n"/>
+      <c r="T55" s="168" t="n"/>
+      <c r="U55" s="168" t="n"/>
+      <c r="V55" s="168" t="n"/>
+      <c r="W55" s="168" t="n"/>
+      <c r="X55" s="168" t="n"/>
+      <c r="Y55" s="168" t="n"/>
+      <c r="Z55" s="168" t="n"/>
+      <c r="AA55" s="168" t="n"/>
+      <c r="AB55" s="168" t="n"/>
+      <c r="AC55" s="168" t="n"/>
+      <c r="AD55" s="168" t="n"/>
+      <c r="AE55" s="168" t="n"/>
+      <c r="AF55" s="168" t="n"/>
+      <c r="AG55" s="168" t="n"/>
+      <c r="AH55" s="168" t="n"/>
+      <c r="AI55" s="168" t="n"/>
     </row>
     <row r="56" ht="16.2" customHeight="1" thickBot="1">
       <c r="A56" s="9" t="n">
@@ -5234,37 +5388,37 @@
           <t>TECH</t>
         </is>
       </c>
-      <c r="E56" s="32" t="n"/>
-      <c r="F56" s="32" t="n"/>
-      <c r="G56" s="32" t="n"/>
-      <c r="H56" s="32" t="n"/>
-      <c r="I56" s="6" t="n"/>
-      <c r="J56" s="6" t="n"/>
-      <c r="K56" s="6" t="n"/>
-      <c r="L56" s="6" t="n"/>
-      <c r="M56" s="6" t="n"/>
-      <c r="N56" s="6" t="n"/>
-      <c r="O56" s="6" t="n"/>
-      <c r="P56" s="6" t="n"/>
-      <c r="Q56" s="6" t="n"/>
-      <c r="R56" s="6" t="n"/>
-      <c r="S56" s="6" t="n"/>
-      <c r="T56" s="6" t="n"/>
-      <c r="U56" s="6" t="n"/>
-      <c r="V56" s="6" t="n"/>
-      <c r="W56" s="6" t="n"/>
-      <c r="X56" s="6" t="n"/>
-      <c r="Y56" s="6" t="n"/>
-      <c r="Z56" s="6" t="n"/>
-      <c r="AA56" s="6" t="n"/>
-      <c r="AB56" s="6" t="n"/>
-      <c r="AC56" s="6" t="n"/>
-      <c r="AD56" s="6" t="n"/>
-      <c r="AE56" s="6" t="n"/>
-      <c r="AF56" s="6" t="n"/>
-      <c r="AG56" s="6" t="n"/>
-      <c r="AH56" s="6" t="n"/>
-      <c r="AI56" s="6" t="n"/>
+      <c r="E56" s="180" t="n"/>
+      <c r="F56" s="180" t="n"/>
+      <c r="G56" s="180" t="n"/>
+      <c r="H56" s="180" t="n"/>
+      <c r="I56" s="168" t="n"/>
+      <c r="J56" s="168" t="n"/>
+      <c r="K56" s="168" t="n"/>
+      <c r="L56" s="168" t="n"/>
+      <c r="M56" s="168" t="n"/>
+      <c r="N56" s="168" t="n"/>
+      <c r="O56" s="168" t="n"/>
+      <c r="P56" s="168" t="n"/>
+      <c r="Q56" s="168" t="n"/>
+      <c r="R56" s="168" t="n"/>
+      <c r="S56" s="168" t="n"/>
+      <c r="T56" s="168" t="n"/>
+      <c r="U56" s="168" t="n"/>
+      <c r="V56" s="168" t="n"/>
+      <c r="W56" s="168" t="n"/>
+      <c r="X56" s="168" t="n"/>
+      <c r="Y56" s="168" t="n"/>
+      <c r="Z56" s="168" t="n"/>
+      <c r="AA56" s="168" t="n"/>
+      <c r="AB56" s="168" t="n"/>
+      <c r="AC56" s="168" t="n"/>
+      <c r="AD56" s="168" t="n"/>
+      <c r="AE56" s="168" t="n"/>
+      <c r="AF56" s="168" t="n"/>
+      <c r="AG56" s="168" t="n"/>
+      <c r="AH56" s="168" t="n"/>
+      <c r="AI56" s="168" t="n"/>
     </row>
     <row r="57" ht="16.2" customHeight="1" thickBot="1">
       <c r="A57" s="9" t="n">
@@ -5273,34 +5427,37 @@
       <c r="B57" s="119" t="n"/>
       <c r="C57" s="120" t="n"/>
       <c r="D57" s="121" t="n"/>
-      <c r="E57" s="6" t="n"/>
-      <c r="I57" s="23" t="n"/>
-      <c r="J57" s="6" t="n"/>
-      <c r="K57" s="6" t="n"/>
-      <c r="L57" s="6" t="n"/>
-      <c r="M57" s="6" t="n"/>
-      <c r="N57" s="6" t="n"/>
-      <c r="O57" s="6" t="n"/>
-      <c r="P57" s="6" t="n"/>
-      <c r="Q57" s="6" t="n"/>
-      <c r="R57" s="6" t="n"/>
-      <c r="S57" s="6" t="n"/>
-      <c r="T57" s="6" t="n"/>
-      <c r="U57" s="6" t="n"/>
-      <c r="V57" s="6" t="n"/>
-      <c r="W57" s="6" t="n"/>
-      <c r="X57" s="6" t="n"/>
-      <c r="Y57" s="6" t="n"/>
-      <c r="Z57" s="6" t="n"/>
-      <c r="AA57" s="6" t="n"/>
-      <c r="AB57" s="6" t="n"/>
-      <c r="AC57" s="6" t="n"/>
-      <c r="AD57" s="6" t="n"/>
-      <c r="AE57" s="6" t="n"/>
-      <c r="AF57" s="6" t="n"/>
-      <c r="AG57" s="6" t="n"/>
-      <c r="AH57" s="6" t="n"/>
-      <c r="AI57" s="6" t="n"/>
+      <c r="E57" s="168" t="n"/>
+      <c r="F57" s="176" t="n"/>
+      <c r="G57" s="176" t="n"/>
+      <c r="H57" s="176" t="n"/>
+      <c r="I57" s="171" t="n"/>
+      <c r="J57" s="168" t="n"/>
+      <c r="K57" s="168" t="n"/>
+      <c r="L57" s="168" t="n"/>
+      <c r="M57" s="168" t="n"/>
+      <c r="N57" s="168" t="n"/>
+      <c r="O57" s="168" t="n"/>
+      <c r="P57" s="168" t="n"/>
+      <c r="Q57" s="168" t="n"/>
+      <c r="R57" s="168" t="n"/>
+      <c r="S57" s="168" t="n"/>
+      <c r="T57" s="168" t="n"/>
+      <c r="U57" s="168" t="n"/>
+      <c r="V57" s="168" t="n"/>
+      <c r="W57" s="168" t="n"/>
+      <c r="X57" s="168" t="n"/>
+      <c r="Y57" s="168" t="n"/>
+      <c r="Z57" s="168" t="n"/>
+      <c r="AA57" s="168" t="n"/>
+      <c r="AB57" s="168" t="n"/>
+      <c r="AC57" s="168" t="n"/>
+      <c r="AD57" s="168" t="n"/>
+      <c r="AE57" s="168" t="n"/>
+      <c r="AF57" s="168" t="n"/>
+      <c r="AG57" s="168" t="n"/>
+      <c r="AH57" s="168" t="n"/>
+      <c r="AI57" s="168" t="n"/>
     </row>
     <row r="58" ht="16.2" customHeight="1" thickBot="1">
       <c r="A58" s="9" t="n">
@@ -5309,34 +5466,37 @@
       <c r="B58" s="119" t="n"/>
       <c r="C58" s="120" t="n"/>
       <c r="D58" s="121" t="n"/>
-      <c r="E58" s="6" t="n"/>
-      <c r="I58" s="23" t="n"/>
-      <c r="J58" s="6" t="n"/>
-      <c r="K58" s="6" t="n"/>
-      <c r="L58" s="6" t="n"/>
-      <c r="M58" s="6" t="n"/>
-      <c r="N58" s="6" t="n"/>
-      <c r="O58" s="6" t="n"/>
-      <c r="P58" s="6" t="n"/>
-      <c r="Q58" s="6" t="n"/>
-      <c r="R58" s="6" t="n"/>
-      <c r="S58" s="6" t="n"/>
-      <c r="T58" s="6" t="n"/>
-      <c r="U58" s="6" t="n"/>
-      <c r="V58" s="6" t="n"/>
-      <c r="W58" s="6" t="n"/>
-      <c r="X58" s="6" t="n"/>
-      <c r="Y58" s="6" t="n"/>
-      <c r="Z58" s="6" t="n"/>
-      <c r="AA58" s="6" t="n"/>
-      <c r="AB58" s="6" t="n"/>
-      <c r="AC58" s="6" t="n"/>
-      <c r="AD58" s="6" t="n"/>
-      <c r="AE58" s="6" t="n"/>
-      <c r="AF58" s="6" t="n"/>
-      <c r="AG58" s="6" t="n"/>
-      <c r="AH58" s="6" t="n"/>
-      <c r="AI58" s="6" t="n"/>
+      <c r="E58" s="168" t="n"/>
+      <c r="F58" s="176" t="n"/>
+      <c r="G58" s="176" t="n"/>
+      <c r="H58" s="176" t="n"/>
+      <c r="I58" s="171" t="n"/>
+      <c r="J58" s="168" t="n"/>
+      <c r="K58" s="168" t="n"/>
+      <c r="L58" s="168" t="n"/>
+      <c r="M58" s="168" t="n"/>
+      <c r="N58" s="168" t="n"/>
+      <c r="O58" s="168" t="n"/>
+      <c r="P58" s="168" t="n"/>
+      <c r="Q58" s="168" t="n"/>
+      <c r="R58" s="168" t="n"/>
+      <c r="S58" s="168" t="n"/>
+      <c r="T58" s="168" t="n"/>
+      <c r="U58" s="168" t="n"/>
+      <c r="V58" s="168" t="n"/>
+      <c r="W58" s="168" t="n"/>
+      <c r="X58" s="168" t="n"/>
+      <c r="Y58" s="168" t="n"/>
+      <c r="Z58" s="168" t="n"/>
+      <c r="AA58" s="168" t="n"/>
+      <c r="AB58" s="168" t="n"/>
+      <c r="AC58" s="168" t="n"/>
+      <c r="AD58" s="168" t="n"/>
+      <c r="AE58" s="168" t="n"/>
+      <c r="AF58" s="168" t="n"/>
+      <c r="AG58" s="168" t="n"/>
+      <c r="AH58" s="168" t="n"/>
+      <c r="AI58" s="168" t="n"/>
     </row>
     <row r="59" ht="16.2" customHeight="1" thickBot="1">
       <c r="A59" s="9" t="n">
@@ -5345,37 +5505,37 @@
       <c r="B59" s="119" t="n"/>
       <c r="C59" s="120" t="n"/>
       <c r="D59" s="121" t="n"/>
-      <c r="E59" s="6" t="n"/>
+      <c r="E59" s="168" t="n"/>
       <c r="F59" s="131" t="n"/>
       <c r="G59" s="131" t="n"/>
       <c r="H59" s="132" t="n"/>
-      <c r="I59" s="23" t="n"/>
-      <c r="J59" s="6" t="n"/>
-      <c r="K59" s="6" t="n"/>
-      <c r="L59" s="6" t="n"/>
-      <c r="M59" s="6" t="n"/>
-      <c r="N59" s="6" t="n"/>
-      <c r="O59" s="6" t="n"/>
-      <c r="P59" s="6" t="n"/>
-      <c r="Q59" s="6" t="n"/>
-      <c r="R59" s="6" t="n"/>
-      <c r="S59" s="6" t="n"/>
-      <c r="T59" s="6" t="n"/>
-      <c r="U59" s="6" t="n"/>
-      <c r="V59" s="6" t="n"/>
-      <c r="W59" s="6" t="n"/>
-      <c r="X59" s="6" t="n"/>
-      <c r="Y59" s="6" t="n"/>
-      <c r="Z59" s="6" t="n"/>
-      <c r="AA59" s="6" t="n"/>
-      <c r="AB59" s="6" t="n"/>
-      <c r="AC59" s="6" t="n"/>
-      <c r="AD59" s="6" t="n"/>
-      <c r="AE59" s="6" t="n"/>
-      <c r="AF59" s="6" t="n"/>
-      <c r="AG59" s="6" t="n"/>
-      <c r="AH59" s="6" t="n"/>
-      <c r="AI59" s="6" t="n"/>
+      <c r="I59" s="171" t="n"/>
+      <c r="J59" s="168" t="n"/>
+      <c r="K59" s="168" t="n"/>
+      <c r="L59" s="168" t="n"/>
+      <c r="M59" s="168" t="n"/>
+      <c r="N59" s="168" t="n"/>
+      <c r="O59" s="168" t="n"/>
+      <c r="P59" s="168" t="n"/>
+      <c r="Q59" s="168" t="n"/>
+      <c r="R59" s="168" t="n"/>
+      <c r="S59" s="168" t="n"/>
+      <c r="T59" s="168" t="n"/>
+      <c r="U59" s="168" t="n"/>
+      <c r="V59" s="168" t="n"/>
+      <c r="W59" s="168" t="n"/>
+      <c r="X59" s="168" t="n"/>
+      <c r="Y59" s="168" t="n"/>
+      <c r="Z59" s="168" t="n"/>
+      <c r="AA59" s="168" t="n"/>
+      <c r="AB59" s="168" t="n"/>
+      <c r="AC59" s="168" t="n"/>
+      <c r="AD59" s="168" t="n"/>
+      <c r="AE59" s="168" t="n"/>
+      <c r="AF59" s="168" t="n"/>
+      <c r="AG59" s="168" t="n"/>
+      <c r="AH59" s="168" t="n"/>
+      <c r="AI59" s="168" t="n"/>
     </row>
     <row r="60" ht="16.2" customHeight="1" thickBot="1">
       <c r="A60" s="9" t="n">
@@ -5384,37 +5544,37 @@
       <c r="B60" s="119" t="n"/>
       <c r="C60" s="120" t="n"/>
       <c r="D60" s="121" t="n"/>
-      <c r="E60" s="6" t="n"/>
+      <c r="E60" s="168" t="n"/>
       <c r="F60" s="131" t="n"/>
       <c r="G60" s="131" t="n"/>
       <c r="H60" s="132" t="n"/>
-      <c r="I60" s="23" t="n"/>
-      <c r="J60" s="6" t="n"/>
-      <c r="K60" s="6" t="n"/>
-      <c r="L60" s="6" t="n"/>
-      <c r="M60" s="6" t="n"/>
-      <c r="N60" s="6" t="n"/>
-      <c r="O60" s="6" t="n"/>
-      <c r="P60" s="6" t="n"/>
-      <c r="Q60" s="6" t="n"/>
-      <c r="R60" s="6" t="n"/>
-      <c r="S60" s="6" t="n"/>
-      <c r="T60" s="6" t="n"/>
-      <c r="U60" s="6" t="n"/>
-      <c r="V60" s="6" t="n"/>
-      <c r="W60" s="6" t="n"/>
-      <c r="X60" s="6" t="n"/>
-      <c r="Y60" s="6" t="n"/>
-      <c r="Z60" s="6" t="n"/>
-      <c r="AA60" s="6" t="n"/>
-      <c r="AB60" s="6" t="n"/>
-      <c r="AC60" s="6" t="n"/>
-      <c r="AD60" s="6" t="n"/>
-      <c r="AE60" s="6" t="n"/>
-      <c r="AF60" s="6" t="n"/>
-      <c r="AG60" s="6" t="n"/>
-      <c r="AH60" s="6" t="n"/>
-      <c r="AI60" s="6" t="n"/>
+      <c r="I60" s="171" t="n"/>
+      <c r="J60" s="168" t="n"/>
+      <c r="K60" s="168" t="n"/>
+      <c r="L60" s="168" t="n"/>
+      <c r="M60" s="168" t="n"/>
+      <c r="N60" s="168" t="n"/>
+      <c r="O60" s="168" t="n"/>
+      <c r="P60" s="168" t="n"/>
+      <c r="Q60" s="168" t="n"/>
+      <c r="R60" s="168" t="n"/>
+      <c r="S60" s="168" t="n"/>
+      <c r="T60" s="168" t="n"/>
+      <c r="U60" s="168" t="n"/>
+      <c r="V60" s="168" t="n"/>
+      <c r="W60" s="168" t="n"/>
+      <c r="X60" s="168" t="n"/>
+      <c r="Y60" s="168" t="n"/>
+      <c r="Z60" s="168" t="n"/>
+      <c r="AA60" s="168" t="n"/>
+      <c r="AB60" s="168" t="n"/>
+      <c r="AC60" s="168" t="n"/>
+      <c r="AD60" s="168" t="n"/>
+      <c r="AE60" s="168" t="n"/>
+      <c r="AF60" s="168" t="n"/>
+      <c r="AG60" s="168" t="n"/>
+      <c r="AH60" s="168" t="n"/>
+      <c r="AI60" s="168" t="n"/>
     </row>
     <row r="61" ht="16.2" customHeight="1" thickBot="1">
       <c r="A61" s="9" t="n">
@@ -5423,34 +5583,37 @@
       <c r="B61" s="119" t="n"/>
       <c r="C61" s="120" t="n"/>
       <c r="D61" s="121" t="n"/>
-      <c r="E61" s="6" t="n"/>
-      <c r="I61" s="23" t="n"/>
-      <c r="J61" s="6" t="n"/>
-      <c r="K61" s="6" t="n"/>
-      <c r="L61" s="6" t="n"/>
-      <c r="M61" s="6" t="n"/>
-      <c r="N61" s="6" t="n"/>
-      <c r="O61" s="6" t="n"/>
-      <c r="P61" s="6" t="n"/>
-      <c r="Q61" s="6" t="n"/>
-      <c r="R61" s="6" t="n"/>
-      <c r="S61" s="6" t="n"/>
-      <c r="T61" s="6" t="n"/>
-      <c r="U61" s="6" t="n"/>
-      <c r="V61" s="6" t="n"/>
-      <c r="W61" s="6" t="n"/>
-      <c r="X61" s="6" t="n"/>
-      <c r="Y61" s="6" t="n"/>
-      <c r="Z61" s="6" t="n"/>
-      <c r="AA61" s="6" t="n"/>
-      <c r="AB61" s="6" t="n"/>
-      <c r="AC61" s="6" t="n"/>
-      <c r="AD61" s="6" t="n"/>
-      <c r="AE61" s="6" t="n"/>
-      <c r="AF61" s="6" t="n"/>
-      <c r="AG61" s="6" t="n"/>
-      <c r="AH61" s="6" t="n"/>
-      <c r="AI61" s="6" t="n"/>
+      <c r="E61" s="168" t="n"/>
+      <c r="F61" s="176" t="n"/>
+      <c r="G61" s="176" t="n"/>
+      <c r="H61" s="176" t="n"/>
+      <c r="I61" s="171" t="n"/>
+      <c r="J61" s="168" t="n"/>
+      <c r="K61" s="168" t="n"/>
+      <c r="L61" s="168" t="n"/>
+      <c r="M61" s="168" t="n"/>
+      <c r="N61" s="168" t="n"/>
+      <c r="O61" s="168" t="n"/>
+      <c r="P61" s="168" t="n"/>
+      <c r="Q61" s="168" t="n"/>
+      <c r="R61" s="168" t="n"/>
+      <c r="S61" s="168" t="n"/>
+      <c r="T61" s="168" t="n"/>
+      <c r="U61" s="168" t="n"/>
+      <c r="V61" s="168" t="n"/>
+      <c r="W61" s="168" t="n"/>
+      <c r="X61" s="168" t="n"/>
+      <c r="Y61" s="168" t="n"/>
+      <c r="Z61" s="168" t="n"/>
+      <c r="AA61" s="168" t="n"/>
+      <c r="AB61" s="168" t="n"/>
+      <c r="AC61" s="168" t="n"/>
+      <c r="AD61" s="168" t="n"/>
+      <c r="AE61" s="168" t="n"/>
+      <c r="AF61" s="168" t="n"/>
+      <c r="AG61" s="168" t="n"/>
+      <c r="AH61" s="168" t="n"/>
+      <c r="AI61" s="168" t="n"/>
     </row>
     <row r="62" ht="16.2" customHeight="1" thickBot="1">
       <c r="A62" s="9" t="n">
@@ -5459,37 +5622,37 @@
       <c r="B62" s="119" t="n"/>
       <c r="C62" s="120" t="n"/>
       <c r="D62" s="121" t="n"/>
-      <c r="E62" s="6" t="n"/>
+      <c r="E62" s="168" t="n"/>
       <c r="F62" s="131" t="n"/>
       <c r="G62" s="131" t="n"/>
       <c r="H62" s="132" t="n"/>
-      <c r="I62" s="23" t="n"/>
-      <c r="J62" s="6" t="n"/>
-      <c r="K62" s="6" t="n"/>
-      <c r="L62" s="6" t="n"/>
-      <c r="M62" s="6" t="n"/>
-      <c r="N62" s="6" t="n"/>
-      <c r="O62" s="6" t="n"/>
-      <c r="P62" s="6" t="n"/>
-      <c r="Q62" s="6" t="n"/>
-      <c r="R62" s="6" t="n"/>
-      <c r="S62" s="6" t="n"/>
-      <c r="T62" s="6" t="n"/>
-      <c r="U62" s="6" t="n"/>
-      <c r="V62" s="6" t="n"/>
-      <c r="W62" s="6" t="n"/>
-      <c r="X62" s="6" t="n"/>
-      <c r="Y62" s="6" t="n"/>
-      <c r="Z62" s="6" t="n"/>
-      <c r="AA62" s="6" t="n"/>
-      <c r="AB62" s="6" t="n"/>
-      <c r="AC62" s="6" t="n"/>
-      <c r="AD62" s="6" t="n"/>
-      <c r="AE62" s="6" t="n"/>
-      <c r="AF62" s="6" t="n"/>
-      <c r="AG62" s="6" t="n"/>
-      <c r="AH62" s="6" t="n"/>
-      <c r="AI62" s="6" t="n"/>
+      <c r="I62" s="171" t="n"/>
+      <c r="J62" s="168" t="n"/>
+      <c r="K62" s="168" t="n"/>
+      <c r="L62" s="168" t="n"/>
+      <c r="M62" s="168" t="n"/>
+      <c r="N62" s="168" t="n"/>
+      <c r="O62" s="168" t="n"/>
+      <c r="P62" s="168" t="n"/>
+      <c r="Q62" s="168" t="n"/>
+      <c r="R62" s="168" t="n"/>
+      <c r="S62" s="168" t="n"/>
+      <c r="T62" s="168" t="n"/>
+      <c r="U62" s="168" t="n"/>
+      <c r="V62" s="168" t="n"/>
+      <c r="W62" s="168" t="n"/>
+      <c r="X62" s="168" t="n"/>
+      <c r="Y62" s="168" t="n"/>
+      <c r="Z62" s="168" t="n"/>
+      <c r="AA62" s="168" t="n"/>
+      <c r="AB62" s="168" t="n"/>
+      <c r="AC62" s="168" t="n"/>
+      <c r="AD62" s="168" t="n"/>
+      <c r="AE62" s="168" t="n"/>
+      <c r="AF62" s="168" t="n"/>
+      <c r="AG62" s="168" t="n"/>
+      <c r="AH62" s="168" t="n"/>
+      <c r="AI62" s="168" t="n"/>
     </row>
     <row r="63" ht="16.2" customHeight="1" thickBot="1">
       <c r="A63" s="9" t="n">
@@ -5498,37 +5661,37 @@
       <c r="B63" s="119" t="n"/>
       <c r="C63" s="120" t="n"/>
       <c r="D63" s="121" t="n"/>
-      <c r="E63" s="6" t="n"/>
+      <c r="E63" s="168" t="n"/>
       <c r="F63" s="131" t="n"/>
       <c r="G63" s="131" t="n"/>
       <c r="H63" s="132" t="n"/>
-      <c r="I63" s="23" t="n"/>
-      <c r="J63" s="6" t="n"/>
-      <c r="K63" s="6" t="n"/>
-      <c r="L63" s="6" t="n"/>
-      <c r="M63" s="6" t="n"/>
-      <c r="N63" s="6" t="n"/>
-      <c r="O63" s="6" t="n"/>
-      <c r="P63" s="6" t="n"/>
-      <c r="Q63" s="6" t="n"/>
-      <c r="R63" s="6" t="n"/>
-      <c r="S63" s="6" t="n"/>
-      <c r="T63" s="6" t="n"/>
-      <c r="U63" s="6" t="n"/>
-      <c r="V63" s="6" t="n"/>
-      <c r="W63" s="6" t="n"/>
-      <c r="X63" s="6" t="n"/>
-      <c r="Y63" s="6" t="n"/>
-      <c r="Z63" s="6" t="n"/>
-      <c r="AA63" s="6" t="n"/>
-      <c r="AB63" s="6" t="n"/>
-      <c r="AC63" s="6" t="n"/>
-      <c r="AD63" s="6" t="n"/>
-      <c r="AE63" s="6" t="n"/>
-      <c r="AF63" s="6" t="n"/>
-      <c r="AG63" s="6" t="n"/>
-      <c r="AH63" s="6" t="n"/>
-      <c r="AI63" s="6" t="n"/>
+      <c r="I63" s="171" t="n"/>
+      <c r="J63" s="168" t="n"/>
+      <c r="K63" s="168" t="n"/>
+      <c r="L63" s="168" t="n"/>
+      <c r="M63" s="168" t="n"/>
+      <c r="N63" s="168" t="n"/>
+      <c r="O63" s="168" t="n"/>
+      <c r="P63" s="168" t="n"/>
+      <c r="Q63" s="168" t="n"/>
+      <c r="R63" s="168" t="n"/>
+      <c r="S63" s="168" t="n"/>
+      <c r="T63" s="168" t="n"/>
+      <c r="U63" s="168" t="n"/>
+      <c r="V63" s="168" t="n"/>
+      <c r="W63" s="168" t="n"/>
+      <c r="X63" s="168" t="n"/>
+      <c r="Y63" s="168" t="n"/>
+      <c r="Z63" s="168" t="n"/>
+      <c r="AA63" s="168" t="n"/>
+      <c r="AB63" s="168" t="n"/>
+      <c r="AC63" s="168" t="n"/>
+      <c r="AD63" s="168" t="n"/>
+      <c r="AE63" s="168" t="n"/>
+      <c r="AF63" s="168" t="n"/>
+      <c r="AG63" s="168" t="n"/>
+      <c r="AH63" s="168" t="n"/>
+      <c r="AI63" s="168" t="n"/>
     </row>
     <row r="64" ht="16.2" customHeight="1" thickBot="1">
       <c r="A64" s="9" t="n">
@@ -5537,37 +5700,37 @@
       <c r="B64" s="119" t="n"/>
       <c r="C64" s="120" t="n"/>
       <c r="D64" s="121" t="n"/>
-      <c r="E64" s="6" t="n"/>
+      <c r="E64" s="168" t="n"/>
       <c r="F64" s="131" t="n"/>
       <c r="G64" s="131" t="n"/>
       <c r="H64" s="132" t="n"/>
-      <c r="I64" s="23" t="n"/>
-      <c r="J64" s="6" t="n"/>
-      <c r="K64" s="6" t="n"/>
-      <c r="L64" s="6" t="n"/>
-      <c r="M64" s="6" t="n"/>
-      <c r="N64" s="6" t="n"/>
-      <c r="O64" s="6" t="n"/>
-      <c r="P64" s="6" t="n"/>
-      <c r="Q64" s="6" t="n"/>
-      <c r="R64" s="6" t="n"/>
-      <c r="S64" s="6" t="n"/>
-      <c r="T64" s="6" t="n"/>
-      <c r="U64" s="6" t="n"/>
-      <c r="V64" s="6" t="n"/>
-      <c r="W64" s="6" t="n"/>
-      <c r="X64" s="6" t="n"/>
-      <c r="Y64" s="6" t="n"/>
-      <c r="Z64" s="6" t="n"/>
-      <c r="AA64" s="6" t="n"/>
-      <c r="AB64" s="6" t="n"/>
-      <c r="AC64" s="6" t="n"/>
-      <c r="AD64" s="6" t="n"/>
-      <c r="AE64" s="6" t="n"/>
-      <c r="AF64" s="6" t="n"/>
-      <c r="AG64" s="6" t="n"/>
-      <c r="AH64" s="6" t="n"/>
-      <c r="AI64" s="6" t="n"/>
+      <c r="I64" s="171" t="n"/>
+      <c r="J64" s="168" t="n"/>
+      <c r="K64" s="168" t="n"/>
+      <c r="L64" s="168" t="n"/>
+      <c r="M64" s="168" t="n"/>
+      <c r="N64" s="168" t="n"/>
+      <c r="O64" s="168" t="n"/>
+      <c r="P64" s="168" t="n"/>
+      <c r="Q64" s="168" t="n"/>
+      <c r="R64" s="168" t="n"/>
+      <c r="S64" s="168" t="n"/>
+      <c r="T64" s="168" t="n"/>
+      <c r="U64" s="168" t="n"/>
+      <c r="V64" s="168" t="n"/>
+      <c r="W64" s="168" t="n"/>
+      <c r="X64" s="168" t="n"/>
+      <c r="Y64" s="168" t="n"/>
+      <c r="Z64" s="168" t="n"/>
+      <c r="AA64" s="168" t="n"/>
+      <c r="AB64" s="168" t="n"/>
+      <c r="AC64" s="168" t="n"/>
+      <c r="AD64" s="168" t="n"/>
+      <c r="AE64" s="168" t="n"/>
+      <c r="AF64" s="168" t="n"/>
+      <c r="AG64" s="168" t="n"/>
+      <c r="AH64" s="168" t="n"/>
+      <c r="AI64" s="168" t="n"/>
     </row>
     <row r="65" ht="16.2" customHeight="1" thickBot="1">
       <c r="A65" s="9" t="n">
@@ -5576,37 +5739,37 @@
       <c r="B65" s="119" t="n"/>
       <c r="C65" s="120" t="n"/>
       <c r="D65" s="121" t="n"/>
-      <c r="E65" s="6" t="n"/>
+      <c r="E65" s="168" t="n"/>
       <c r="F65" s="131" t="n"/>
       <c r="G65" s="131" t="n"/>
       <c r="H65" s="132" t="n"/>
-      <c r="I65" s="23" t="n"/>
-      <c r="J65" s="6" t="n"/>
-      <c r="K65" s="6" t="n"/>
-      <c r="L65" s="6" t="n"/>
-      <c r="M65" s="6" t="n"/>
-      <c r="N65" s="6" t="n"/>
-      <c r="O65" s="6" t="n"/>
-      <c r="P65" s="6" t="n"/>
-      <c r="Q65" s="6" t="n"/>
-      <c r="R65" s="6" t="n"/>
-      <c r="S65" s="6" t="n"/>
-      <c r="T65" s="6" t="n"/>
-      <c r="U65" s="6" t="n"/>
-      <c r="V65" s="6" t="n"/>
-      <c r="W65" s="6" t="n"/>
-      <c r="X65" s="6" t="n"/>
-      <c r="Y65" s="6" t="n"/>
-      <c r="Z65" s="6" t="n"/>
-      <c r="AA65" s="6" t="n"/>
-      <c r="AB65" s="6" t="n"/>
-      <c r="AC65" s="6" t="n"/>
-      <c r="AD65" s="6" t="n"/>
-      <c r="AE65" s="6" t="n"/>
-      <c r="AF65" s="6" t="n"/>
-      <c r="AG65" s="6" t="n"/>
-      <c r="AH65" s="6" t="n"/>
-      <c r="AI65" s="6" t="n"/>
+      <c r="I65" s="171" t="n"/>
+      <c r="J65" s="168" t="n"/>
+      <c r="K65" s="168" t="n"/>
+      <c r="L65" s="168" t="n"/>
+      <c r="M65" s="168" t="n"/>
+      <c r="N65" s="168" t="n"/>
+      <c r="O65" s="168" t="n"/>
+      <c r="P65" s="168" t="n"/>
+      <c r="Q65" s="168" t="n"/>
+      <c r="R65" s="168" t="n"/>
+      <c r="S65" s="168" t="n"/>
+      <c r="T65" s="168" t="n"/>
+      <c r="U65" s="168" t="n"/>
+      <c r="V65" s="168" t="n"/>
+      <c r="W65" s="168" t="n"/>
+      <c r="X65" s="168" t="n"/>
+      <c r="Y65" s="168" t="n"/>
+      <c r="Z65" s="168" t="n"/>
+      <c r="AA65" s="168" t="n"/>
+      <c r="AB65" s="168" t="n"/>
+      <c r="AC65" s="168" t="n"/>
+      <c r="AD65" s="168" t="n"/>
+      <c r="AE65" s="168" t="n"/>
+      <c r="AF65" s="168" t="n"/>
+      <c r="AG65" s="168" t="n"/>
+      <c r="AH65" s="168" t="n"/>
+      <c r="AI65" s="168" t="n"/>
     </row>
     <row r="66" ht="16.2" customHeight="1" thickBot="1">
       <c r="A66" s="9" t="n">
@@ -5615,37 +5778,37 @@
       <c r="B66" s="119" t="n"/>
       <c r="C66" s="120" t="n"/>
       <c r="D66" s="121" t="n"/>
-      <c r="E66" s="133" t="n"/>
-      <c r="F66" s="7" t="n"/>
-      <c r="G66" s="7" t="n"/>
-      <c r="H66" s="23" t="n"/>
-      <c r="I66" s="23" t="n"/>
-      <c r="J66" s="6" t="n"/>
-      <c r="K66" s="6" t="n"/>
-      <c r="L66" s="6" t="n"/>
-      <c r="M66" s="6" t="n"/>
-      <c r="N66" s="6" t="n"/>
-      <c r="O66" s="6" t="n"/>
-      <c r="P66" s="6" t="n"/>
-      <c r="Q66" s="6" t="n"/>
-      <c r="R66" s="6" t="n"/>
-      <c r="S66" s="6" t="n"/>
-      <c r="T66" s="6" t="n"/>
-      <c r="U66" s="6" t="n"/>
-      <c r="V66" s="6" t="n"/>
-      <c r="W66" s="6" t="n"/>
-      <c r="X66" s="6" t="n"/>
-      <c r="Y66" s="6" t="n"/>
-      <c r="Z66" s="6" t="n"/>
-      <c r="AA66" s="6" t="n"/>
-      <c r="AB66" s="6" t="n"/>
-      <c r="AC66" s="6" t="n"/>
-      <c r="AD66" s="6" t="n"/>
-      <c r="AE66" s="6" t="n"/>
-      <c r="AF66" s="6" t="n"/>
-      <c r="AG66" s="6" t="n"/>
-      <c r="AH66" s="6" t="n"/>
-      <c r="AI66" s="6" t="n"/>
+      <c r="E66" s="181" t="n"/>
+      <c r="F66" s="169" t="n"/>
+      <c r="G66" s="169" t="n"/>
+      <c r="H66" s="171" t="n"/>
+      <c r="I66" s="171" t="n"/>
+      <c r="J66" s="168" t="n"/>
+      <c r="K66" s="168" t="n"/>
+      <c r="L66" s="168" t="n"/>
+      <c r="M66" s="168" t="n"/>
+      <c r="N66" s="168" t="n"/>
+      <c r="O66" s="168" t="n"/>
+      <c r="P66" s="168" t="n"/>
+      <c r="Q66" s="168" t="n"/>
+      <c r="R66" s="168" t="n"/>
+      <c r="S66" s="168" t="n"/>
+      <c r="T66" s="168" t="n"/>
+      <c r="U66" s="168" t="n"/>
+      <c r="V66" s="168" t="n"/>
+      <c r="W66" s="168" t="n"/>
+      <c r="X66" s="168" t="n"/>
+      <c r="Y66" s="168" t="n"/>
+      <c r="Z66" s="168" t="n"/>
+      <c r="AA66" s="168" t="n"/>
+      <c r="AB66" s="168" t="n"/>
+      <c r="AC66" s="168" t="n"/>
+      <c r="AD66" s="168" t="n"/>
+      <c r="AE66" s="168" t="n"/>
+      <c r="AF66" s="168" t="n"/>
+      <c r="AG66" s="168" t="n"/>
+      <c r="AH66" s="168" t="n"/>
+      <c r="AI66" s="168" t="n"/>
     </row>
     <row r="67" ht="16.2" customHeight="1" thickBot="1">
       <c r="A67" s="9" t="n">
@@ -5654,37 +5817,37 @@
       <c r="B67" s="119" t="n"/>
       <c r="C67" s="120" t="n"/>
       <c r="D67" s="121" t="n"/>
-      <c r="E67" s="133" t="n"/>
-      <c r="F67" s="7" t="n"/>
-      <c r="G67" s="7" t="n"/>
-      <c r="H67" s="23" t="n"/>
-      <c r="I67" s="23" t="n"/>
-      <c r="J67" s="6" t="n"/>
-      <c r="K67" s="6" t="n"/>
-      <c r="L67" s="6" t="n"/>
-      <c r="M67" s="6" t="n"/>
-      <c r="N67" s="6" t="n"/>
-      <c r="O67" s="6" t="n"/>
-      <c r="P67" s="6" t="n"/>
-      <c r="Q67" s="6" t="n"/>
-      <c r="R67" s="6" t="n"/>
-      <c r="S67" s="6" t="n"/>
-      <c r="T67" s="6" t="n"/>
-      <c r="U67" s="6" t="n"/>
-      <c r="V67" s="6" t="n"/>
-      <c r="W67" s="6" t="n"/>
-      <c r="X67" s="6" t="n"/>
-      <c r="Y67" s="6" t="n"/>
-      <c r="Z67" s="6" t="n"/>
-      <c r="AA67" s="6" t="n"/>
-      <c r="AB67" s="6" t="n"/>
-      <c r="AC67" s="6" t="n"/>
-      <c r="AD67" s="6" t="n"/>
-      <c r="AE67" s="6" t="n"/>
-      <c r="AF67" s="6" t="n"/>
-      <c r="AG67" s="6" t="n"/>
-      <c r="AH67" s="6" t="n"/>
-      <c r="AI67" s="6" t="n"/>
+      <c r="E67" s="181" t="n"/>
+      <c r="F67" s="169" t="n"/>
+      <c r="G67" s="169" t="n"/>
+      <c r="H67" s="171" t="n"/>
+      <c r="I67" s="171" t="n"/>
+      <c r="J67" s="168" t="n"/>
+      <c r="K67" s="168" t="n"/>
+      <c r="L67" s="168" t="n"/>
+      <c r="M67" s="168" t="n"/>
+      <c r="N67" s="168" t="n"/>
+      <c r="O67" s="168" t="n"/>
+      <c r="P67" s="168" t="n"/>
+      <c r="Q67" s="168" t="n"/>
+      <c r="R67" s="168" t="n"/>
+      <c r="S67" s="168" t="n"/>
+      <c r="T67" s="168" t="n"/>
+      <c r="U67" s="168" t="n"/>
+      <c r="V67" s="168" t="n"/>
+      <c r="W67" s="168" t="n"/>
+      <c r="X67" s="168" t="n"/>
+      <c r="Y67" s="168" t="n"/>
+      <c r="Z67" s="168" t="n"/>
+      <c r="AA67" s="168" t="n"/>
+      <c r="AB67" s="168" t="n"/>
+      <c r="AC67" s="168" t="n"/>
+      <c r="AD67" s="168" t="n"/>
+      <c r="AE67" s="168" t="n"/>
+      <c r="AF67" s="168" t="n"/>
+      <c r="AG67" s="168" t="n"/>
+      <c r="AH67" s="168" t="n"/>
+      <c r="AI67" s="168" t="n"/>
     </row>
     <row r="68" ht="16.2" customHeight="1" thickBot="1">
       <c r="A68" s="9" t="n">
@@ -5693,37 +5856,37 @@
       <c r="B68" s="119" t="n"/>
       <c r="C68" s="120" t="n"/>
       <c r="D68" s="121" t="n"/>
-      <c r="E68" s="133" t="n"/>
-      <c r="F68" s="7" t="n"/>
-      <c r="G68" s="7" t="n"/>
-      <c r="H68" s="23" t="n"/>
-      <c r="I68" s="23" t="n"/>
-      <c r="J68" s="6" t="n"/>
-      <c r="K68" s="6" t="n"/>
-      <c r="L68" s="6" t="n"/>
-      <c r="M68" s="6" t="n"/>
-      <c r="N68" s="6" t="n"/>
-      <c r="O68" s="6" t="n"/>
-      <c r="P68" s="6" t="n"/>
-      <c r="Q68" s="6" t="n"/>
-      <c r="R68" s="6" t="n"/>
-      <c r="S68" s="6" t="n"/>
-      <c r="T68" s="6" t="n"/>
-      <c r="U68" s="6" t="n"/>
-      <c r="V68" s="6" t="n"/>
-      <c r="W68" s="6" t="n"/>
-      <c r="X68" s="6" t="n"/>
-      <c r="Y68" s="6" t="n"/>
-      <c r="Z68" s="6" t="n"/>
-      <c r="AA68" s="6" t="n"/>
-      <c r="AB68" s="6" t="n"/>
-      <c r="AC68" s="6" t="n"/>
-      <c r="AD68" s="6" t="n"/>
-      <c r="AE68" s="6" t="n"/>
-      <c r="AF68" s="6" t="n"/>
-      <c r="AG68" s="6" t="n"/>
-      <c r="AH68" s="6" t="n"/>
-      <c r="AI68" s="6" t="n"/>
+      <c r="E68" s="181" t="n"/>
+      <c r="F68" s="169" t="n"/>
+      <c r="G68" s="169" t="n"/>
+      <c r="H68" s="171" t="n"/>
+      <c r="I68" s="171" t="n"/>
+      <c r="J68" s="168" t="n"/>
+      <c r="K68" s="168" t="n"/>
+      <c r="L68" s="168" t="n"/>
+      <c r="M68" s="168" t="n"/>
+      <c r="N68" s="168" t="n"/>
+      <c r="O68" s="168" t="n"/>
+      <c r="P68" s="168" t="n"/>
+      <c r="Q68" s="168" t="n"/>
+      <c r="R68" s="168" t="n"/>
+      <c r="S68" s="168" t="n"/>
+      <c r="T68" s="168" t="n"/>
+      <c r="U68" s="168" t="n"/>
+      <c r="V68" s="168" t="n"/>
+      <c r="W68" s="168" t="n"/>
+      <c r="X68" s="168" t="n"/>
+      <c r="Y68" s="168" t="n"/>
+      <c r="Z68" s="168" t="n"/>
+      <c r="AA68" s="168" t="n"/>
+      <c r="AB68" s="168" t="n"/>
+      <c r="AC68" s="168" t="n"/>
+      <c r="AD68" s="168" t="n"/>
+      <c r="AE68" s="168" t="n"/>
+      <c r="AF68" s="168" t="n"/>
+      <c r="AG68" s="168" t="n"/>
+      <c r="AH68" s="168" t="n"/>
+      <c r="AI68" s="168" t="n"/>
     </row>
     <row r="69" ht="16.2" customHeight="1" thickBot="1">
       <c r="A69" s="9" t="n">
@@ -5732,37 +5895,37 @@
       <c r="B69" s="119" t="n"/>
       <c r="C69" s="120" t="n"/>
       <c r="D69" s="121" t="n"/>
-      <c r="E69" s="133" t="n"/>
-      <c r="F69" s="7" t="n"/>
-      <c r="G69" s="7" t="n"/>
-      <c r="H69" s="23" t="n"/>
-      <c r="I69" s="23" t="n"/>
-      <c r="J69" s="6" t="n"/>
-      <c r="K69" s="6" t="n"/>
-      <c r="L69" s="6" t="n"/>
-      <c r="M69" s="6" t="n"/>
-      <c r="N69" s="6" t="n"/>
-      <c r="O69" s="6" t="n"/>
-      <c r="P69" s="6" t="n"/>
-      <c r="Q69" s="6" t="n"/>
-      <c r="R69" s="6" t="n"/>
-      <c r="S69" s="6" t="n"/>
-      <c r="T69" s="6" t="n"/>
-      <c r="U69" s="6" t="n"/>
-      <c r="V69" s="6" t="n"/>
-      <c r="W69" s="6" t="n"/>
-      <c r="X69" s="6" t="n"/>
-      <c r="Y69" s="6" t="n"/>
-      <c r="Z69" s="6" t="n"/>
-      <c r="AA69" s="6" t="n"/>
-      <c r="AB69" s="6" t="n"/>
-      <c r="AC69" s="6" t="n"/>
-      <c r="AD69" s="6" t="n"/>
-      <c r="AE69" s="6" t="n"/>
-      <c r="AF69" s="6" t="n"/>
-      <c r="AG69" s="6" t="n"/>
-      <c r="AH69" s="6" t="n"/>
-      <c r="AI69" s="6" t="n"/>
+      <c r="E69" s="181" t="n"/>
+      <c r="F69" s="169" t="n"/>
+      <c r="G69" s="169" t="n"/>
+      <c r="H69" s="171" t="n"/>
+      <c r="I69" s="171" t="n"/>
+      <c r="J69" s="168" t="n"/>
+      <c r="K69" s="168" t="n"/>
+      <c r="L69" s="168" t="n"/>
+      <c r="M69" s="168" t="n"/>
+      <c r="N69" s="168" t="n"/>
+      <c r="O69" s="168" t="n"/>
+      <c r="P69" s="168" t="n"/>
+      <c r="Q69" s="168" t="n"/>
+      <c r="R69" s="168" t="n"/>
+      <c r="S69" s="168" t="n"/>
+      <c r="T69" s="168" t="n"/>
+      <c r="U69" s="168" t="n"/>
+      <c r="V69" s="168" t="n"/>
+      <c r="W69" s="168" t="n"/>
+      <c r="X69" s="168" t="n"/>
+      <c r="Y69" s="168" t="n"/>
+      <c r="Z69" s="168" t="n"/>
+      <c r="AA69" s="168" t="n"/>
+      <c r="AB69" s="168" t="n"/>
+      <c r="AC69" s="168" t="n"/>
+      <c r="AD69" s="168" t="n"/>
+      <c r="AE69" s="168" t="n"/>
+      <c r="AF69" s="168" t="n"/>
+      <c r="AG69" s="168" t="n"/>
+      <c r="AH69" s="168" t="n"/>
+      <c r="AI69" s="168" t="n"/>
     </row>
     <row r="70" ht="16.2" customHeight="1" thickBot="1">
       <c r="A70" s="9" t="n">
@@ -5771,37 +5934,37 @@
       <c r="B70" s="119" t="n"/>
       <c r="C70" s="120" t="n"/>
       <c r="D70" s="121" t="n"/>
-      <c r="E70" s="133" t="n"/>
-      <c r="F70" s="7" t="n"/>
-      <c r="G70" s="7" t="n"/>
-      <c r="H70" s="23" t="n"/>
-      <c r="I70" s="23" t="n"/>
-      <c r="J70" s="6" t="n"/>
-      <c r="K70" s="6" t="n"/>
-      <c r="L70" s="6" t="n"/>
-      <c r="M70" s="6" t="n"/>
-      <c r="N70" s="6" t="n"/>
-      <c r="O70" s="6" t="n"/>
-      <c r="P70" s="6" t="n"/>
-      <c r="Q70" s="6" t="n"/>
-      <c r="R70" s="6" t="n"/>
-      <c r="S70" s="6" t="n"/>
-      <c r="T70" s="6" t="n"/>
-      <c r="U70" s="6" t="n"/>
-      <c r="V70" s="6" t="n"/>
-      <c r="W70" s="6" t="n"/>
-      <c r="X70" s="6" t="n"/>
-      <c r="Y70" s="6" t="n"/>
-      <c r="Z70" s="6" t="n"/>
-      <c r="AA70" s="6" t="n"/>
-      <c r="AB70" s="6" t="n"/>
-      <c r="AC70" s="6" t="n"/>
-      <c r="AD70" s="6" t="n"/>
-      <c r="AE70" s="6" t="n"/>
-      <c r="AF70" s="6" t="n"/>
-      <c r="AG70" s="6" t="n"/>
-      <c r="AH70" s="6" t="n"/>
-      <c r="AI70" s="6" t="n"/>
+      <c r="E70" s="181" t="n"/>
+      <c r="F70" s="169" t="n"/>
+      <c r="G70" s="169" t="n"/>
+      <c r="H70" s="171" t="n"/>
+      <c r="I70" s="171" t="n"/>
+      <c r="J70" s="168" t="n"/>
+      <c r="K70" s="168" t="n"/>
+      <c r="L70" s="168" t="n"/>
+      <c r="M70" s="168" t="n"/>
+      <c r="N70" s="168" t="n"/>
+      <c r="O70" s="168" t="n"/>
+      <c r="P70" s="168" t="n"/>
+      <c r="Q70" s="168" t="n"/>
+      <c r="R70" s="168" t="n"/>
+      <c r="S70" s="168" t="n"/>
+      <c r="T70" s="168" t="n"/>
+      <c r="U70" s="168" t="n"/>
+      <c r="V70" s="168" t="n"/>
+      <c r="W70" s="168" t="n"/>
+      <c r="X70" s="168" t="n"/>
+      <c r="Y70" s="168" t="n"/>
+      <c r="Z70" s="168" t="n"/>
+      <c r="AA70" s="168" t="n"/>
+      <c r="AB70" s="168" t="n"/>
+      <c r="AC70" s="168" t="n"/>
+      <c r="AD70" s="168" t="n"/>
+      <c r="AE70" s="168" t="n"/>
+      <c r="AF70" s="168" t="n"/>
+      <c r="AG70" s="168" t="n"/>
+      <c r="AH70" s="168" t="n"/>
+      <c r="AI70" s="168" t="n"/>
     </row>
     <row r="71" ht="16.2" customHeight="1" thickBot="1">
       <c r="A71" s="9" t="n">
@@ -5810,37 +5973,37 @@
       <c r="B71" s="119" t="n"/>
       <c r="C71" s="120" t="n"/>
       <c r="D71" s="121" t="n"/>
-      <c r="E71" s="133" t="n"/>
-      <c r="F71" s="7" t="n"/>
-      <c r="G71" s="7" t="n"/>
-      <c r="H71" s="23" t="n"/>
-      <c r="I71" s="23" t="n"/>
-      <c r="J71" s="6" t="n"/>
-      <c r="K71" s="6" t="n"/>
-      <c r="L71" s="6" t="n"/>
-      <c r="M71" s="6" t="n"/>
-      <c r="N71" s="6" t="n"/>
-      <c r="O71" s="6" t="n"/>
-      <c r="P71" s="6" t="n"/>
-      <c r="Q71" s="6" t="n"/>
-      <c r="R71" s="6" t="n"/>
-      <c r="S71" s="6" t="n"/>
-      <c r="T71" s="6" t="n"/>
-      <c r="U71" s="6" t="n"/>
-      <c r="V71" s="6" t="n"/>
-      <c r="W71" s="6" t="n"/>
-      <c r="X71" s="6" t="n"/>
-      <c r="Y71" s="6" t="n"/>
-      <c r="Z71" s="6" t="n"/>
-      <c r="AA71" s="6" t="n"/>
-      <c r="AB71" s="6" t="n"/>
-      <c r="AC71" s="6" t="n"/>
-      <c r="AD71" s="6" t="n"/>
-      <c r="AE71" s="6" t="n"/>
-      <c r="AF71" s="6" t="n"/>
-      <c r="AG71" s="6" t="n"/>
-      <c r="AH71" s="6" t="n"/>
-      <c r="AI71" s="6" t="n"/>
+      <c r="E71" s="181" t="n"/>
+      <c r="F71" s="169" t="n"/>
+      <c r="G71" s="169" t="n"/>
+      <c r="H71" s="171" t="n"/>
+      <c r="I71" s="171" t="n"/>
+      <c r="J71" s="168" t="n"/>
+      <c r="K71" s="168" t="n"/>
+      <c r="L71" s="168" t="n"/>
+      <c r="M71" s="168" t="n"/>
+      <c r="N71" s="168" t="n"/>
+      <c r="O71" s="168" t="n"/>
+      <c r="P71" s="168" t="n"/>
+      <c r="Q71" s="168" t="n"/>
+      <c r="R71" s="168" t="n"/>
+      <c r="S71" s="168" t="n"/>
+      <c r="T71" s="168" t="n"/>
+      <c r="U71" s="168" t="n"/>
+      <c r="V71" s="168" t="n"/>
+      <c r="W71" s="168" t="n"/>
+      <c r="X71" s="168" t="n"/>
+      <c r="Y71" s="168" t="n"/>
+      <c r="Z71" s="168" t="n"/>
+      <c r="AA71" s="168" t="n"/>
+      <c r="AB71" s="168" t="n"/>
+      <c r="AC71" s="168" t="n"/>
+      <c r="AD71" s="168" t="n"/>
+      <c r="AE71" s="168" t="n"/>
+      <c r="AF71" s="168" t="n"/>
+      <c r="AG71" s="168" t="n"/>
+      <c r="AH71" s="168" t="n"/>
+      <c r="AI71" s="168" t="n"/>
     </row>
     <row r="72" ht="16.2" customHeight="1" thickBot="1">
       <c r="A72" s="9" t="n">
@@ -5849,51 +6012,74 @@
       <c r="B72" s="119" t="n"/>
       <c r="C72" s="120" t="n"/>
       <c r="D72" s="121" t="n"/>
-      <c r="E72" s="6" t="n"/>
-      <c r="I72" s="23" t="n"/>
-      <c r="J72" s="6" t="n"/>
-      <c r="K72" s="6" t="n"/>
-      <c r="L72" s="6" t="n"/>
-      <c r="M72" s="6" t="n"/>
-      <c r="N72" s="6" t="n"/>
-      <c r="O72" s="6" t="n"/>
-      <c r="P72" s="6" t="n"/>
-      <c r="Q72" s="6" t="n"/>
-      <c r="R72" s="6" t="n"/>
-      <c r="S72" s="6" t="n"/>
-      <c r="T72" s="6" t="n"/>
-      <c r="U72" s="6" t="n"/>
-      <c r="V72" s="6" t="n"/>
-      <c r="W72" s="6" t="n"/>
-      <c r="X72" s="6" t="n"/>
-      <c r="Y72" s="6" t="n"/>
-      <c r="Z72" s="6" t="n"/>
-      <c r="AA72" s="6" t="n"/>
-      <c r="AB72" s="6" t="n"/>
-      <c r="AC72" s="6" t="n"/>
-      <c r="AD72" s="6" t="n"/>
-      <c r="AE72" s="6" t="n"/>
-      <c r="AF72" s="6" t="n"/>
-      <c r="AG72" s="6" t="n"/>
-      <c r="AH72" s="6" t="n"/>
-      <c r="AI72" s="6" t="n"/>
+      <c r="E72" s="168" t="n"/>
+      <c r="F72" s="176" t="n"/>
+      <c r="G72" s="176" t="n"/>
+      <c r="H72" s="176" t="n"/>
+      <c r="I72" s="171" t="n"/>
+      <c r="J72" s="168" t="n"/>
+      <c r="K72" s="168" t="n"/>
+      <c r="L72" s="168" t="n"/>
+      <c r="M72" s="168" t="n"/>
+      <c r="N72" s="168" t="n"/>
+      <c r="O72" s="168" t="n"/>
+      <c r="P72" s="168" t="n"/>
+      <c r="Q72" s="168" t="n"/>
+      <c r="R72" s="168" t="n"/>
+      <c r="S72" s="168" t="n"/>
+      <c r="T72" s="168" t="n"/>
+      <c r="U72" s="168" t="n"/>
+      <c r="V72" s="168" t="n"/>
+      <c r="W72" s="168" t="n"/>
+      <c r="X72" s="168" t="n"/>
+      <c r="Y72" s="168" t="n"/>
+      <c r="Z72" s="168" t="n"/>
+      <c r="AA72" s="168" t="n"/>
+      <c r="AB72" s="168" t="n"/>
+      <c r="AC72" s="168" t="n"/>
+      <c r="AD72" s="168" t="n"/>
+      <c r="AE72" s="168" t="n"/>
+      <c r="AF72" s="168" t="n"/>
+      <c r="AG72" s="168" t="n"/>
+      <c r="AH72" s="168" t="n"/>
+      <c r="AI72" s="168" t="n"/>
     </row>
     <row r="73" ht="16.2" customHeight="1" thickBot="1">
       <c r="A73" s="13" t="n"/>
       <c r="B73" s="129" t="n"/>
       <c r="C73" s="130" t="n"/>
       <c r="D73" s="129" t="n"/>
-      <c r="E73" s="14" t="n"/>
-      <c r="F73" s="14" t="n"/>
-      <c r="G73" s="14" t="n"/>
-      <c r="H73" s="14" t="n"/>
-      <c r="I73" s="14" t="n"/>
-      <c r="J73" s="14" t="n"/>
-      <c r="K73" s="14" t="n"/>
-      <c r="L73" s="14" t="n"/>
-      <c r="M73" s="14" t="n"/>
-      <c r="N73" s="14" t="n"/>
-      <c r="O73" s="14" t="n"/>
+      <c r="E73" s="176" t="n"/>
+      <c r="F73" s="176" t="n"/>
+      <c r="G73" s="176" t="n"/>
+      <c r="H73" s="176" t="n"/>
+      <c r="I73" s="176" t="n"/>
+      <c r="J73" s="176" t="n"/>
+      <c r="K73" s="176" t="n"/>
+      <c r="L73" s="176" t="n"/>
+      <c r="M73" s="176" t="n"/>
+      <c r="N73" s="176" t="n"/>
+      <c r="O73" s="176" t="n"/>
+      <c r="P73" s="176" t="n"/>
+      <c r="Q73" s="176" t="n"/>
+      <c r="R73" s="176" t="n"/>
+      <c r="S73" s="176" t="n"/>
+      <c r="T73" s="176" t="n"/>
+      <c r="U73" s="176" t="n"/>
+      <c r="V73" s="176" t="n"/>
+      <c r="W73" s="176" t="n"/>
+      <c r="X73" s="176" t="n"/>
+      <c r="Y73" s="176" t="n"/>
+      <c r="Z73" s="176" t="n"/>
+      <c r="AA73" s="176" t="n"/>
+      <c r="AB73" s="176" t="n"/>
+      <c r="AC73" s="176" t="n"/>
+      <c r="AD73" s="176" t="n"/>
+      <c r="AE73" s="176" t="n"/>
+      <c r="AF73" s="176" t="n"/>
+      <c r="AG73" s="176" t="n"/>
+      <c r="AH73" s="176" t="n"/>
+      <c r="AI73" s="176" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1" thickBot="1">
       <c r="A74" s="134" t="inlineStr">

</xml_diff>